<commit_message>
L03: rebuild from the final class deck (62 slides): new depth slides, 7 quick checks, nomogram and onset interactive figures; extractor drops running footers
</commit_message>
<xml_diff>
--- a/docs/sketch/kahoot/unit2_L03.xlsx
+++ b/docs/sketch/kahoot/unit2_L03.xlsx
@@ -1870,27 +1870,27 @@
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>Which set lists methotrexate's key adverse effects from the lecture?</t>
+          <t>Why is celecoxib associated with more cardiovascular events than its GI profile would suggest?</t>
         </is>
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>Hypersensitivity, lymphoma, heart failure</t>
+          <t>TXA2 falls while PGI2 is preserved</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
         <is>
-          <t>Tinnitus, aseptic meningitis, rash</t>
+          <t>It raises renal blood flow excessively</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>Hepatotoxicity, marrow suppression, pulmonary toxicity</t>
+          <t>It depletes glutathione in the heart</t>
         </is>
       </c>
       <c r="F9" s="14" t="inlineStr">
         <is>
-          <t>Retinopathy, cardiomyopathy, myopathy</t>
+          <t>PGI2 falls while platelet TXA2 is preserved</t>
         </is>
       </c>
       <c r="G9" s="14" t="n">
@@ -1898,7 +1898,7 @@
       </c>
       <c r="H9" s="15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I9" s="1" t="n"/>
@@ -1927,27 +1927,27 @@
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>A patient with RA cannot tolerate methotrexate. Which conventional DMARD does the lecture name as the alternative?</t>
+          <t>Which set lists methotrexate's key adverse effects from the lecture?</t>
         </is>
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>Leflunomide</t>
+          <t>Tinnitus, aseptic meningitis, rash</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>Celecoxib</t>
+          <t>GI bleeding, AKI, cardiovascular events</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Hydroxychloroquine</t>
+          <t>Hepatotoxicity, marrow suppression, pulmonary toxicity</t>
         </is>
       </c>
       <c r="F10" s="14" t="inlineStr">
         <is>
-          <t>Rituximab</t>
+          <t>Hypersensitivity, lymphoma, heart failure</t>
         </is>
       </c>
       <c r="G10" s="14" t="n">
@@ -1955,7 +1955,7 @@
       </c>
       <c r="H10" s="15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I10" s="1" t="n"/>
@@ -1984,35 +1984,35 @@
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>Rituximab treats rheumatoid arthritis by which mechanism?</t>
+          <t>Which sequence describes joint destruction in rheumatoid arthritis, as opposed to osteoarthritis?</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>Depleting or modulating B lymphocytes</t>
+          <t>Prostaglandin loss thins the gastric mucosa</t>
         </is>
       </c>
       <c r="D11" s="21" t="inlineStr">
         <is>
-          <t>Blocking T-cell costimulation</t>
+          <t>NAPQI binds proteins in the synovial lining</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Blocking TNF-α signaling</t>
+          <t>Uric acid crystals deposit and trigger a flare</t>
         </is>
       </c>
       <c r="F11" s="14" t="inlineStr">
         <is>
-          <t>Blocking IL-6 receptor signaling</t>
+          <t>Synovitis forms a pannus; TNF-α and IL-6 drive erosion</t>
         </is>
       </c>
       <c r="G11" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H11" s="15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I11" s="1" t="n"/>
@@ -2041,27 +2041,27 @@
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>A patient will start infliximab next month and is due for a live vaccine. When should the vaccine be given?</t>
+          <t>A patient with RA cannot tolerate methotrexate. Which conventional DMARD does the lecture name as the alternative?</t>
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>Any time, since biologics don't affect immunity</t>
+          <t>Hydroxychloroquine</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>Before infliximab is started</t>
+          <t>Celecoxib</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>One week after the first infusion</t>
+          <t>Sulfasalazine</t>
         </is>
       </c>
       <c r="F12" s="14" t="inlineStr">
         <is>
-          <t>Only if a fever develops on therapy</t>
+          <t>Leflunomide</t>
         </is>
       </c>
       <c r="G12" s="14" t="n">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="H12" s="15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I12" s="1" t="n"/>
@@ -2098,27 +2098,27 @@
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>Which NSAID is noted for oral and topical formulations?</t>
+          <t>Rituximab treats rheumatoid arthritis by which mechanism?</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>Indomethacin</t>
+          <t>Blocking IL-6 receptor signaling</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>Celecoxib</t>
+          <t>Blocking T-cell costimulation</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Diclofenac</t>
+          <t>Blocking TNF-α signaling</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
-          <t>Ketorolac</t>
+          <t>Depleting or modulating B lymphocytes</t>
         </is>
       </c>
       <c r="G13" s="14" t="n">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I13" s="1" t="n"/>
@@ -2155,27 +2155,27 @@
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>Why do corticosteroids suppress a broader range of inflammatory mediators than NSAIDs?</t>
+          <t>A patient will start infliximab next month and is due for a live vaccine. When should the vaccine be given?</t>
         </is>
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>They act centrally on the hypothalamus</t>
+          <t>Any time, since biologics don't affect immunity</t>
         </is>
       </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
-          <t>They block COX-2 more strongly than any NSAID</t>
+          <t>Never — vaccines are banned for life</t>
         </is>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>They deplete B cells that release prostaglandins</t>
+          <t>Before infliximab is started</t>
         </is>
       </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
-          <t>They block phospholipase A₂, upstream of COX</t>
+          <t>Only if a fever develops on therapy</t>
         </is>
       </c>
       <c r="G14" s="14" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="H14" s="15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I14" s="1" t="n"/>
@@ -2212,27 +2212,27 @@
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>Which drug pairing does the lecture flag for a higher GI ulcer risk?</t>
+          <t>Which NSAID is noted for oral and topical formulations?</t>
         </is>
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>NSAID plus an anticoagulant</t>
+          <t>Celecoxib</t>
         </is>
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>Acetaminophen plus N-acetylcysteine</t>
+          <t>Ketorolac</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>NSAID plus a corticosteroid</t>
+          <t>Diclofenac</t>
         </is>
       </c>
       <c r="F15" s="14" t="inlineStr">
         <is>
-          <t>NSAID plus a diuretic</t>
+          <t>Indomethacin</t>
         </is>
       </c>
       <c r="G15" s="14" t="n">
@@ -2269,27 +2269,27 @@
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>Which statement correctly describes COX-1?</t>
+          <t>Why do corticosteroids suppress a broader range of inflammatory mediators than NSAIDs?</t>
         </is>
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>Inducible enzyme found mainly at inflamed sites</t>
+          <t>They block phospholipase A₂, upstream of COX</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr">
         <is>
-          <t>Target of celecoxib's selective inhibition</t>
+          <t>They deplete B cells that release prostaglandins</t>
         </is>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>Housekeeping enzyme protecting stomach and renal flow</t>
+          <t>They block COX-2 more strongly than any NSAID</t>
         </is>
       </c>
       <c r="F16" s="14" t="inlineStr">
         <is>
-          <t>Main source of inflammatory prostaglandins</t>
+          <t>They act centrally on the hypothalamus</t>
         </is>
       </c>
       <c r="G16" s="14" t="n">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="H16" s="15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I16" s="1" t="n"/>
@@ -2326,27 +2326,27 @@
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>Per the textbook, which instruction about ketorolac is correct?</t>
+          <t>Which drug pairing does the lecture flag for a higher GI ulcer risk?</t>
         </is>
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>Maximum daily dose is 240 mg</t>
+          <t>NSAID plus a corticosteroid</t>
         </is>
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>Double the dose in patients over 65</t>
+          <t>Acetaminophen plus N-acetylcysteine</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>Safe long-term in renal impairment</t>
+          <t>NSAID plus an anticoagulant</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>Use no longer than 5 days</t>
+          <t>NSAID plus a diuretic</t>
         </is>
       </c>
       <c r="G17" s="14" t="n">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="H17" s="15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I17" s="1" t="n"/>
@@ -2383,35 +2383,35 @@
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>Which effect is acetaminophen least reliable for?</t>
+          <t>Which statement correctly describes COX-1?</t>
         </is>
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>Lowering fever</t>
+          <t>Target of celecoxib's selective inhibition</t>
         </is>
       </c>
       <c r="D18" s="14" t="inlineStr">
         <is>
-          <t>Relieving mild-to-moderate pain</t>
+          <t>Inducible enzyme found mainly at inflamed sites</t>
         </is>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>Pain in a patient with CKD</t>
+          <t>Housekeeping enzyme protecting stomach and renal flow</t>
         </is>
       </c>
       <c r="F18" s="14" t="inlineStr">
         <is>
-          <t>Reducing peripheral inflammation</t>
+          <t>Enzyme that converts acetaminophen to NAPQI</t>
         </is>
       </c>
       <c r="G18" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H18" s="15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I18" s="1" t="n"/>
@@ -2440,35 +2440,35 @@
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>What defines a drug as “disease-modifying” in rheumatoid arthritis?</t>
+          <t>Per the textbook, which instruction about ketorolac is correct?</t>
         </is>
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>It slows or halts joint destruction</t>
+          <t>Double the dose in patients over 65</t>
         </is>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>It relieves pain faster than NSAIDs</t>
+          <t>Maximum daily dose is 240 mg</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>It is given only as an injection</t>
+          <t>Start therapy with an oral dose</t>
         </is>
       </c>
       <c r="F19" s="14" t="inlineStr">
         <is>
-          <t>It lowers fever through the hypothalamus</t>
+          <t>Use no longer than 5 days</t>
         </is>
       </c>
       <c r="G19" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H19" s="15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I19" s="1" t="n"/>
@@ -2497,35 +2497,35 @@
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>Which non-drug approaches does the lecture include in osteoarthritis management?</t>
+          <t>Which effect is acetaminophen least reliable for?</t>
         </is>
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>Glutathione replenishment, label review</t>
+          <t>Pain in a patient with CKD</t>
         </is>
       </c>
       <c r="D20" s="14" t="inlineStr">
         <is>
-          <t>Nerve ablation, spinal cord stimulation</t>
+          <t>Lowering fever</t>
         </is>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>Live vaccines, TB screening, folate</t>
+          <t>Reducing peripheral inflammation</t>
         </is>
       </c>
       <c r="F20" s="14" t="inlineStr">
         <is>
-          <t>Activity modification, physical therapy, weight management</t>
+          <t>First-line mild osteoarthritis pain</t>
         </is>
       </c>
       <c r="G20" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H20" s="15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I20" s="1" t="n"/>
@@ -2554,31 +2554,31 @@
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>A pharmacist calls: a new prescription reads “methotrexate 15 mg by mouth daily” for RA. What is the safety problem?</t>
+          <t>What defines a drug as “disease-modifying” in rheumatoid arthritis?</t>
         </is>
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>It needs N-acetylcysteine with each dose</t>
+          <t>It lowers fever through the hypothalamus</t>
         </is>
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>It should be IV only in RA</t>
+          <t>It selectively blocks the COX-2 isoform</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>It should be twice daily for steady levels</t>
+          <t>It relieves pain faster than NSAIDs</t>
         </is>
       </c>
       <c r="F21" s="14" t="inlineStr">
         <is>
-          <t>It should be weekly; daily dosing can be fatal</t>
+          <t>It slows or halts joint destruction</t>
         </is>
       </c>
       <c r="G21" s="14" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="H21" s="15" t="inlineStr">
         <is>
@@ -2611,27 +2611,27 @@
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>Which sequence describes how tissue injury produces musculoskeletal pain?</t>
+          <t>Which non-drug approaches does the lecture include in osteoarthritis management?</t>
         </is>
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>Injury → glutathione loss → NAPQI build-up → pain</t>
+          <t>Fasting, high-protein diet, bed rest</t>
         </is>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>Injury → nerve transection → cortical atrophy → pain</t>
+          <t>Glutathione replenishment, label review</t>
         </is>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>Injury → mediator release → nociceptor sensitization → pain</t>
+          <t>Activity modification, physical therapy, weight management</t>
         </is>
       </c>
       <c r="F22" s="14" t="inlineStr">
         <is>
-          <t>Injury → T-cell depletion → B-cell surge → pain</t>
+          <t>Live vaccines, TB screening, folate</t>
         </is>
       </c>
       <c r="G22" s="14" t="n">
@@ -2668,27 +2668,27 @@
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>Which drug is a TNF inhibitor?</t>
+          <t>A prescription reads infliximab. What does the stem “-ximab” tell you?</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>Tocilizumab</t>
+          <t>A kinase inhibitor</t>
         </is>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
-          <t>Rituximab</t>
+          <t>A chimeric monoclonal antibody</t>
         </is>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>Abatacept</t>
+          <t>A humanized monoclonal antibody</t>
         </is>
       </c>
       <c r="F23" s="14" t="inlineStr">
         <is>
-          <t>Etanercept</t>
+          <t>A fully human monoclonal antibody</t>
         </is>
       </c>
       <c r="G23" s="14" t="n">
@@ -2696,7 +2696,7 @@
       </c>
       <c r="H23" s="15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I23" s="1" t="n"/>
@@ -2725,31 +2725,31 @@
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>Which set lists the inflammatory mediators the lecture names as sensitizing nociceptors in musculoskeletal pain?</t>
+          <t>A pharmacist calls: a new prescription reads “methotrexate 15 mg by mouth daily” for RA. What is the safety problem?</t>
         </is>
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>Thromboxane, glutathione, NAPQI, and bradykinin</t>
+          <t>Nothing — daily dosing is standard for RA</t>
         </is>
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
-          <t>Cytokines, calcium, vitamin D, and histamine</t>
+          <t>It should be twice daily for steady levels</t>
         </is>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>Prostaglandins, bradykinin, histamine, and cytokines</t>
+          <t>It should be weekly; daily dosing can be fatal</t>
         </is>
       </c>
       <c r="F24" s="14" t="inlineStr">
         <is>
-          <t>Prostaglandins, dopamine, serotonin, and insulin</t>
+          <t>It should be IV only in RA</t>
         </is>
       </c>
       <c r="G24" s="14" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="H24" s="15" t="inlineStr">
         <is>
@@ -2782,27 +2782,27 @@
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>In acetaminophen overdose, why is N-acetylcysteine effective?</t>
+          <t>Which sequence describes how tissue injury produces musculoskeletal pain?</t>
         </is>
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
-          <t>It binds acetaminophen in the gut and prevents absorption</t>
+          <t>Injury → nerve transection → cortical atrophy → pain</t>
         </is>
       </c>
       <c r="D25" s="14" t="inlineStr">
         <is>
-          <t>It speeds renal excretion of unchanged acetaminophen</t>
+          <t>Injury → T-cell depletion → B-cell surge → pain</t>
         </is>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>It is a glutathione precursor that restores NAPQI detoxification</t>
+          <t>Injury → glutathione loss → NAPQI build-up → pain</t>
         </is>
       </c>
       <c r="F25" s="14" t="inlineStr">
         <is>
-          <t>It blocks COX in the liver and lowers prostaglandin levels</t>
+          <t>Injury → mediator release → nociceptor sensitization → pain</t>
         </is>
       </c>
       <c r="G25" s="14" t="n">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="H25" s="15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I25" s="1" t="n"/>
@@ -2839,31 +2839,31 @@
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>Which statement best explains why nonselective NSAIDs cause GI and renal adverse effects?</t>
+          <t>Which drug is a TNF inhibitor?</t>
         </is>
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>They block TNF-α, which normally protects the stomach lining</t>
+          <t>Rituximab</t>
         </is>
       </c>
       <c r="D26" s="14" t="inlineStr">
         <is>
-          <t>They deplete glutathione, which injures the gut and kidney</t>
+          <t>Abatacept</t>
         </is>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>They inhibit COX-1, which protects gastric mucosa and renal blood flow</t>
+          <t>Etanercept</t>
         </is>
       </c>
       <c r="F26" s="14" t="inlineStr">
         <is>
-          <t>They inhibit COX-2, the only source of protective prostaglandins</t>
+          <t>Tocilizumab</t>
         </is>
       </c>
       <c r="G26" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H26" s="15" t="inlineStr">
         <is>
@@ -2896,27 +2896,27 @@
       </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>Which nonselective NSAID does the lecture restrict to short-term use because of significant GI and renal risk?</t>
+          <t>Which mediator is the primary target of NSAID therapy within the inflammatory pain pathway?</t>
         </is>
       </c>
       <c r="C27" s="14" t="inlineStr">
         <is>
-          <t>Celecoxib</t>
+          <t>Bradykinin</t>
         </is>
       </c>
       <c r="D27" s="14" t="inlineStr">
         <is>
-          <t>Ibuprofen</t>
+          <t>Histamine</t>
         </is>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
-          <t>Naproxen</t>
+          <t>Cytokines broadly (e.g., all of TNF-α, IL-1, IL-6)</t>
         </is>
       </c>
       <c r="F27" s="14" t="inlineStr">
         <is>
-          <t>Ketorolac</t>
+          <t>Prostaglandins</t>
         </is>
       </c>
       <c r="G27" s="14" t="n">
@@ -2953,27 +2953,27 @@
       </c>
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>What is the key difference in treatment goals between osteoarthritis and rheumatoid arthritis?</t>
+          <t>In acetaminophen overdose, hepatotoxicity results primarily from which mechanism?</t>
         </is>
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
-          <t>OA aims at pain and function; RA aims to suppress disease activity</t>
+          <t>Excess Phase II glucuronidation</t>
         </is>
       </c>
       <c r="D28" s="14" t="inlineStr">
         <is>
-          <t>RA aims at weight loss; OA aims at infection control</t>
+          <t>Accumulation of NAPQI after glutathione stores are depleted</t>
         </is>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>OA aims at cartilage regrowth with DMARDs</t>
+          <t>Direct COX inhibition in the liver</t>
         </is>
       </c>
       <c r="F28" s="14" t="inlineStr">
         <is>
-          <t>OA aims to suppress immunity; RA aims at pain relief only</t>
+          <t>Renal crystal formation</t>
         </is>
       </c>
       <c r="G28" s="14" t="n">
@@ -2981,7 +2981,7 @@
       </c>
       <c r="H28" s="15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I28" s="1" t="n"/>
@@ -3010,27 +3010,27 @@
       </c>
       <c r="B29" s="16" t="inlineStr">
         <is>
-          <t>What is methotrexate’s mechanism as taught in the lecture, and what is co-prescribed to reduce its toxicity?</t>
+          <t>In acetaminophen overdose, why is N-acetylcysteine effective?</t>
         </is>
       </c>
       <c r="C29" s="16" t="inlineStr">
         <is>
-          <t>Dihydrofolate reductase inhibition; folate supplementation</t>
+          <t>It blocks COX in the liver and lowers prostaglandin levels</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
         <is>
-          <t>COX-2 inhibition; a proton pump inhibitor</t>
+          <t>It is a glutathione precursor that restores NAPQI detoxification</t>
         </is>
       </c>
       <c r="E29" s="16" t="inlineStr">
         <is>
-          <t>Glutathione depletion; N-acetylcysteine</t>
+          <t>It inhibits the enzyme that forms NAPQI from the drug</t>
         </is>
       </c>
       <c r="F29" s="16" t="inlineStr">
         <is>
-          <t>TNF-α blockade; tuberculosis screening</t>
+          <t>It binds acetaminophen in the gut and prevents absorption</t>
         </is>
       </c>
       <c r="G29" s="14" t="n">
@@ -3038,7 +3038,7 @@
       </c>
       <c r="H29" s="17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I29" s="1" t="n"/>
@@ -3067,35 +3067,35 @@
       </c>
       <c r="B30" s="16" t="inlineStr">
         <is>
-          <t>A 29-year-old with active RA who is planning a pregnancy needs a DMARD. Which drug from the lecture is contraindicated?</t>
+          <t>Which statement best explains why nonselective NSAIDs cause GI and renal adverse effects?</t>
         </is>
       </c>
       <c r="C30" s="16" t="inlineStr">
         <is>
-          <t>Celecoxib, because it is a disease-modifying drug</t>
+          <t>They deplete glutathione, which injures the gut and kidney</t>
         </is>
       </c>
       <c r="D30" s="16" t="inlineStr">
         <is>
-          <t>Acetaminophen, because it is a DMARD</t>
+          <t>They block TNF-α, which normally protects the stomach lining</t>
         </is>
       </c>
       <c r="E30" s="16" t="inlineStr">
         <is>
-          <t>Sulfasalazine, because it is only used alone</t>
+          <t>They inhibit COX-1, which protects gastric mucosa and renal blood flow</t>
         </is>
       </c>
       <c r="F30" s="16" t="inlineStr">
         <is>
-          <t>Methotrexate, because it is teratogenic</t>
+          <t>They block phospholipase A₂ and stop all mediator release</t>
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="H30" s="17" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I30" s="1" t="n"/>
@@ -3124,27 +3124,27 @@
       </c>
       <c r="B31" s="16" t="inlineStr">
         <is>
-          <t>Which single feature distinguishes a DMARD from an NSAID in rheumatoid arthritis?</t>
+          <t>Which nonselective NSAID does the lecture restrict to short-term use because of significant GI and renal risk?</t>
         </is>
       </c>
       <c r="C31" s="16" t="inlineStr">
         <is>
-          <t>It gives faster, stronger analgesia than any NSAID</t>
+          <t>Celecoxib</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
         <is>
-          <t>It changes the disease course, not just the symptoms</t>
+          <t>Ketorolac</t>
         </is>
       </c>
       <c r="E31" s="16" t="inlineStr">
         <is>
-          <t>It blocks COX more selectively than an NSAID</t>
+          <t>Naproxen</t>
         </is>
       </c>
       <c r="F31" s="16" t="inlineStr">
         <is>
-          <t>It is always a biologic given by injection</t>
+          <t>Diclofenac</t>
         </is>
       </c>
       <c r="G31" s="14" t="n">
@@ -3181,27 +3181,27 @@
       </c>
       <c r="B32" s="16" t="inlineStr">
         <is>
-          <t>Before starting adalimumab for rheumatoid arthritis, which baseline step does the lecture specifically call for?</t>
+          <t>What is the key difference in treatment goals between osteoarthritis and rheumatoid arthritis?</t>
         </is>
       </c>
       <c r="C32" s="16" t="inlineStr">
         <is>
-          <t>Adding an ACE inhibitor to protect the kidney</t>
+          <t>OA aims at pain and function; RA aims to suppress disease activity</t>
         </is>
       </c>
       <c r="D32" s="16" t="inlineStr">
         <is>
-          <t>Avoiding all vaccines until therapy has begun</t>
+          <t>OA aims at cartilage regrowth with DMARDs</t>
         </is>
       </c>
       <c r="E32" s="16" t="inlineStr">
         <is>
-          <t>Screening for tuberculosis and hepatitis B/C</t>
+          <t>OA aims to suppress immunity; RA aims at pain relief only</t>
         </is>
       </c>
       <c r="F32" s="16" t="inlineStr">
         <is>
-          <t>Starting folate to prevent bone marrow toxicity</t>
+          <t>RA aims at weight loss; OA aims at infection control</t>
         </is>
       </c>
       <c r="G32" s="14" t="n">
@@ -3209,7 +3209,7 @@
       </c>
       <c r="H32" s="17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I32" s="1" t="n"/>
@@ -3238,27 +3238,27 @@
       </c>
       <c r="B33" s="16" t="inlineStr">
         <is>
-          <t>Which biologic DMARD works by blocking the second (costimulatory) signal needed for T-cell activation?</t>
+          <t>What is methotrexate’s mechanism as taught in the lecture, and what is co-prescribed to reduce its toxicity?</t>
         </is>
       </c>
       <c r="C33" s="16" t="inlineStr">
         <is>
-          <t>Tocilizumab</t>
+          <t>COX-2 inhibition; a proton pump inhibitor</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
         <is>
-          <t>Abatacept</t>
+          <t>Phospholipase A₂ blockade; calcium supplementation</t>
         </is>
       </c>
       <c r="E33" s="16" t="inlineStr">
         <is>
-          <t>Etanercept</t>
+          <t>TNF-α blockade; tuberculosis screening</t>
         </is>
       </c>
       <c r="F33" s="16" t="inlineStr">
         <is>
-          <t>Rituximab</t>
+          <t>Dihydrofolate reductase inhibition; folate supplementation</t>
         </is>
       </c>
       <c r="G33" s="14" t="n">
@@ -3266,7 +3266,7 @@
       </c>
       <c r="H33" s="17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I33" s="1" t="n"/>
@@ -3295,31 +3295,31 @@
       </c>
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>Match the drug to its target: which pairing is correct?</t>
+          <t>A 29-year-old with active RA who is planning a pregnancy needs a DMARD. Which drug from the lecture is contraindicated?</t>
         </is>
       </c>
       <c r="C34" s="16" t="inlineStr">
         <is>
-          <t>Abatacept — B-lymphocyte depletion</t>
+          <t>Celecoxib, because it is a disease-modifying drug</t>
         </is>
       </c>
       <c r="D34" s="16" t="inlineStr">
         <is>
-          <t>Adalimumab — T-cell costimulation</t>
+          <t>Acetaminophen, because it is a DMARD</t>
         </is>
       </c>
       <c r="E34" s="16" t="inlineStr">
         <is>
-          <t>Etanercept — IL-6 receptor signaling</t>
+          <t>Hydroxychloroquine, because of its poor safety profile</t>
         </is>
       </c>
       <c r="F34" s="16" t="inlineStr">
         <is>
-          <t>Tocilizumab — IL-6 receptor signaling</t>
+          <t>Methotrexate, because it is teratogenic</t>
         </is>
       </c>
       <c r="G34" s="14" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="H34" s="17" t="inlineStr">
         <is>
@@ -3352,31 +3352,31 @@
       </c>
       <c r="B35" s="16" t="inlineStr">
         <is>
-          <t>Which conventional DMARD requires a baseline eye exam and annual screening after 5 years because of retinopathy?</t>
+          <t>Before starting adalimumab for rheumatoid arthritis, which baseline step does the lecture specifically call for?</t>
         </is>
       </c>
       <c r="C35" s="16" t="inlineStr">
         <is>
-          <t>Mycophenolate mofetil</t>
+          <t>Checking for all hidden acetaminophen sources</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>Sulfasalazine</t>
+          <t>Starting folate to prevent bone marrow toxicity</t>
         </is>
       </c>
       <c r="E35" s="16" t="inlineStr">
         <is>
-          <t>Hydroxychloroquine</t>
+          <t>Screening for tuberculosis and hepatitis B/C</t>
         </is>
       </c>
       <c r="F35" s="16" t="inlineStr">
         <is>
-          <t>Leflunomide</t>
+          <t>Adding an ACE inhibitor to protect the kidney</t>
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="H35" s="17" t="inlineStr">
         <is>
@@ -3409,35 +3409,35 @@
       </c>
       <c r="B36" s="16" t="inlineStr">
         <is>
-          <t>Pain by mechanism: which is right?</t>
+          <t>Match the drug to its target: which pairing is correct?</t>
         </is>
       </c>
       <c r="C36" s="16" t="inlineStr">
         <is>
-          <t>Baseline eye exam; annual after 5 years</t>
+          <t>Abatacept — B-lymphocyte depletion</t>
         </is>
       </c>
       <c r="D36" s="16" t="inlineStr">
         <is>
-          <t>N-acetylcysteine — glutathione precursor</t>
+          <t>Tocilizumab — IL-6 receptor signaling</t>
         </is>
       </c>
       <c r="E36" s="16" t="inlineStr">
         <is>
-          <t>Common first-line for mild-moderate pain</t>
+          <t>Etanercept — IL-6 receptor signaling</t>
         </is>
       </c>
       <c r="F36" s="16" t="inlineStr">
         <is>
-          <t>Nociceptive · inflammatory · neuropathic</t>
+          <t>Rituximab — TNF-α signaling</t>
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H36" s="17" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I36" s="1" t="n"/>
@@ -3466,35 +3466,35 @@
       </c>
       <c r="B37" s="16" t="inlineStr">
         <is>
-          <t>Chronic pain: which is right?</t>
+          <t>Which conventional DMARD requires a baseline eye exam and annual screening after 5 years because of retinopathy?</t>
         </is>
       </c>
       <c r="C37" s="16" t="inlineStr">
         <is>
-          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
+          <t>Methotrexate</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>Persists beyond expected healing, often &gt; 3 months</t>
+          <t>Mycophenolate mofetil</t>
         </is>
       </c>
       <c r="E37" s="16" t="inlineStr">
         <is>
-          <t>TB + hepatitis B/C screen; update vaccines (live) first</t>
+          <t>Leflunomide</t>
         </is>
       </c>
       <c r="F37" s="16" t="inlineStr">
         <is>
-          <t>Housekeeping: gastric protection, renal blood flow</t>
+          <t>Hydroxychloroquine</t>
         </is>
       </c>
       <c r="G37" s="14" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="H37" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I37" s="1" t="n"/>
@@ -3523,27 +3523,27 @@
       </c>
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t>4 pain mediators: which is right?</t>
+          <t>Pain by mechanism: which is right?</t>
         </is>
       </c>
       <c r="C38" s="16" t="inlineStr">
         <is>
-          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
+          <t>CBC, liver, kidney labs every 1–3 months</t>
         </is>
       </c>
       <c r="D38" s="16" t="inlineStr">
         <is>
-          <t>Prostaglandins, bradykinin, histamine, cytokines (TNF-α, IL-1, IL-6)</t>
+          <t>N-acetylcysteine — glutathione precursor</t>
         </is>
       </c>
       <c r="E38" s="16" t="inlineStr">
         <is>
-          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
+          <t>Common first-line for mild-moderate pain</t>
         </is>
       </c>
       <c r="F38" s="16" t="inlineStr">
         <is>
-          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
+          <t>Nociceptive · inflammatory · neuropathic</t>
         </is>
       </c>
       <c r="G38" s="14" t="n">
@@ -3551,7 +3551,7 @@
       </c>
       <c r="H38" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I38" s="1" t="n"/>
@@ -3580,27 +3580,27 @@
       </c>
       <c r="B39" s="16" t="inlineStr">
         <is>
-          <t>Corticosteroid site: which is right?</t>
+          <t>Chronic pain: which is right?</t>
         </is>
       </c>
       <c r="C39" s="16" t="inlineStr">
         <is>
-          <t>TB + hepatitis B/C screen; update vaccines (live) first</t>
+          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
         <is>
-          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
+          <t>Persists beyond expected healing, often &gt; 3 months</t>
         </is>
       </c>
       <c r="E39" s="16" t="inlineStr">
         <is>
-          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
+          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
         </is>
       </c>
       <c r="F39" s="16" t="inlineStr">
         <is>
-          <t>Baricitinib, tofacitinib, upadacitinib — oral; zoster, ↑ LDL</t>
+          <t>Housekeeping: gastric protection, renal blood flow</t>
         </is>
       </c>
       <c r="G39" s="14" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="H39" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I39" s="1" t="n"/>
@@ -3637,35 +3637,35 @@
       </c>
       <c r="B40" s="16" t="inlineStr">
         <is>
-          <t>NSAID site: which is right?</t>
+          <t>4 pain mediators: which is right?</t>
         </is>
       </c>
       <c r="C40" s="16" t="inlineStr">
         <is>
-          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
+          <t>Prostaglandins, bradykinin, histamine, cytokines (TNF-α, IL-1, IL-6)</t>
         </is>
       </c>
       <c r="D40" s="16" t="inlineStr">
         <is>
-          <t>COX → prostaglandins specifically</t>
+          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
         </is>
       </c>
       <c r="E40" s="16" t="inlineStr">
         <is>
-          <t>More potent; more GI/CNS effects</t>
+          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
         </is>
       </c>
       <c r="F40" s="16" t="inlineStr">
         <is>
-          <t>Adalimumab, etanercept, infliximab</t>
+          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
         </is>
       </c>
       <c r="G40" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H40" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I40" s="1" t="n"/>
@@ -3694,27 +3694,27 @@
       </c>
       <c r="B41" s="16" t="inlineStr">
         <is>
-          <t>Acetaminophen effects: which is right?</t>
+          <t>Corticosteroid site: which is right?</t>
         </is>
       </c>
       <c r="C41" s="16" t="inlineStr">
         <is>
-          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
+          <t>TB + hepatitis B/C screen; update vaccines (live) first</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>TB + hepatitis B/C screen; update vaccines (live) first</t>
+          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
         </is>
       </c>
       <c r="E41" s="16" t="inlineStr">
         <is>
-          <t>Persists beyond expected healing, often &gt; 3 months</t>
+          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
         </is>
       </c>
       <c r="F41" s="16" t="inlineStr">
         <is>
-          <t>Housekeeping: gastric protection, renal blood flow</t>
+          <t>Anti-CD20; after TNF-inhibitor failure; check hepatitis B</t>
         </is>
       </c>
       <c r="G41" s="14" t="n">
@@ -3722,7 +3722,7 @@
       </c>
       <c r="H41" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I41" s="1" t="n"/>
@@ -3751,27 +3751,27 @@
       </c>
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>Acetaminophen toxic metabolite: which is right?</t>
+          <t>NSAID site: which is right?</t>
         </is>
       </c>
       <c r="C42" s="16" t="inlineStr">
         <is>
-          <t>Alters RA’s course, not just symptoms</t>
+          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
         </is>
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
+          <t>COX → prostaglandins specifically</t>
         </is>
       </c>
       <c r="E42" s="16" t="inlineStr">
         <is>
-          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
+          <t>More potent; more GI/CNS effects</t>
         </is>
       </c>
       <c r="F42" s="16" t="inlineStr">
         <is>
-          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
+          <t>Alters lysosomal and TLR signaling</t>
         </is>
       </c>
       <c r="G42" s="14" t="n">
@@ -3808,27 +3808,27 @@
       </c>
       <c r="B43" s="16" t="inlineStr">
         <is>
-          <t>Acetaminophen antidote: which is right?</t>
+          <t>Acetaminophen effects: which is right?</t>
         </is>
       </c>
       <c r="C43" s="16" t="inlineStr">
         <is>
-          <t>Common first-line for mild-moderate pain</t>
+          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>Nociceptive · inflammatory · neuropathic</t>
+          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
         </is>
       </c>
       <c r="E43" s="16" t="inlineStr">
         <is>
-          <t>N-acetylcysteine — glutathione precursor</t>
+          <t>Persists beyond expected healing, often &gt; 3 months</t>
         </is>
       </c>
       <c r="F43" s="16" t="inlineStr">
         <is>
-          <t>Baseline eye exam; annual after 5 years</t>
+          <t>Housekeeping: gastric protection, renal blood flow</t>
         </is>
       </c>
       <c r="G43" s="14" t="n">
@@ -3836,7 +3836,7 @@
       </c>
       <c r="H43" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I43" s="1" t="n"/>
@@ -3865,35 +3865,35 @@
       </c>
       <c r="B44" s="16" t="inlineStr">
         <is>
-          <t>Hidden acetaminophen: which is right?</t>
+          <t>Acetaminophen toxic metabolite: which is right?</t>
         </is>
       </c>
       <c r="C44" s="16" t="inlineStr">
         <is>
-          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
+          <t>Alters RA’s course, not just symptoms</t>
         </is>
       </c>
       <c r="D44" s="16" t="inlineStr">
         <is>
-          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
+          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
         </is>
       </c>
       <c r="E44" s="16" t="inlineStr">
         <is>
-          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
+          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
         </is>
       </c>
       <c r="F44" s="16" t="inlineStr">
         <is>
-          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
+          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
         </is>
       </c>
       <c r="G44" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H44" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I44" s="1" t="n"/>
@@ -3922,27 +3922,27 @@
       </c>
       <c r="B45" s="16" t="inlineStr">
         <is>
-          <t>COX-1: which is right?</t>
+          <t>Acetaminophen antidote: which is right?</t>
         </is>
       </c>
       <c r="C45" s="16" t="inlineStr">
         <is>
-          <t>Persists beyond expected healing, often &gt; 3 months</t>
+          <t>Common first-line for mild-moderate pain</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
-          <t>Housekeeping: gastric protection, renal blood flow</t>
+          <t>CBC, liver, kidney labs every 1–3 months</t>
         </is>
       </c>
       <c r="E45" s="16" t="inlineStr">
         <is>
-          <t>TB + hepatitis B/C screen; update vaccines (live) first</t>
+          <t>Nociceptive · inflammatory · neuropathic</t>
         </is>
       </c>
       <c r="F45" s="16" t="inlineStr">
         <is>
-          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
+          <t>N-acetylcysteine — glutathione precursor</t>
         </is>
       </c>
       <c r="G45" s="14" t="n">
@@ -3950,7 +3950,7 @@
       </c>
       <c r="H45" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I45" s="1" t="n"/>
@@ -3979,27 +3979,27 @@
       </c>
       <c r="B46" s="16" t="inlineStr">
         <is>
-          <t>COX-2: which is right?</t>
+          <t>Hidden acetaminophen: which is right?</t>
         </is>
       </c>
       <c r="C46" s="16" t="inlineStr">
         <is>
+          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
+        </is>
+      </c>
+      <c r="D46" s="16" t="inlineStr">
+        <is>
+          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
+        </is>
+      </c>
+      <c r="E46" s="16" t="inlineStr">
+        <is>
+          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
+        </is>
+      </c>
+      <c r="F46" s="16" t="inlineStr">
+        <is>
           <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
-        </is>
-      </c>
-      <c r="D46" s="16" t="inlineStr">
-        <is>
-          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
-        </is>
-      </c>
-      <c r="E46" s="16" t="inlineStr">
-        <is>
-          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
-        </is>
-      </c>
-      <c r="F46" s="16" t="inlineStr">
-        <is>
-          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
         </is>
       </c>
       <c r="G46" s="14" t="n">
@@ -4007,7 +4007,7 @@
       </c>
       <c r="H46" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I46" s="1" t="n"/>
@@ -4036,27 +4036,27 @@
       </c>
       <c r="B47" s="16" t="inlineStr">
         <is>
-          <t>Ibuprofen: which is right?</t>
+          <t>COX-1: which is right?</t>
         </is>
       </c>
       <c r="C47" s="16" t="inlineStr">
         <is>
-          <t>Nociceptive · inflammatory · neuropathic</t>
+          <t>Persists beyond expected healing, often &gt; 3 months</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>N-acetylcysteine — glutathione precursor</t>
+          <t>Housekeeping: gastric protection, renal blood flow</t>
         </is>
       </c>
       <c r="E47" s="16" t="inlineStr">
         <is>
-          <t>Common first-line for mild-moderate pain</t>
+          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
         </is>
       </c>
       <c r="F47" s="16" t="inlineStr">
         <is>
-          <t>Baseline eye exam; annual after 5 years</t>
+          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
         </is>
       </c>
       <c r="G47" s="14" t="n">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="H47" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I47" s="1" t="n"/>
@@ -4093,35 +4093,35 @@
       </c>
       <c r="B48" s="16" t="inlineStr">
         <is>
-          <t>Naproxen: which is right?</t>
+          <t>COX-2: which is right?</t>
         </is>
       </c>
       <c r="C48" s="16" t="inlineStr">
         <is>
-          <t>≤ 7.5 mg daily long term, taper</t>
+          <t>~90% glucuronidation/sulfation (safe) · ~5–10% CYP2E1 → NAPQI</t>
         </is>
       </c>
       <c r="D48" s="16" t="inlineStr">
         <is>
-          <t>Immunosuppression → infection</t>
+          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
         </is>
       </c>
       <c r="E48" s="16" t="inlineStr">
         <is>
-          <t>10–20× more selective for COX-2</t>
+          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
         </is>
       </c>
       <c r="F48" s="16" t="inlineStr">
         <is>
-          <t>Longer half-life, twice-daily</t>
+          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
         </is>
       </c>
       <c r="G48" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H48" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I48" s="1" t="n"/>
@@ -4150,35 +4150,35 @@
       </c>
       <c r="B49" s="16" t="inlineStr">
         <is>
-          <t>Diclofenac: which is right?</t>
+          <t>Ibuprofen: which is right?</t>
         </is>
       </c>
       <c r="C49" s="16" t="inlineStr">
         <is>
-          <t>Abatacept</t>
+          <t>Nociceptive · inflammatory · neuropathic</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
         <is>
-          <t>Tocilizumab</t>
+          <t>N-acetylcysteine — glutathione precursor</t>
         </is>
       </c>
       <c r="E49" s="16" t="inlineStr">
         <is>
-          <t>↑ GI ulcer risk</t>
+          <t>Common first-line for mild-moderate pain</t>
         </is>
       </c>
       <c r="F49" s="16" t="inlineStr">
         <is>
-          <t>Oral and topical</t>
+          <t>CBC, liver, kidney labs every 1–3 months</t>
         </is>
       </c>
       <c r="G49" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H49" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I49" s="1" t="n"/>
@@ -4207,27 +4207,27 @@
       </c>
       <c r="B50" s="16" t="inlineStr">
         <is>
-          <t>Indomethacin: which is right?</t>
+          <t>Naproxen: which is right?</t>
         </is>
       </c>
       <c r="C50" s="16" t="inlineStr">
         <is>
-          <t>More potent; more GI/CNS effects</t>
+          <t>≤ 7.5 mg daily long term, taper</t>
         </is>
       </c>
       <c r="D50" s="16" t="inlineStr">
         <is>
-          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
+          <t>Immunosuppression → infection</t>
         </is>
       </c>
       <c r="E50" s="16" t="inlineStr">
         <is>
-          <t>10–20× more selective for COX-2</t>
+          <t>DHODH (pyrimidine synthesis)</t>
         </is>
       </c>
       <c r="F50" s="16" t="inlineStr">
         <is>
-          <t>COX → prostaglandins specifically</t>
+          <t>Longer half-life, twice-daily</t>
         </is>
       </c>
       <c r="G50" s="14" t="n">
@@ -4235,7 +4235,7 @@
       </c>
       <c r="H50" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I50" s="1" t="n"/>
@@ -4264,31 +4264,31 @@
       </c>
       <c r="B51" s="16" t="inlineStr">
         <is>
-          <t>Ketorolac: which is right?</t>
+          <t>Diclofenac: which is right?</t>
         </is>
       </c>
       <c r="C51" s="16" t="inlineStr">
         <is>
-          <t>Nociceptive · inflammatory · neuropathic</t>
+          <t>Centrilobular necrosis</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>N-acetylcysteine — glutathione precursor</t>
+          <t>Tocilizumab</t>
         </is>
       </c>
       <c r="E51" s="16" t="inlineStr">
         <is>
-          <t>Common first-line for mild-moderate pain</t>
+          <t>↑ GI ulcer risk</t>
         </is>
       </c>
       <c r="F51" s="16" t="inlineStr">
         <is>
-          <t>Short-term only; significant GI/renal risk</t>
+          <t>Oral and topical</t>
         </is>
       </c>
       <c r="G51" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H51" s="18" t="inlineStr">
         <is>
@@ -4321,27 +4321,27 @@
       </c>
       <c r="B52" s="16" t="inlineStr">
         <is>
-          <t>Celecoxib trade-off: which is right?</t>
+          <t>Indomethacin: which is right?</t>
         </is>
       </c>
       <c r="C52" s="16" t="inlineStr">
         <is>
-          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
+          <t>More potent; more GI/CNS effects</t>
         </is>
       </c>
       <c r="D52" s="16" t="inlineStr">
         <is>
-          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
+          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
         </is>
       </c>
       <c r="E52" s="16" t="inlineStr">
         <is>
-          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
+          <t>10–20× more selective for COX-2</t>
         </is>
       </c>
       <c r="F52" s="16" t="inlineStr">
         <is>
-          <t>Alters RA’s course, not just symptoms</t>
+          <t>COX → prostaglandins specifically</t>
         </is>
       </c>
       <c r="G52" s="14" t="n">
@@ -4349,7 +4349,7 @@
       </c>
       <c r="H52" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I52" s="1" t="n"/>
@@ -4378,27 +4378,27 @@
       </c>
       <c r="B53" s="16" t="inlineStr">
         <is>
-          <t>NSAID adverse effects: which is right?</t>
+          <t>Ketorolac: which is right?</t>
         </is>
       </c>
       <c r="C53" s="16" t="inlineStr">
         <is>
-          <t>TB + hepatitis B/C screen; update vaccines (live) first</t>
+          <t>Nociceptive · inflammatory · neuropathic</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
+          <t>CBC, liver, kidney labs every 1–3 months</t>
         </is>
       </c>
       <c r="E53" s="16" t="inlineStr">
         <is>
-          <t>Baricitinib, tofacitinib, upadacitinib — oral; zoster, ↑ LDL</t>
+          <t>8 h, 120 mcg/mL → above the line → start NAC</t>
         </is>
       </c>
       <c r="F53" s="16" t="inlineStr">
         <is>
-          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
+          <t>Short-term only; significant GI/renal risk</t>
         </is>
       </c>
       <c r="G53" s="14" t="n">
@@ -4435,31 +4435,31 @@
       </c>
       <c r="B54" s="16" t="inlineStr">
         <is>
-          <t>NSAID cautions: which is right?</t>
+          <t>Celecoxib trade-off: which is right?</t>
         </is>
       </c>
       <c r="C54" s="16" t="inlineStr">
         <is>
-          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
+          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
         </is>
       </c>
       <c r="D54" s="16" t="inlineStr">
         <is>
-          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
+          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
         </is>
       </c>
       <c r="E54" s="16" t="inlineStr">
         <is>
-          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
+          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
         </is>
       </c>
       <c r="F54" s="16" t="inlineStr">
         <is>
-          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
+          <t>Alters RA’s course, not just symptoms</t>
         </is>
       </c>
       <c r="G54" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H54" s="18" t="inlineStr">
         <is>
@@ -4492,35 +4492,35 @@
       </c>
       <c r="B55" s="16" t="inlineStr">
         <is>
-          <t>Triple whammy: which is right?</t>
+          <t>NSAID adverse effects: which is right?</t>
         </is>
       </c>
       <c r="C55" s="16" t="inlineStr">
         <is>
-          <t>Adalimumab, etanercept, infliximab</t>
+          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
+          <t>Anti-CD20; after TNF-inhibitor failure; check hepatitis B</t>
         </is>
       </c>
       <c r="E55" s="16" t="inlineStr">
         <is>
-          <t>COX → prostaglandins specifically</t>
+          <t>NSAID relief in days · DMARD protection over weeks–months</t>
         </is>
       </c>
       <c r="F55" s="16" t="inlineStr">
         <is>
-          <t>More potent; more GI/CNS effects</t>
+          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
         </is>
       </c>
       <c r="G55" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H55" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I55" s="1" t="n"/>
@@ -4549,31 +4549,31 @@
       </c>
       <c r="B56" s="16" t="inlineStr">
         <is>
-          <t>NSAID + corticosteroid: which is right?</t>
+          <t>NSAID cautions: which is right?</t>
         </is>
       </c>
       <c r="C56" s="16" t="inlineStr">
         <is>
-          <t>Tocilizumab</t>
+          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
         </is>
       </c>
       <c r="D56" s="16" t="inlineStr">
         <is>
-          <t>↑ GI ulcer risk</t>
+          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
         </is>
       </c>
       <c r="E56" s="16" t="inlineStr">
         <is>
-          <t>Rituximab</t>
+          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
         </is>
       </c>
       <c r="F56" s="16" t="inlineStr">
         <is>
-          <t>Oral and topical</t>
+          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
         </is>
       </c>
       <c r="G56" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H56" s="18" t="inlineStr">
         <is>
@@ -4606,35 +4606,35 @@
       </c>
       <c r="B57" s="16" t="inlineStr">
         <is>
-          <t>OA vs. RA: which is right?</t>
+          <t>Triple whammy: which is right?</t>
         </is>
       </c>
       <c r="C57" s="16" t="inlineStr">
         <is>
-          <t>Baricitinib, tofacitinib, upadacitinib — oral; zoster, ↑ LDL</t>
+          <t>Alters lysosomal and TLR signaling</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
+          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
         </is>
       </c>
       <c r="E57" s="16" t="inlineStr">
         <is>
-          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
+          <t>COX → prostaglandins specifically</t>
         </is>
       </c>
       <c r="F57" s="16" t="inlineStr">
         <is>
-          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
+          <t>More potent; more GI/CNS effects</t>
         </is>
       </c>
       <c r="G57" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H57" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I57" s="1" t="n"/>
@@ -4663,27 +4663,27 @@
       </c>
       <c r="B58" s="16" t="inlineStr">
         <is>
-          <t>DMARD: which is right?</t>
+          <t>NSAID + corticosteroid: which is right?</t>
         </is>
       </c>
       <c r="C58" s="16" t="inlineStr">
         <is>
-          <t>Alters RA’s course, not just symptoms</t>
+          <t>Tocilizumab</t>
         </is>
       </c>
       <c r="D58" s="16" t="inlineStr">
         <is>
-          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
+          <t>↑ GI ulcer risk</t>
         </is>
       </c>
       <c r="E58" s="16" t="inlineStr">
         <is>
-          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
+          <t>Rituximab</t>
         </is>
       </c>
       <c r="F58" s="16" t="inlineStr">
         <is>
-          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
+          <t>Oral and topical</t>
         </is>
       </c>
       <c r="G58" s="14" t="n">
@@ -4691,7 +4691,7 @@
       </c>
       <c r="H58" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I58" s="1" t="n"/>
@@ -4720,27 +4720,27 @@
       </c>
       <c r="B59" s="16" t="inlineStr">
         <is>
-          <t>Methotrexate: which is right?</t>
+          <t>OA vs. RA: which is right?</t>
         </is>
       </c>
       <c r="C59" s="16" t="inlineStr">
         <is>
-          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
+          <t>Baricitinib, tofacitinib, upadacitinib — oral; zoster, ↑ LDL</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
         <is>
-          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
+          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
         </is>
       </c>
       <c r="E59" s="16" t="inlineStr">
         <is>
-          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
+          <t>~90% glucuronidation/sulfation (safe) · ~5–10% CYP2E1 → NAPQI</t>
         </is>
       </c>
       <c r="F59" s="16" t="inlineStr">
         <is>
-          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
+          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
         </is>
       </c>
       <c r="G59" s="14" t="n">
@@ -4777,27 +4777,27 @@
       </c>
       <c r="B60" s="16" t="inlineStr">
         <is>
-          <t>TNF inhibitors: which is right?</t>
+          <t>DMARD: which is right?</t>
         </is>
       </c>
       <c r="C60" s="16" t="inlineStr">
         <is>
-          <t>More potent; more GI/CNS effects</t>
+          <t>Alters RA’s course, not just symptoms</t>
         </is>
       </c>
       <c r="D60" s="16" t="inlineStr">
         <is>
-          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
+          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
         </is>
       </c>
       <c r="E60" s="16" t="inlineStr">
         <is>
-          <t>COX → prostaglandins specifically</t>
+          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
         </is>
       </c>
       <c r="F60" s="16" t="inlineStr">
         <is>
-          <t>Adalimumab, etanercept, infliximab</t>
+          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
         </is>
       </c>
       <c r="G60" s="14" t="n">
@@ -4805,7 +4805,7 @@
       </c>
       <c r="H60" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I60" s="1" t="n"/>
@@ -4834,35 +4834,35 @@
       </c>
       <c r="B61" s="16" t="inlineStr">
         <is>
-          <t>IL-6 inhibitor: which is right?</t>
+          <t>Methotrexate: which is right?</t>
         </is>
       </c>
       <c r="C61" s="16" t="inlineStr">
         <is>
-          <t>Tocilizumab</t>
+          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>Rituximab</t>
+          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
         </is>
       </c>
       <c r="E61" s="16" t="inlineStr">
         <is>
-          <t>Abatacept</t>
+          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
         </is>
       </c>
       <c r="F61" s="16" t="inlineStr">
         <is>
-          <t>↑ GI ulcer risk</t>
+          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
         </is>
       </c>
       <c r="G61" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H61" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I61" s="1" t="n"/>
@@ -4891,27 +4891,27 @@
       </c>
       <c r="B62" s="16" t="inlineStr">
         <is>
-          <t>B-cell therapy: which is right?</t>
+          <t>TNF inhibitors: which is right?</t>
         </is>
       </c>
       <c r="C62" s="16" t="inlineStr">
         <is>
-          <t>Abatacept</t>
+          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
         </is>
       </c>
       <c r="D62" s="16" t="inlineStr">
         <is>
-          <t>Tocilizumab</t>
+          <t>COX → prostaglandins specifically</t>
         </is>
       </c>
       <c r="E62" s="16" t="inlineStr">
         <is>
-          <t>Rituximab</t>
+          <t>Alters lysosomal and TLR signaling</t>
         </is>
       </c>
       <c r="F62" s="16" t="inlineStr">
         <is>
-          <t>↑ GI ulcer risk</t>
+          <t>Adalimumab, etanercept, infliximab</t>
         </is>
       </c>
       <c r="G62" s="14" t="n">
@@ -4919,7 +4919,7 @@
       </c>
       <c r="H62" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I62" s="1" t="n"/>
@@ -4948,22 +4948,22 @@
       </c>
       <c r="B63" s="16" t="inlineStr">
         <is>
-          <t>T-cell costimulation: which is right?</t>
+          <t>IL-6 inhibitor: which is right?</t>
         </is>
       </c>
       <c r="C63" s="16" t="inlineStr">
         <is>
+          <t>Tocilizumab</t>
+        </is>
+      </c>
+      <c r="D63" s="16" t="inlineStr">
+        <is>
           <t>Rituximab</t>
         </is>
       </c>
-      <c r="D63" s="16" t="inlineStr">
+      <c r="E63" s="16" t="inlineStr">
         <is>
           <t>Abatacept</t>
-        </is>
-      </c>
-      <c r="E63" s="16" t="inlineStr">
-        <is>
-          <t>Tocilizumab</t>
         </is>
       </c>
       <c r="F63" s="16" t="inlineStr">
@@ -4976,7 +4976,7 @@
       </c>
       <c r="H63" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I63" s="1" t="n"/>
@@ -5005,27 +5005,27 @@
       </c>
       <c r="B64" s="16" t="inlineStr">
         <is>
-          <t>DMARD shared risk: which is right?</t>
+          <t>B-cell therapy: which is right?</t>
         </is>
       </c>
       <c r="C64" s="16" t="inlineStr">
         <is>
-          <t>Immunosuppression → infection</t>
+          <t>Abatacept</t>
         </is>
       </c>
       <c r="D64" s="16" t="inlineStr">
         <is>
-          <t>≤ 7.5 mg daily long term, taper</t>
+          <t>Tocilizumab</t>
         </is>
       </c>
       <c r="E64" s="16" t="inlineStr">
         <is>
-          <t>Longer half-life, twice-daily</t>
+          <t>Rituximab</t>
         </is>
       </c>
       <c r="F64" s="16" t="inlineStr">
         <is>
-          <t>7.5 mg weekly → 15–25 mg weekly</t>
+          <t>↑ GI ulcer risk</t>
         </is>
       </c>
       <c r="G64" s="14" t="n">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="H64" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I64" s="1" t="n"/>
@@ -5062,35 +5062,35 @@
       </c>
       <c r="B65" s="16" t="inlineStr">
         <is>
-          <t>Before biologics: which is right?</t>
+          <t>T-cell costimulation: which is right?</t>
         </is>
       </c>
       <c r="C65" s="16" t="inlineStr">
         <is>
-          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
+          <t>Rituximab</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
         <is>
-          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
+          <t>Abatacept</t>
         </is>
       </c>
       <c r="E65" s="16" t="inlineStr">
         <is>
-          <t>TB + hepatitis B/C screen; update vaccines (live) first</t>
+          <t>Tocilizumab</t>
         </is>
       </c>
       <c r="F65" s="16" t="inlineStr">
         <is>
-          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
+          <t>↑ GI ulcer risk</t>
         </is>
       </c>
       <c r="G65" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H65" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I65" s="1" t="n"/>
@@ -5119,27 +5119,27 @@
       </c>
       <c r="B66" s="16" t="inlineStr">
         <is>
-          <t>Acetaminophen max (adults): which is right?</t>
+          <t>DMARD shared risk: which is right?</t>
         </is>
       </c>
       <c r="C66" s="16" t="inlineStr">
         <is>
-          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
+          <t>DHODH (pyrimidine synthesis)</t>
         </is>
       </c>
       <c r="D66" s="16" t="inlineStr">
         <is>
-          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
+          <t>Immunosuppression → infection</t>
         </is>
       </c>
       <c r="E66" s="16" t="inlineStr">
         <is>
-          <t>Alters RA’s course, not just symptoms</t>
+          <t>≤ 7.5 mg daily long term, taper</t>
         </is>
       </c>
       <c r="F66" s="16" t="inlineStr">
         <is>
-          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
+          <t>Longer half-life, twice-daily</t>
         </is>
       </c>
       <c r="G66" s="14" t="n">
@@ -5147,7 +5147,7 @@
       </c>
       <c r="H66" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I66" s="1" t="n"/>
@@ -5176,27 +5176,27 @@
       </c>
       <c r="B67" s="16" t="inlineStr">
         <is>
-          <t>Aspirin vs. other NSAIDs: which is right?</t>
+          <t>Before biologics: which is right?</t>
         </is>
       </c>
       <c r="C67" s="16" t="inlineStr">
         <is>
-          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
+          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
         <is>
-          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
+          <t>TB + hepatitis B/C screen; update vaccines (live) first</t>
         </is>
       </c>
       <c r="E67" s="16" t="inlineStr">
         <is>
-          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
+          <t>NSAID relief in days · DMARD protection over weeks–months</t>
         </is>
       </c>
       <c r="F67" s="16" t="inlineStr">
         <is>
-          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
+          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
         </is>
       </c>
       <c r="G67" s="14" t="n">
@@ -5233,35 +5233,35 @@
       </c>
       <c r="B68" s="16" t="inlineStr">
         <is>
-          <t>Celecoxib selectivity: which is right?</t>
+          <t>Acetaminophen routes: which is right?</t>
         </is>
       </c>
       <c r="C68" s="16" t="inlineStr">
         <is>
-          <t>Malignancy, especially lymphoma</t>
+          <t>~90% glucuronidation/sulfation (safe) · ~5–10% CYP2E1 → NAPQI</t>
         </is>
       </c>
       <c r="D68" s="16" t="inlineStr">
         <is>
-          <t>10–20× more selective for COX-2</t>
+          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
         </is>
       </c>
       <c r="E68" s="16" t="inlineStr">
         <is>
-          <t>≤ 7.5 mg daily long term, taper</t>
+          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
         </is>
       </c>
       <c r="F68" s="16" t="inlineStr">
         <is>
-          <t>7.5 mg weekly → 15–25 mg weekly</t>
+          <t>Baricitinib, tofacitinib, upadacitinib — oral; zoster, ↑ LDL</t>
         </is>
       </c>
       <c r="G68" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H68" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I68" s="1" t="n"/>
@@ -5290,35 +5290,35 @@
       </c>
       <c r="B69" s="16" t="inlineStr">
         <is>
-          <t>Methotrexate dose: which is right?</t>
+          <t>Who's at higher acetaminophen risk: which is right?</t>
         </is>
       </c>
       <c r="C69" s="16" t="inlineStr">
         <is>
-          <t>10–20× more selective for COX-2</t>
+          <t>Synovitis → pannus; TNF-α and IL-6 drive erosion</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
         <is>
-          <t>Malignancy, especially lymphoma</t>
+          <t>Chronic alcohol use, fasting (↓ GSH, ↑ CYP2E1)</t>
         </is>
       </c>
       <c r="E69" s="16" t="inlineStr">
         <is>
-          <t>≤ 7.5 mg daily long term, taper</t>
+          <t>Likely anti-inflammatory via adenosine release</t>
         </is>
       </c>
       <c r="F69" s="16" t="inlineStr">
         <is>
-          <t>7.5 mg weekly → 15–25 mg weekly</t>
+          <t>8 h, 120 mcg/mL → above the line → start NAC</t>
         </is>
       </c>
       <c r="G69" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H69" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I69" s="1" t="n"/>
@@ -5347,27 +5347,27 @@
       </c>
       <c r="B70" s="16" t="inlineStr">
         <is>
-          <t>Hydroxychloroquine monitoring: which is right?</t>
+          <t>Liver lesion in overdose: which is right?</t>
         </is>
       </c>
       <c r="C70" s="16" t="inlineStr">
         <is>
-          <t>Baseline eye exam; annual after 5 years</t>
+          <t>PGI2 falls, TXA2 preserved</t>
         </is>
       </c>
       <c r="D70" s="16" t="inlineStr">
         <is>
-          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
+          <t>Centrilobular necrosis</t>
         </is>
       </c>
       <c r="E70" s="16" t="inlineStr">
         <is>
-          <t>Nociceptive · inflammatory · neuropathic</t>
+          <t>VTE (DVT/PE), MACE, cancer</t>
         </is>
       </c>
       <c r="F70" s="16" t="inlineStr">
         <is>
-          <t>Common first-line for mild-moderate pain</t>
+          <t>DHODH (pyrimidine synthesis)</t>
         </is>
       </c>
       <c r="G70" s="14" t="n">
@@ -5375,7 +5375,7 @@
       </c>
       <c r="H70" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I70" s="1" t="n"/>
@@ -5404,35 +5404,35 @@
       </c>
       <c r="B71" s="16" t="inlineStr">
         <is>
-          <t>TNF inhibitor boxed warning: which is right?</t>
+          <t>Rumack-Matthew nomogram: which is right?</t>
         </is>
       </c>
       <c r="C71" s="16" t="inlineStr">
         <is>
-          <t>10–20× more selective for COX-2</t>
+          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
         <is>
-          <t>7.5 mg weekly → 15–25 mg weekly</t>
+          <t>Single acute ingestion; level ≥ 4 h; above the line → NAC; not used &gt; 24 h</t>
         </is>
       </c>
       <c r="E71" s="16" t="inlineStr">
         <is>
-          <t>Malignancy, especially lymphoma</t>
+          <t>Prostaglandins, bradykinin, histamine, cytokines (TNF-α, IL-1, IL-6)</t>
         </is>
       </c>
       <c r="F71" s="16" t="inlineStr">
         <is>
-          <t>≤ 7.5 mg daily long term, taper</t>
+          <t>GI: ↓ mucus/bicarbonate · kidney: ↓ afferent dilation · platelets: ↓ TXA2</t>
         </is>
       </c>
       <c r="G71" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H71" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I71" s="1" t="n"/>
@@ -5461,31 +5461,31 @@
       </c>
       <c r="B72" s="16" t="inlineStr">
         <is>
-          <t>JAK inhibitor boxed warning: which is right?</t>
+          <t>Nomogram example: which is right?</t>
         </is>
       </c>
       <c r="C72" s="16" t="inlineStr">
         <is>
-          <t>Immunosuppression → infection</t>
+          <t>Chronic alcohol use, fasting (↓ GSH, ↑ CYP2E1)</t>
         </is>
       </c>
       <c r="D72" s="16" t="inlineStr">
         <is>
-          <t>VTE (DVT/PE), MACE, cancer</t>
+          <t>8 h, 120 mcg/mL → above the line → start NAC</t>
         </is>
       </c>
       <c r="E72" s="16" t="inlineStr">
         <is>
-          <t>Longer half-life, twice-daily</t>
+          <t>Likely anti-inflammatory via adenosine release</t>
         </is>
       </c>
       <c r="F72" s="16" t="inlineStr">
         <is>
-          <t>7.5 mg weekly → 15–25 mg weekly</t>
+          <t>Short-term only; significant GI/renal risk</t>
         </is>
       </c>
       <c r="G72" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H72" s="18" t="inlineStr">
         <is>
@@ -5518,27 +5518,27 @@
       </c>
       <c r="B73" s="16" t="inlineStr">
         <is>
-          <t>JAK inhibitors: which is right?</t>
+          <t>Nomogram line (illustrative): which is right?</t>
         </is>
       </c>
       <c r="C73" s="16" t="inlineStr">
         <is>
-          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
+          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
         </is>
       </c>
       <c r="D73" s="16" t="inlineStr">
         <is>
-          <t>Baricitinib, tofacitinib, upadacitinib — oral; zoster, ↑ LDL</t>
+          <t>Persists beyond expected healing, often &gt; 3 months</t>
         </is>
       </c>
       <c r="E73" s="16" t="inlineStr">
         <is>
-          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
+          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
         </is>
       </c>
       <c r="F73" s="16" t="inlineStr">
         <is>
-          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
+          <t>Housekeeping: gastric protection, renal blood flow</t>
         </is>
       </c>
       <c r="G73" s="14" t="n">
@@ -5546,7 +5546,7 @@
       </c>
       <c r="H73" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I73" s="1" t="n"/>
@@ -5575,27 +5575,27 @@
       </c>
       <c r="B74" s="16" t="inlineStr">
         <is>
-          <t>RA prednisone ceiling: which is right?</t>
+          <t>Celecoxib CV mechanism: which is right?</t>
         </is>
       </c>
       <c r="C74" s="16" t="inlineStr">
         <is>
-          <t>7.5 mg weekly → 15–25 mg weekly</t>
+          <t>Longer half-life, twice-daily</t>
         </is>
       </c>
       <c r="D74" s="16" t="inlineStr">
         <is>
-          <t>≤ 7.5 mg daily long term, taper</t>
+          <t>VTE (DVT/PE), MACE, cancer</t>
         </is>
       </c>
       <c r="E74" s="16" t="inlineStr">
         <is>
-          <t>Malignancy, especially lymphoma</t>
+          <t>PGI2 falls, TXA2 preserved</t>
         </is>
       </c>
       <c r="F74" s="16" t="inlineStr">
         <is>
-          <t>10–20× more selective for COX-2</t>
+          <t>DHODH (pyrimidine synthesis)</t>
         </is>
       </c>
       <c r="G74" s="14" t="n">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="H74" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I74" s="1" t="n"/>
@@ -5627,14 +5627,42 @@
       <c r="AA74" s="1" t="n"/>
     </row>
     <row r="75" ht="25.5" customHeight="1">
-      <c r="A75" s="11" t="n"/>
-      <c r="B75" s="16" t="n"/>
-      <c r="C75" s="16" t="n"/>
-      <c r="D75" s="16" t="n"/>
-      <c r="E75" s="16" t="n"/>
-      <c r="F75" s="16" t="n"/>
-      <c r="G75" s="14" t="n"/>
-      <c r="H75" s="18" t="n"/>
+      <c r="A75" s="11" t="n">
+        <v>67</v>
+      </c>
+      <c r="B75" s="16" t="inlineStr">
+        <is>
+          <t>NSAID organ effects: which is right?</t>
+        </is>
+      </c>
+      <c r="C75" s="16" t="inlineStr">
+        <is>
+          <t>GI: ↓ mucus/bicarbonate · kidney: ↓ afferent dilation · platelets: ↓ TXA2</t>
+        </is>
+      </c>
+      <c r="D75" s="16" t="inlineStr">
+        <is>
+          <t>Prostaglandins, bradykinin, histamine, cytokines (TNF-α, IL-1, IL-6)</t>
+        </is>
+      </c>
+      <c r="E75" s="16" t="inlineStr">
+        <is>
+          <t>Single acute ingestion; level ≥ 4 h; above the line → NAC; not used &gt; 24 h</t>
+        </is>
+      </c>
+      <c r="F75" s="16" t="inlineStr">
+        <is>
+          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
+        </is>
+      </c>
+      <c r="G75" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="H75" s="18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="I75" s="1" t="n"/>
       <c r="J75" s="1" t="n"/>
       <c r="K75" s="1" t="n"/>
@@ -5656,14 +5684,42 @@
       <c r="AA75" s="1" t="n"/>
     </row>
     <row r="76" ht="25.5" customHeight="1">
-      <c r="A76" s="11" t="n"/>
-      <c r="B76" s="16" t="n"/>
-      <c r="C76" s="16" t="n"/>
-      <c r="D76" s="16" t="n"/>
-      <c r="E76" s="16" t="n"/>
-      <c r="F76" s="16" t="n"/>
-      <c r="G76" s="14" t="n"/>
-      <c r="H76" s="18" t="n"/>
+      <c r="A76" s="11" t="n">
+        <v>68</v>
+      </c>
+      <c r="B76" s="16" t="inlineStr">
+        <is>
+          <t>RA joint destruction: which is right?</t>
+        </is>
+      </c>
+      <c r="C76" s="16" t="inlineStr">
+        <is>
+          <t>Synovitis → pannus; TNF-α and IL-6 drive erosion</t>
+        </is>
+      </c>
+      <c r="D76" s="16" t="inlineStr">
+        <is>
+          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
+        </is>
+      </c>
+      <c r="E76" s="16" t="inlineStr">
+        <is>
+          <t>Housekeeping: gastric protection, renal blood flow</t>
+        </is>
+      </c>
+      <c r="F76" s="16" t="inlineStr">
+        <is>
+          <t>Chronic alcohol use, fasting (↓ GSH, ↑ CYP2E1)</t>
+        </is>
+      </c>
+      <c r="G76" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="H76" s="18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="I76" s="1" t="n"/>
       <c r="J76" s="1" t="n"/>
       <c r="K76" s="1" t="n"/>
@@ -5685,14 +5741,42 @@
       <c r="AA76" s="1" t="n"/>
     </row>
     <row r="77" ht="25.5" customHeight="1">
-      <c r="A77" s="11" t="n"/>
-      <c r="B77" s="16" t="n"/>
-      <c r="C77" s="16" t="n"/>
-      <c r="D77" s="16" t="n"/>
-      <c r="E77" s="16" t="n"/>
-      <c r="F77" s="16" t="n"/>
-      <c r="G77" s="14" t="n"/>
-      <c r="H77" s="18" t="n"/>
+      <c r="A77" s="11" t="n">
+        <v>69</v>
+      </c>
+      <c r="B77" s="16" t="inlineStr">
+        <is>
+          <t>NSAID vs. DMARD onset: which is right?</t>
+        </is>
+      </c>
+      <c r="C77" s="16" t="inlineStr">
+        <is>
+          <t>Anti-CD20; after TNF-inhibitor failure; check hepatitis B</t>
+        </is>
+      </c>
+      <c r="D77" s="16" t="inlineStr">
+        <is>
+          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
+        </is>
+      </c>
+      <c r="E77" s="16" t="inlineStr">
+        <is>
+          <t>NSAID relief in days · DMARD protection over weeks–months</t>
+        </is>
+      </c>
+      <c r="F77" s="16" t="inlineStr">
+        <is>
+          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
+        </is>
+      </c>
+      <c r="G77" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="H77" s="18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="I77" s="1" t="n"/>
       <c r="J77" s="1" t="n"/>
       <c r="K77" s="1" t="n"/>
@@ -5714,14 +5798,42 @@
       <c r="AA77" s="1" t="n"/>
     </row>
     <row r="78" ht="25.5" customHeight="1">
-      <c r="A78" s="11" t="n"/>
-      <c r="B78" s="16" t="n"/>
-      <c r="C78" s="16" t="n"/>
-      <c r="D78" s="16" t="n"/>
-      <c r="E78" s="16" t="n"/>
-      <c r="F78" s="16" t="n"/>
-      <c r="G78" s="14" t="n"/>
-      <c r="H78" s="18" t="n"/>
+      <c r="A78" s="11" t="n">
+        <v>70</v>
+      </c>
+      <c r="B78" s="16" t="inlineStr">
+        <is>
+          <t>Leflunomide target: which is right?</t>
+        </is>
+      </c>
+      <c r="C78" s="16" t="inlineStr">
+        <is>
+          <t>PGI2 falls, TXA2 preserved</t>
+        </is>
+      </c>
+      <c r="D78" s="16" t="inlineStr">
+        <is>
+          <t>Immunosuppression → infection</t>
+        </is>
+      </c>
+      <c r="E78" s="16" t="inlineStr">
+        <is>
+          <t>DHODH (pyrimidine synthesis)</t>
+        </is>
+      </c>
+      <c r="F78" s="16" t="inlineStr">
+        <is>
+          <t>Longer half-life, twice-daily</t>
+        </is>
+      </c>
+      <c r="G78" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="H78" s="18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="I78" s="1" t="n"/>
       <c r="J78" s="1" t="n"/>
       <c r="K78" s="1" t="n"/>
@@ -5743,14 +5855,42 @@
       <c r="AA78" s="1" t="n"/>
     </row>
     <row r="79" ht="25.5" customHeight="1">
-      <c r="A79" s="11" t="n"/>
-      <c r="B79" s="16" t="n"/>
-      <c r="C79" s="16" t="n"/>
-      <c r="D79" s="16" t="n"/>
-      <c r="E79" s="16" t="n"/>
-      <c r="F79" s="16" t="n"/>
-      <c r="G79" s="14" t="n"/>
-      <c r="H79" s="18" t="n"/>
+      <c r="A79" s="11" t="n">
+        <v>71</v>
+      </c>
+      <c r="B79" s="16" t="inlineStr">
+        <is>
+          <t>Hydroxychloroquine action: which is right?</t>
+        </is>
+      </c>
+      <c r="C79" s="16" t="inlineStr">
+        <is>
+          <t>Alters lysosomal and TLR signaling</t>
+        </is>
+      </c>
+      <c r="D79" s="16" t="inlineStr">
+        <is>
+          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
+        </is>
+      </c>
+      <c r="E79" s="16" t="inlineStr">
+        <is>
+          <t>COX → prostaglandins specifically</t>
+        </is>
+      </c>
+      <c r="F79" s="16" t="inlineStr">
+        <is>
+          <t>Adalimumab, etanercept, infliximab</t>
+        </is>
+      </c>
+      <c r="G79" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="H79" s="18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="I79" s="1" t="n"/>
       <c r="J79" s="1" t="n"/>
       <c r="K79" s="1" t="n"/>
@@ -5772,14 +5912,42 @@
       <c r="AA79" s="1" t="n"/>
     </row>
     <row r="80" ht="25.5" customHeight="1">
-      <c r="A80" s="11" t="n"/>
-      <c r="B80" s="16" t="n"/>
-      <c r="C80" s="16" t="n"/>
-      <c r="D80" s="16" t="n"/>
-      <c r="E80" s="16" t="n"/>
-      <c r="F80" s="16" t="n"/>
-      <c r="G80" s="14" t="n"/>
-      <c r="H80" s="18" t="n"/>
+      <c r="A80" s="11" t="n">
+        <v>72</v>
+      </c>
+      <c r="B80" s="16" t="inlineStr">
+        <is>
+          <t>Methotrexate at low dose: which is right?</t>
+        </is>
+      </c>
+      <c r="C80" s="16" t="inlineStr">
+        <is>
+          <t>Synovitis → pannus; TNF-α and IL-6 drive erosion</t>
+        </is>
+      </c>
+      <c r="D80" s="16" t="inlineStr">
+        <is>
+          <t>Chronic alcohol use, fasting (↓ GSH, ↑ CYP2E1)</t>
+        </is>
+      </c>
+      <c r="E80" s="16" t="inlineStr">
+        <is>
+          <t>Likely anti-inflammatory via adenosine release</t>
+        </is>
+      </c>
+      <c r="F80" s="16" t="inlineStr">
+        <is>
+          <t>8 h, 120 mcg/mL → above the line → start NAC</t>
+        </is>
+      </c>
+      <c r="G80" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="H80" s="18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="I80" s="1" t="n"/>
       <c r="J80" s="1" t="n"/>
       <c r="K80" s="1" t="n"/>
@@ -5801,14 +5969,42 @@
       <c r="AA80" s="1" t="n"/>
     </row>
     <row r="81" ht="25.5" customHeight="1">
-      <c r="A81" s="11" t="n"/>
-      <c r="B81" s="16" t="n"/>
-      <c r="C81" s="16" t="n"/>
-      <c r="D81" s="16" t="n"/>
-      <c r="E81" s="16" t="n"/>
-      <c r="F81" s="16" t="n"/>
-      <c r="G81" s="14" t="n"/>
-      <c r="H81" s="18" t="n"/>
+      <c r="A81" s="11" t="n">
+        <v>73</v>
+      </c>
+      <c r="B81" s="16" t="inlineStr">
+        <is>
+          <t>Abatacept: which is right?</t>
+        </is>
+      </c>
+      <c r="C81" s="16" t="inlineStr">
+        <is>
+          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
+        </is>
+      </c>
+      <c r="D81" s="16" t="inlineStr">
+        <is>
+          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
+        </is>
+      </c>
+      <c r="E81" s="16" t="inlineStr">
+        <is>
+          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
+        </is>
+      </c>
+      <c r="F81" s="16" t="inlineStr">
+        <is>
+          <t>Prostaglandins, bradykinin, histamine, cytokines (TNF-α, IL-1, IL-6)</t>
+        </is>
+      </c>
+      <c r="G81" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="H81" s="18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="I81" s="1" t="n"/>
       <c r="J81" s="1" t="n"/>
       <c r="K81" s="1" t="n"/>
@@ -5830,14 +6026,42 @@
       <c r="AA81" s="1" t="n"/>
     </row>
     <row r="82" ht="25.5" customHeight="1">
-      <c r="A82" s="11" t="n"/>
-      <c r="B82" s="16" t="n"/>
-      <c r="C82" s="16" t="n"/>
-      <c r="D82" s="16" t="n"/>
-      <c r="E82" s="16" t="n"/>
-      <c r="F82" s="16" t="n"/>
-      <c r="G82" s="14" t="n"/>
-      <c r="H82" s="18" t="n"/>
+      <c r="A82" s="11" t="n">
+        <v>74</v>
+      </c>
+      <c r="B82" s="16" t="inlineStr">
+        <is>
+          <t>Rituximab: which is right?</t>
+        </is>
+      </c>
+      <c r="C82" s="16" t="inlineStr">
+        <is>
+          <t>Anti-CD20; after TNF-inhibitor failure; check hepatitis B</t>
+        </is>
+      </c>
+      <c r="D82" s="16" t="inlineStr">
+        <is>
+          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
+        </is>
+      </c>
+      <c r="E82" s="16" t="inlineStr">
+        <is>
+          <t>NSAID relief in days · DMARD protection over weeks–months</t>
+        </is>
+      </c>
+      <c r="F82" s="16" t="inlineStr">
+        <is>
+          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
+        </is>
+      </c>
+      <c r="G82" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="H82" s="18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="I82" s="1" t="n"/>
       <c r="J82" s="1" t="n"/>
       <c r="K82" s="1" t="n"/>
@@ -5859,14 +6083,42 @@
       <c r="AA82" s="1" t="n"/>
     </row>
     <row r="83" ht="25.5" customHeight="1">
-      <c r="A83" s="11" t="n"/>
-      <c r="B83" s="16" t="n"/>
-      <c r="C83" s="16" t="n"/>
-      <c r="D83" s="16" t="n"/>
-      <c r="E83" s="16" t="n"/>
-      <c r="F83" s="16" t="n"/>
-      <c r="G83" s="14" t="n"/>
-      <c r="H83" s="18" t="n"/>
+      <c r="A83" s="11" t="n">
+        <v>75</v>
+      </c>
+      <c r="B83" s="16" t="inlineStr">
+        <is>
+          <t>Infection monitoring on DMARDs: which is right?</t>
+        </is>
+      </c>
+      <c r="C83" s="16" t="inlineStr">
+        <is>
+          <t>CBC, liver, kidney labs every 1–3 months</t>
+        </is>
+      </c>
+      <c r="D83" s="16" t="inlineStr">
+        <is>
+          <t>Nociceptive · inflammatory · neuropathic</t>
+        </is>
+      </c>
+      <c r="E83" s="16" t="inlineStr">
+        <is>
+          <t>Common first-line for mild-moderate pain</t>
+        </is>
+      </c>
+      <c r="F83" s="16" t="inlineStr">
+        <is>
+          <t>N-acetylcysteine — glutathione precursor</t>
+        </is>
+      </c>
+      <c r="G83" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="H83" s="18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="I83" s="1" t="n"/>
       <c r="J83" s="1" t="n"/>
       <c r="K83" s="1" t="n"/>
@@ -5888,14 +6140,42 @@
       <c r="AA83" s="1" t="n"/>
     </row>
     <row r="84" ht="25.5" customHeight="1">
-      <c r="A84" s="11" t="n"/>
-      <c r="B84" s="16" t="n"/>
-      <c r="C84" s="16" t="n"/>
-      <c r="D84" s="16" t="n"/>
-      <c r="E84" s="16" t="n"/>
-      <c r="F84" s="16" t="n"/>
-      <c r="G84" s="14" t="n"/>
-      <c r="H84" s="18" t="n"/>
+      <c r="A84" s="11" t="n">
+        <v>76</v>
+      </c>
+      <c r="B84" s="16" t="inlineStr">
+        <is>
+          <t>Acetaminophen max (adults): which is right?</t>
+        </is>
+      </c>
+      <c r="C84" s="16" t="inlineStr">
+        <is>
+          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
+        </is>
+      </c>
+      <c r="D84" s="16" t="inlineStr">
+        <is>
+          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
+        </is>
+      </c>
+      <c r="E84" s="16" t="inlineStr">
+        <is>
+          <t>Alters RA’s course, not just symptoms</t>
+        </is>
+      </c>
+      <c r="F84" s="16" t="inlineStr">
+        <is>
+          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
+        </is>
+      </c>
+      <c r="G84" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="H84" s="18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="I84" s="1" t="n"/>
       <c r="J84" s="1" t="n"/>
       <c r="K84" s="1" t="n"/>
@@ -5917,14 +6197,42 @@
       <c r="AA84" s="1" t="n"/>
     </row>
     <row r="85" ht="25.5" customHeight="1">
-      <c r="A85" s="11" t="n"/>
-      <c r="B85" s="16" t="n"/>
-      <c r="C85" s="16" t="n"/>
-      <c r="D85" s="16" t="n"/>
-      <c r="E85" s="16" t="n"/>
-      <c r="F85" s="16" t="n"/>
-      <c r="G85" s="14" t="n"/>
-      <c r="H85" s="18" t="n"/>
+      <c r="A85" s="11" t="n">
+        <v>77</v>
+      </c>
+      <c r="B85" s="16" t="inlineStr">
+        <is>
+          <t>Aspirin vs. other NSAIDs: which is right?</t>
+        </is>
+      </c>
+      <c r="C85" s="16" t="inlineStr">
+        <is>
+          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
+        </is>
+      </c>
+      <c r="D85" s="16" t="inlineStr">
+        <is>
+          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
+        </is>
+      </c>
+      <c r="E85" s="16" t="inlineStr">
+        <is>
+          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
+        </is>
+      </c>
+      <c r="F85" s="16" t="inlineStr">
+        <is>
+          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
+        </is>
+      </c>
+      <c r="G85" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="H85" s="18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="I85" s="1" t="n"/>
       <c r="J85" s="1" t="n"/>
       <c r="K85" s="1" t="n"/>
@@ -5946,14 +6254,42 @@
       <c r="AA85" s="1" t="n"/>
     </row>
     <row r="86" ht="25.5" customHeight="1">
-      <c r="A86" s="11" t="n"/>
-      <c r="B86" s="16" t="n"/>
-      <c r="C86" s="16" t="n"/>
-      <c r="D86" s="16" t="n"/>
-      <c r="E86" s="16" t="n"/>
-      <c r="F86" s="16" t="n"/>
-      <c r="G86" s="14" t="n"/>
-      <c r="H86" s="18" t="n"/>
+      <c r="A86" s="11" t="n">
+        <v>78</v>
+      </c>
+      <c r="B86" s="16" t="inlineStr">
+        <is>
+          <t>Celecoxib selectivity: which is right?</t>
+        </is>
+      </c>
+      <c r="C86" s="16" t="inlineStr">
+        <is>
+          <t>Malignancy, especially lymphoma</t>
+        </is>
+      </c>
+      <c r="D86" s="16" t="inlineStr">
+        <is>
+          <t>10–20× more selective for COX-2</t>
+        </is>
+      </c>
+      <c r="E86" s="16" t="inlineStr">
+        <is>
+          <t>≤ 7.5 mg daily long term, taper</t>
+        </is>
+      </c>
+      <c r="F86" s="16" t="inlineStr">
+        <is>
+          <t>7.5 mg weekly → 15–25 mg weekly</t>
+        </is>
+      </c>
+      <c r="G86" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="H86" s="18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="I86" s="1" t="n"/>
       <c r="J86" s="1" t="n"/>
       <c r="K86" s="1" t="n"/>
@@ -5975,14 +6311,42 @@
       <c r="AA86" s="1" t="n"/>
     </row>
     <row r="87" ht="25.5" customHeight="1">
-      <c r="A87" s="11" t="n"/>
-      <c r="B87" s="16" t="n"/>
-      <c r="C87" s="16" t="n"/>
-      <c r="D87" s="16" t="n"/>
-      <c r="E87" s="16" t="n"/>
-      <c r="F87" s="16" t="n"/>
-      <c r="G87" s="14" t="n"/>
-      <c r="H87" s="18" t="n"/>
+      <c r="A87" s="11" t="n">
+        <v>79</v>
+      </c>
+      <c r="B87" s="16" t="inlineStr">
+        <is>
+          <t>Methotrexate dose: which is right?</t>
+        </is>
+      </c>
+      <c r="C87" s="16" t="inlineStr">
+        <is>
+          <t>10–20× more selective for COX-2</t>
+        </is>
+      </c>
+      <c r="D87" s="16" t="inlineStr">
+        <is>
+          <t>Malignancy, especially lymphoma</t>
+        </is>
+      </c>
+      <c r="E87" s="16" t="inlineStr">
+        <is>
+          <t>≤ 7.5 mg daily long term, taper</t>
+        </is>
+      </c>
+      <c r="F87" s="16" t="inlineStr">
+        <is>
+          <t>7.5 mg weekly → 15–25 mg weekly</t>
+        </is>
+      </c>
+      <c r="G87" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="H87" s="18" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="I87" s="1" t="n"/>
       <c r="J87" s="1" t="n"/>
       <c r="K87" s="1" t="n"/>
@@ -6004,14 +6368,42 @@
       <c r="AA87" s="1" t="n"/>
     </row>
     <row r="88" ht="25.5" customHeight="1">
-      <c r="A88" s="11" t="n"/>
-      <c r="B88" s="16" t="n"/>
-      <c r="C88" s="16" t="n"/>
-      <c r="D88" s="16" t="n"/>
-      <c r="E88" s="16" t="n"/>
-      <c r="F88" s="16" t="n"/>
-      <c r="G88" s="14" t="n"/>
-      <c r="H88" s="18" t="n"/>
+      <c r="A88" s="11" t="n">
+        <v>80</v>
+      </c>
+      <c r="B88" s="16" t="inlineStr">
+        <is>
+          <t>Hydroxychloroquine monitoring: which is right?</t>
+        </is>
+      </c>
+      <c r="C88" s="16" t="inlineStr">
+        <is>
+          <t>Baseline eye exam; annual after 5 years</t>
+        </is>
+      </c>
+      <c r="D88" s="16" t="inlineStr">
+        <is>
+          <t>CBC, liver, kidney labs every 1–3 months</t>
+        </is>
+      </c>
+      <c r="E88" s="16" t="inlineStr">
+        <is>
+          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
+        </is>
+      </c>
+      <c r="F88" s="16" t="inlineStr">
+        <is>
+          <t>Common first-line for mild-moderate pain</t>
+        </is>
+      </c>
+      <c r="G88" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="H88" s="18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="I88" s="1" t="n"/>
       <c r="J88" s="1" t="n"/>
       <c r="K88" s="1" t="n"/>
@@ -6033,14 +6425,42 @@
       <c r="AA88" s="1" t="n"/>
     </row>
     <row r="89" ht="25.5" customHeight="1">
-      <c r="A89" s="11" t="n"/>
-      <c r="B89" s="16" t="n"/>
-      <c r="C89" s="16" t="n"/>
-      <c r="D89" s="16" t="n"/>
-      <c r="E89" s="16" t="n"/>
-      <c r="F89" s="16" t="n"/>
-      <c r="G89" s="14" t="n"/>
-      <c r="H89" s="18" t="n"/>
+      <c r="A89" s="11" t="n">
+        <v>81</v>
+      </c>
+      <c r="B89" s="16" t="inlineStr">
+        <is>
+          <t>TNF inhibitor boxed warning: which is right?</t>
+        </is>
+      </c>
+      <c r="C89" s="16" t="inlineStr">
+        <is>
+          <t>10–20× more selective for COX-2</t>
+        </is>
+      </c>
+      <c r="D89" s="16" t="inlineStr">
+        <is>
+          <t>7.5 mg weekly → 15–25 mg weekly</t>
+        </is>
+      </c>
+      <c r="E89" s="16" t="inlineStr">
+        <is>
+          <t>Malignancy, especially lymphoma</t>
+        </is>
+      </c>
+      <c r="F89" s="16" t="inlineStr">
+        <is>
+          <t>≤ 7.5 mg daily long term, taper</t>
+        </is>
+      </c>
+      <c r="G89" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="H89" s="18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="I89" s="1" t="n"/>
       <c r="J89" s="1" t="n"/>
       <c r="K89" s="1" t="n"/>
@@ -6062,14 +6482,42 @@
       <c r="AA89" s="1" t="n"/>
     </row>
     <row r="90" ht="25.5" customHeight="1">
-      <c r="A90" s="11" t="n"/>
-      <c r="B90" s="16" t="n"/>
-      <c r="C90" s="16" t="n"/>
-      <c r="D90" s="16" t="n"/>
-      <c r="E90" s="16" t="n"/>
-      <c r="F90" s="16" t="n"/>
-      <c r="G90" s="14" t="n"/>
-      <c r="H90" s="18" t="n"/>
+      <c r="A90" s="11" t="n">
+        <v>82</v>
+      </c>
+      <c r="B90" s="16" t="inlineStr">
+        <is>
+          <t>JAK inhibitor boxed warning: which is right?</t>
+        </is>
+      </c>
+      <c r="C90" s="16" t="inlineStr">
+        <is>
+          <t>VTE (DVT/PE), MACE, cancer</t>
+        </is>
+      </c>
+      <c r="D90" s="16" t="inlineStr">
+        <is>
+          <t>Longer half-life, twice-daily</t>
+        </is>
+      </c>
+      <c r="E90" s="16" t="inlineStr">
+        <is>
+          <t>PGI2 falls, TXA2 preserved</t>
+        </is>
+      </c>
+      <c r="F90" s="16" t="inlineStr">
+        <is>
+          <t>DHODH (pyrimidine synthesis)</t>
+        </is>
+      </c>
+      <c r="G90" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="H90" s="18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="I90" s="1" t="n"/>
       <c r="J90" s="1" t="n"/>
       <c r="K90" s="1" t="n"/>
@@ -6091,14 +6539,42 @@
       <c r="AA90" s="1" t="n"/>
     </row>
     <row r="91" ht="25.5" customHeight="1">
-      <c r="A91" s="11" t="n"/>
-      <c r="B91" s="16" t="n"/>
-      <c r="C91" s="16" t="n"/>
-      <c r="D91" s="16" t="n"/>
-      <c r="E91" s="16" t="n"/>
-      <c r="F91" s="16" t="n"/>
-      <c r="G91" s="14" t="n"/>
-      <c r="H91" s="18" t="n"/>
+      <c r="A91" s="11" t="n">
+        <v>83</v>
+      </c>
+      <c r="B91" s="16" t="inlineStr">
+        <is>
+          <t>JAK inhibitors: which is right?</t>
+        </is>
+      </c>
+      <c r="C91" s="16" t="inlineStr">
+        <is>
+          <t>~90% glucuronidation/sulfation (safe) · ~5–10% CYP2E1 → NAPQI</t>
+        </is>
+      </c>
+      <c r="D91" s="16" t="inlineStr">
+        <is>
+          <t>Baricitinib, tofacitinib, upadacitinib — oral; zoster, ↑ LDL</t>
+        </is>
+      </c>
+      <c r="E91" s="16" t="inlineStr">
+        <is>
+          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
+        </is>
+      </c>
+      <c r="F91" s="16" t="inlineStr">
+        <is>
+          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
+        </is>
+      </c>
+      <c r="G91" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="H91" s="18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="I91" s="1" t="n"/>
       <c r="J91" s="1" t="n"/>
       <c r="K91" s="1" t="n"/>
@@ -6120,14 +6596,42 @@
       <c r="AA91" s="1" t="n"/>
     </row>
     <row r="92" ht="25.5" customHeight="1">
-      <c r="A92" s="11" t="n"/>
-      <c r="B92" s="16" t="n"/>
-      <c r="C92" s="16" t="n"/>
-      <c r="D92" s="16" t="n"/>
-      <c r="E92" s="16" t="n"/>
-      <c r="F92" s="16" t="n"/>
-      <c r="G92" s="14" t="n"/>
-      <c r="H92" s="18" t="n"/>
+      <c r="A92" s="11" t="n">
+        <v>84</v>
+      </c>
+      <c r="B92" s="16" t="inlineStr">
+        <is>
+          <t>RA prednisone ceiling: which is right?</t>
+        </is>
+      </c>
+      <c r="C92" s="16" t="inlineStr">
+        <is>
+          <t>7.5 mg weekly → 15–25 mg weekly</t>
+        </is>
+      </c>
+      <c r="D92" s="16" t="inlineStr">
+        <is>
+          <t>≤ 7.5 mg daily long term, taper</t>
+        </is>
+      </c>
+      <c r="E92" s="16" t="inlineStr">
+        <is>
+          <t>Malignancy, especially lymphoma</t>
+        </is>
+      </c>
+      <c r="F92" s="16" t="inlineStr">
+        <is>
+          <t>10–20× more selective for COX-2</t>
+        </is>
+      </c>
+      <c r="G92" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="H92" s="18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="I92" s="1" t="n"/>
       <c r="J92" s="1" t="n"/>
       <c r="K92" s="1" t="n"/>

</xml_diff>

<commit_message>
Add Lecture 4 (Unit 2 Session 2): gout, muscle relaxants, bone
Study guide, deck, 5 interactive figures, 28 lecture questions, 28 new drug cards,
and 20 Session 2 questions in the Unit 2 practice exam (now 50).
</commit_message>
<xml_diff>
--- a/docs/sketch/kahoot/unit2_L03.xlsx
+++ b/docs/sketch/kahoot/unit2_L03.xlsx
@@ -1885,12 +1885,12 @@
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
+          <t>PGI2 falls while platelet TXA2 is preserved</t>
+        </is>
+      </c>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
           <t>It depletes glutathione in the heart</t>
-        </is>
-      </c>
-      <c r="F9" s="14" t="inlineStr">
-        <is>
-          <t>PGI2 falls while platelet TXA2 is preserved</t>
         </is>
       </c>
       <c r="G9" s="14" t="n">
@@ -1898,7 +1898,7 @@
       </c>
       <c r="H9" s="15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I9" s="1" t="n"/>
@@ -1932,22 +1932,22 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
+          <t>Hypersensitivity, lymphoma, heart failure</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="inlineStr">
+        <is>
+          <t>Retinopathy, cardiomyopathy, myopathy</t>
+        </is>
+      </c>
+      <c r="E10" s="14" t="inlineStr">
+        <is>
+          <t>Hepatotoxicity, marrow suppression, pulmonary toxicity</t>
+        </is>
+      </c>
+      <c r="F10" s="14" t="inlineStr">
+        <is>
           <t>Tinnitus, aseptic meningitis, rash</t>
-        </is>
-      </c>
-      <c r="D10" s="14" t="inlineStr">
-        <is>
-          <t>GI bleeding, AKI, cardiovascular events</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="inlineStr">
-        <is>
-          <t>Hepatotoxicity, marrow suppression, pulmonary toxicity</t>
-        </is>
-      </c>
-      <c r="F10" s="14" t="inlineStr">
-        <is>
-          <t>Hypersensitivity, lymphoma, heart failure</t>
         </is>
       </c>
       <c r="G10" s="14" t="n">
@@ -1989,22 +1989,22 @@
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>Prostaglandin loss thins the gastric mucosa</t>
+          <t>Uric acid crystals deposit and trigger a flare</t>
         </is>
       </c>
       <c r="D11" s="21" t="inlineStr">
         <is>
+          <t>Synovitis forms a pannus; TNF-α and IL-6 drive erosion</t>
+        </is>
+      </c>
+      <c r="E11" s="14" t="inlineStr">
+        <is>
+          <t>Mechanical wear degrades cartilage; osteophytes form</t>
+        </is>
+      </c>
+      <c r="F11" s="14" t="inlineStr">
+        <is>
           <t>NAPQI binds proteins in the synovial lining</t>
-        </is>
-      </c>
-      <c r="E11" s="14" t="inlineStr">
-        <is>
-          <t>Uric acid crystals deposit and trigger a flare</t>
-        </is>
-      </c>
-      <c r="F11" s="14" t="inlineStr">
-        <is>
-          <t>Synovitis forms a pannus; TNF-α and IL-6 drive erosion</t>
         </is>
       </c>
       <c r="G11" s="14" t="n">
@@ -2012,7 +2012,7 @@
       </c>
       <c r="H11" s="15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I11" s="1" t="n"/>
@@ -2051,7 +2051,7 @@
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>Celecoxib</t>
+          <t>Rituximab</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr">
@@ -2103,22 +2103,22 @@
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
+          <t>Depleting or modulating B lymphocytes</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
           <t>Blocking IL-6 receptor signaling</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>Blocking T-cell costimulation</t>
-        </is>
-      </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
+          <t>Inhibiting dihydrofolate reductase</t>
+        </is>
+      </c>
+      <c r="F13" s="14" t="inlineStr">
+        <is>
           <t>Blocking TNF-α signaling</t>
-        </is>
-      </c>
-      <c r="F13" s="14" t="inlineStr">
-        <is>
-          <t>Depleting or modulating B lymphocytes</t>
         </is>
       </c>
       <c r="G13" s="14" t="n">
@@ -2126,7 +2126,7 @@
       </c>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I13" s="1" t="n"/>
@@ -2160,22 +2160,22 @@
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
+          <t>Before infliximab is started</t>
+        </is>
+      </c>
+      <c r="D14" s="14" t="inlineStr">
+        <is>
+          <t>One week after the first infusion</t>
+        </is>
+      </c>
+      <c r="E14" s="14" t="inlineStr">
+        <is>
+          <t>Only if a fever develops on therapy</t>
+        </is>
+      </c>
+      <c r="F14" s="14" t="inlineStr">
+        <is>
           <t>Any time, since biologics don't affect immunity</t>
-        </is>
-      </c>
-      <c r="D14" s="14" t="inlineStr">
-        <is>
-          <t>Never — vaccines are banned for life</t>
-        </is>
-      </c>
-      <c r="E14" s="14" t="inlineStr">
-        <is>
-          <t>Before infliximab is started</t>
-        </is>
-      </c>
-      <c r="F14" s="14" t="inlineStr">
-        <is>
-          <t>Only if a fever develops on therapy</t>
         </is>
       </c>
       <c r="G14" s="14" t="n">
@@ -2183,7 +2183,7 @@
       </c>
       <c r="H14" s="15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I14" s="1" t="n"/>
@@ -2217,7 +2217,7 @@
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>Celecoxib</t>
+          <t>Naproxen</t>
         </is>
       </c>
       <c r="D15" s="14" t="inlineStr">
@@ -2274,22 +2274,22 @@
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
+          <t>They deplete B cells that release prostaglandins</t>
+        </is>
+      </c>
+      <c r="D16" s="14" t="inlineStr">
+        <is>
           <t>They block phospholipase A₂, upstream of COX</t>
         </is>
       </c>
-      <c r="D16" s="14" t="inlineStr">
-        <is>
-          <t>They deplete B cells that release prostaglandins</t>
-        </is>
-      </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
+          <t>They act centrally on the hypothalamus</t>
+        </is>
+      </c>
+      <c r="F16" s="14" t="inlineStr">
+        <is>
           <t>They block COX-2 more strongly than any NSAID</t>
-        </is>
-      </c>
-      <c r="F16" s="14" t="inlineStr">
-        <is>
-          <t>They act centrally on the hypothalamus</t>
         </is>
       </c>
       <c r="G16" s="14" t="n">
@@ -2297,7 +2297,7 @@
       </c>
       <c r="H16" s="15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I16" s="1" t="n"/>
@@ -2326,35 +2326,35 @@
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>Which drug pairing does the lecture flag for a higher GI ulcer risk?</t>
+          <t>A 72-year-old with CKD, hypertension, and anticoagulation has an acute gout flare. Which option is often preferred?</t>
         </is>
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>NSAID plus a corticosteroid</t>
+          <t>Full-dose oral naproxen</t>
         </is>
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>Acetaminophen plus N-acetylcysteine</t>
+          <t>Starting allopurinol today</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>NSAID plus an anticoagulant</t>
+          <t>A short corticosteroid course</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>NSAID plus a diuretic</t>
+          <t>Probenecid to clear uric acid</t>
         </is>
       </c>
       <c r="G17" s="14" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="H17" s="15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I17" s="1" t="n"/>
@@ -2383,31 +2383,31 @@
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>Which statement correctly describes COX-1?</t>
+          <t>Which drug pairing does the lecture flag for a higher GI ulcer risk?</t>
         </is>
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>Target of celecoxib's selective inhibition</t>
+          <t>NSAID plus an ACE inhibitor</t>
         </is>
       </c>
       <c r="D18" s="14" t="inlineStr">
         <is>
-          <t>Inducible enzyme found mainly at inflamed sites</t>
+          <t>NSAID plus a diuretic</t>
         </is>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>Housekeeping enzyme protecting stomach and renal flow</t>
+          <t>NSAID plus a corticosteroid</t>
         </is>
       </c>
       <c r="F18" s="14" t="inlineStr">
         <is>
-          <t>Enzyme that converts acetaminophen to NAPQI</t>
+          <t>Acetaminophen plus N-acetylcysteine</t>
         </is>
       </c>
       <c r="G18" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H18" s="15" t="inlineStr">
         <is>
@@ -2440,31 +2440,31 @@
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>Per the textbook, which instruction about ketorolac is correct?</t>
+          <t>Which statement correctly describes COX-1?</t>
         </is>
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>Double the dose in patients over 65</t>
+          <t>Inducible enzyme found mainly at inflamed sites</t>
         </is>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>Maximum daily dose is 240 mg</t>
+          <t>Main source of inflammatory prostaglandins</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>Start therapy with an oral dose</t>
+          <t>Target of celecoxib's selective inhibition</t>
         </is>
       </c>
       <c r="F19" s="14" t="inlineStr">
         <is>
-          <t>Use no longer than 5 days</t>
+          <t>Housekeeping enzyme protecting stomach and renal flow</t>
         </is>
       </c>
       <c r="G19" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H19" s="15" t="inlineStr">
         <is>
@@ -2497,27 +2497,27 @@
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>Which effect is acetaminophen least reliable for?</t>
+          <t>Per the textbook, which instruction about ketorolac is correct?</t>
         </is>
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>Pain in a patient with CKD</t>
+          <t>Maximum daily dose is 240 mg</t>
         </is>
       </c>
       <c r="D20" s="14" t="inlineStr">
         <is>
-          <t>Lowering fever</t>
+          <t>Safe long-term in renal impairment</t>
         </is>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>Reducing peripheral inflammation</t>
+          <t>Start therapy with an oral dose</t>
         </is>
       </c>
       <c r="F20" s="14" t="inlineStr">
         <is>
-          <t>First-line mild osteoarthritis pain</t>
+          <t>Use no longer than 5 days</t>
         </is>
       </c>
       <c r="G20" s="14" t="n">
@@ -2525,7 +2525,7 @@
       </c>
       <c r="H20" s="15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I20" s="1" t="n"/>
@@ -2554,35 +2554,35 @@
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>What defines a drug as “disease-modifying” in rheumatoid arthritis?</t>
+          <t>Which effect is acetaminophen least reliable for?</t>
         </is>
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>It lowers fever through the hypothalamus</t>
+          <t>Pain in a patient with CKD</t>
         </is>
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>It selectively blocks the COX-2 isoform</t>
+          <t>Reducing peripheral inflammation</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>It relieves pain faster than NSAIDs</t>
+          <t>Relieving mild-to-moderate pain</t>
         </is>
       </c>
       <c r="F21" s="14" t="inlineStr">
         <is>
-          <t>It slows or halts joint destruction</t>
+          <t>Lowering fever</t>
         </is>
       </c>
       <c r="G21" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H21" s="15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I21" s="1" t="n"/>
@@ -2611,27 +2611,27 @@
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>Which non-drug approaches does the lecture include in osteoarthritis management?</t>
+          <t>What defines a drug as “disease-modifying” in rheumatoid arthritis?</t>
         </is>
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>Fasting, high-protein diet, bed rest</t>
+          <t>It lowers fever through the hypothalamus</t>
         </is>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>Glutathione replenishment, label review</t>
+          <t>It relieves pain faster than NSAIDs</t>
         </is>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>Activity modification, physical therapy, weight management</t>
+          <t>It slows or halts joint destruction</t>
         </is>
       </c>
       <c r="F22" s="14" t="inlineStr">
         <is>
-          <t>Live vaccines, TB screening, folate</t>
+          <t>It selectively blocks the COX-2 isoform</t>
         </is>
       </c>
       <c r="G22" s="14" t="n">
@@ -2668,31 +2668,31 @@
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>A prescription reads infliximab. What does the stem “-ximab” tell you?</t>
+          <t>Which non-drug approaches does the lecture include in osteoarthritis management?</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>A kinase inhibitor</t>
+          <t>Glutathione replenishment, label review</t>
         </is>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
-          <t>A chimeric monoclonal antibody</t>
+          <t>Activity modification, physical therapy, weight management</t>
         </is>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>A humanized monoclonal antibody</t>
+          <t>Live vaccines, TB screening, folate</t>
         </is>
       </c>
       <c r="F23" s="14" t="inlineStr">
         <is>
-          <t>A fully human monoclonal antibody</t>
+          <t>Nerve ablation, spinal cord stimulation</t>
         </is>
       </c>
       <c r="G23" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H23" s="15" t="inlineStr">
         <is>
@@ -2725,31 +2725,31 @@
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>A pharmacist calls: a new prescription reads “methotrexate 15 mg by mouth daily” for RA. What is the safety problem?</t>
+          <t>A prescription reads infliximab. What does the stem “-ximab” tell you?</t>
         </is>
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>Nothing — daily dosing is standard for RA</t>
+          <t>A receptor fusion protein</t>
         </is>
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
-          <t>It should be twice daily for steady levels</t>
+          <t>A fully human monoclonal antibody</t>
         </is>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>It should be weekly; daily dosing can be fatal</t>
+          <t>A chimeric monoclonal antibody</t>
         </is>
       </c>
       <c r="F24" s="14" t="inlineStr">
         <is>
-          <t>It should be IV only in RA</t>
+          <t>A kinase inhibitor</t>
         </is>
       </c>
       <c r="G24" s="14" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="H24" s="15" t="inlineStr">
         <is>
@@ -2782,35 +2782,35 @@
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>Which sequence describes how tissue injury produces musculoskeletal pain?</t>
+          <t>A pharmacist calls: a new prescription reads “methotrexate 15 mg by mouth daily” for RA. What is the safety problem?</t>
         </is>
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
-          <t>Injury → nerve transection → cortical atrophy → pain</t>
+          <t>It should be IV only in RA</t>
         </is>
       </c>
       <c r="D25" s="14" t="inlineStr">
         <is>
-          <t>Injury → T-cell depletion → B-cell surge → pain</t>
+          <t>It needs N-acetylcysteine with each dose</t>
         </is>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>Injury → glutathione loss → NAPQI build-up → pain</t>
+          <t>It should be weekly; daily dosing can be fatal</t>
         </is>
       </c>
       <c r="F25" s="14" t="inlineStr">
         <is>
-          <t>Injury → mediator release → nociceptor sensitization → pain</t>
+          <t>It should be twice daily for steady levels</t>
         </is>
       </c>
       <c r="G25" s="14" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="H25" s="15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I25" s="1" t="n"/>
@@ -2839,35 +2839,35 @@
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>Which drug is a TNF inhibitor?</t>
+          <t>Which sequence describes how tissue injury produces musculoskeletal pain?</t>
         </is>
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>Rituximab</t>
+          <t>Injury → COX-1 induction → gastric protection → pain</t>
         </is>
       </c>
       <c r="D26" s="14" t="inlineStr">
         <is>
-          <t>Abatacept</t>
+          <t>Injury → nerve transection → cortical atrophy → pain</t>
         </is>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>Etanercept</t>
+          <t>Injury → T-cell depletion → B-cell surge → pain</t>
         </is>
       </c>
       <c r="F26" s="14" t="inlineStr">
         <is>
-          <t>Tocilizumab</t>
+          <t>Injury → mediator release → nociceptor sensitization → pain</t>
         </is>
       </c>
       <c r="G26" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H26" s="15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I26" s="1" t="n"/>
@@ -2896,31 +2896,31 @@
       </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>Which mediator is the primary target of NSAID therapy within the inflammatory pain pathway?</t>
+          <t>Which drug is a TNF inhibitor?</t>
         </is>
       </c>
       <c r="C27" s="14" t="inlineStr">
         <is>
-          <t>Bradykinin</t>
+          <t>Rituximab</t>
         </is>
       </c>
       <c r="D27" s="14" t="inlineStr">
         <is>
-          <t>Histamine</t>
+          <t>Abatacept</t>
         </is>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
-          <t>Cytokines broadly (e.g., all of TNF-α, IL-1, IL-6)</t>
+          <t>Tocilizumab</t>
         </is>
       </c>
       <c r="F27" s="14" t="inlineStr">
         <is>
-          <t>Prostaglandins</t>
+          <t>Etanercept</t>
         </is>
       </c>
       <c r="G27" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H27" s="15" t="inlineStr">
         <is>
@@ -2953,27 +2953,27 @@
       </c>
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>In acetaminophen overdose, hepatotoxicity results primarily from which mechanism?</t>
+          <t>Which mediator is the primary target of NSAID therapy within the inflammatory pain pathway?</t>
         </is>
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
-          <t>Excess Phase II glucuronidation</t>
+          <t>Bradykinin</t>
         </is>
       </c>
       <c r="D28" s="14" t="inlineStr">
         <is>
-          <t>Accumulation of NAPQI after glutathione stores are depleted</t>
+          <t>Histamine</t>
         </is>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>Direct COX inhibition in the liver</t>
+          <t>Cytokines broadly (e.g., all of TNF-α, IL-1, IL-6)</t>
         </is>
       </c>
       <c r="F28" s="14" t="inlineStr">
         <is>
-          <t>Renal crystal formation</t>
+          <t>Prostaglandins</t>
         </is>
       </c>
       <c r="G28" s="14" t="n">
@@ -2981,7 +2981,7 @@
       </c>
       <c r="H28" s="15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I28" s="1" t="n"/>
@@ -3010,27 +3010,27 @@
       </c>
       <c r="B29" s="16" t="inlineStr">
         <is>
-          <t>In acetaminophen overdose, why is N-acetylcysteine effective?</t>
+          <t>In acetaminophen overdose, hepatotoxicity results primarily from which mechanism?</t>
         </is>
       </c>
       <c r="C29" s="16" t="inlineStr">
         <is>
-          <t>It blocks COX in the liver and lowers prostaglandin levels</t>
+          <t>Excess Phase II glucuronidation</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
         <is>
-          <t>It is a glutathione precursor that restores NAPQI detoxification</t>
+          <t>Accumulation of NAPQI after glutathione stores are depleted</t>
         </is>
       </c>
       <c r="E29" s="16" t="inlineStr">
         <is>
-          <t>It inhibits the enzyme that forms NAPQI from the drug</t>
+          <t>Direct COX inhibition in the liver</t>
         </is>
       </c>
       <c r="F29" s="16" t="inlineStr">
         <is>
-          <t>It binds acetaminophen in the gut and prevents absorption</t>
+          <t>Renal crystal formation</t>
         </is>
       </c>
       <c r="G29" s="14" t="n">
@@ -3067,27 +3067,27 @@
       </c>
       <c r="B30" s="16" t="inlineStr">
         <is>
-          <t>Which statement best explains why nonselective NSAIDs cause GI and renal adverse effects?</t>
+          <t>In acetaminophen overdose, why is N-acetylcysteine effective?</t>
         </is>
       </c>
       <c r="C30" s="16" t="inlineStr">
         <is>
-          <t>They deplete glutathione, which injures the gut and kidney</t>
+          <t>It blocks COX in the liver and lowers prostaglandin levels</t>
         </is>
       </c>
       <c r="D30" s="16" t="inlineStr">
         <is>
-          <t>They block TNF-α, which normally protects the stomach lining</t>
+          <t>It is a glutathione precursor that restores NAPQI detoxification</t>
         </is>
       </c>
       <c r="E30" s="16" t="inlineStr">
         <is>
-          <t>They inhibit COX-1, which protects gastric mucosa and renal blood flow</t>
+          <t>It inhibits the enzyme that forms NAPQI from the drug</t>
         </is>
       </c>
       <c r="F30" s="16" t="inlineStr">
         <is>
-          <t>They block phospholipase A₂ and stop all mediator release</t>
+          <t>It binds acetaminophen in the gut and prevents absorption</t>
         </is>
       </c>
       <c r="G30" s="14" t="n">
@@ -3095,7 +3095,7 @@
       </c>
       <c r="H30" s="17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I30" s="1" t="n"/>
@@ -3124,27 +3124,27 @@
       </c>
       <c r="B31" s="16" t="inlineStr">
         <is>
-          <t>Which nonselective NSAID does the lecture restrict to short-term use because of significant GI and renal risk?</t>
+          <t>Which statement best explains why nonselective NSAIDs cause GI and renal adverse effects?</t>
         </is>
       </c>
       <c r="C31" s="16" t="inlineStr">
         <is>
-          <t>Celecoxib</t>
+          <t>They deplete glutathione, which injures the gut and kidney</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
         <is>
-          <t>Ketorolac</t>
+          <t>They block TNF-α, which normally protects the stomach lining</t>
         </is>
       </c>
       <c r="E31" s="16" t="inlineStr">
         <is>
-          <t>Naproxen</t>
+          <t>They inhibit COX-1, which protects gastric mucosa and renal blood flow</t>
         </is>
       </c>
       <c r="F31" s="16" t="inlineStr">
         <is>
-          <t>Diclofenac</t>
+          <t>They block phospholipase A₂ and stop all mediator release</t>
         </is>
       </c>
       <c r="G31" s="14" t="n">
@@ -3152,7 +3152,7 @@
       </c>
       <c r="H31" s="17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I31" s="1" t="n"/>
@@ -3181,27 +3181,27 @@
       </c>
       <c r="B32" s="16" t="inlineStr">
         <is>
-          <t>What is the key difference in treatment goals between osteoarthritis and rheumatoid arthritis?</t>
+          <t>Which nonselective NSAID does the lecture restrict to short-term use because of significant GI and renal risk?</t>
         </is>
       </c>
       <c r="C32" s="16" t="inlineStr">
         <is>
-          <t>OA aims at pain and function; RA aims to suppress disease activity</t>
+          <t>Celecoxib</t>
         </is>
       </c>
       <c r="D32" s="16" t="inlineStr">
         <is>
-          <t>OA aims at cartilage regrowth with DMARDs</t>
+          <t>Ketorolac</t>
         </is>
       </c>
       <c r="E32" s="16" t="inlineStr">
         <is>
-          <t>OA aims to suppress immunity; RA aims at pain relief only</t>
+          <t>Naproxen</t>
         </is>
       </c>
       <c r="F32" s="16" t="inlineStr">
         <is>
-          <t>RA aims at weight loss; OA aims at infection control</t>
+          <t>Diclofenac</t>
         </is>
       </c>
       <c r="G32" s="14" t="n">
@@ -3209,7 +3209,7 @@
       </c>
       <c r="H32" s="17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I32" s="1" t="n"/>
@@ -3238,27 +3238,27 @@
       </c>
       <c r="B33" s="16" t="inlineStr">
         <is>
-          <t>What is methotrexate’s mechanism as taught in the lecture, and what is co-prescribed to reduce its toxicity?</t>
+          <t>What is the key difference in treatment goals between osteoarthritis and rheumatoid arthritis?</t>
         </is>
       </c>
       <c r="C33" s="16" t="inlineStr">
         <is>
-          <t>COX-2 inhibition; a proton pump inhibitor</t>
+          <t>OA aims at pain and function; RA aims to suppress disease activity</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
         <is>
-          <t>Phospholipase A₂ blockade; calcium supplementation</t>
+          <t>OA aims at cartilage regrowth with DMARDs</t>
         </is>
       </c>
       <c r="E33" s="16" t="inlineStr">
         <is>
-          <t>TNF-α blockade; tuberculosis screening</t>
+          <t>OA aims to suppress immunity; RA aims at pain relief only</t>
         </is>
       </c>
       <c r="F33" s="16" t="inlineStr">
         <is>
-          <t>Dihydrofolate reductase inhibition; folate supplementation</t>
+          <t>RA aims at weight loss; OA aims at infection control</t>
         </is>
       </c>
       <c r="G33" s="14" t="n">
@@ -3266,7 +3266,7 @@
       </c>
       <c r="H33" s="17" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I33" s="1" t="n"/>
@@ -3295,31 +3295,31 @@
       </c>
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>A 29-year-old with active RA who is planning a pregnancy needs a DMARD. Which drug from the lecture is contraindicated?</t>
+          <t>What is methotrexate’s mechanism as taught in the lecture, and what is co-prescribed to reduce its toxicity?</t>
         </is>
       </c>
       <c r="C34" s="16" t="inlineStr">
         <is>
-          <t>Celecoxib, because it is a disease-modifying drug</t>
+          <t>COX-2 inhibition; a proton pump inhibitor</t>
         </is>
       </c>
       <c r="D34" s="16" t="inlineStr">
         <is>
-          <t>Acetaminophen, because it is a DMARD</t>
+          <t>Phospholipase A₂ blockade; calcium supplementation</t>
         </is>
       </c>
       <c r="E34" s="16" t="inlineStr">
         <is>
-          <t>Hydroxychloroquine, because of its poor safety profile</t>
+          <t>TNF-α blockade; tuberculosis screening</t>
         </is>
       </c>
       <c r="F34" s="16" t="inlineStr">
         <is>
-          <t>Methotrexate, because it is teratogenic</t>
+          <t>Dihydrofolate reductase inhibition; folate supplementation</t>
         </is>
       </c>
       <c r="G34" s="14" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="H34" s="17" t="inlineStr">
         <is>
@@ -3352,35 +3352,35 @@
       </c>
       <c r="B35" s="16" t="inlineStr">
         <is>
-          <t>Before starting adalimumab for rheumatoid arthritis, which baseline step does the lecture specifically call for?</t>
+          <t>A 29-year-old with active RA who is planning a pregnancy needs a DMARD. Which drug from the lecture is contraindicated?</t>
         </is>
       </c>
       <c r="C35" s="16" t="inlineStr">
         <is>
-          <t>Checking for all hidden acetaminophen sources</t>
+          <t>Celecoxib, because it is a disease-modifying drug</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>Starting folate to prevent bone marrow toxicity</t>
+          <t>Acetaminophen, because it is a DMARD</t>
         </is>
       </c>
       <c r="E35" s="16" t="inlineStr">
         <is>
-          <t>Screening for tuberculosis and hepatitis B/C</t>
+          <t>Hydroxychloroquine, because of its poor safety profile</t>
         </is>
       </c>
       <c r="F35" s="16" t="inlineStr">
         <is>
-          <t>Adding an ACE inhibitor to protect the kidney</t>
+          <t>Methotrexate, because it is teratogenic</t>
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="H35" s="17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I35" s="1" t="n"/>
@@ -3409,35 +3409,35 @@
       </c>
       <c r="B36" s="16" t="inlineStr">
         <is>
-          <t>Match the drug to its target: which pairing is correct?</t>
+          <t>Before starting adalimumab for rheumatoid arthritis, which baseline step does the lecture specifically call for?</t>
         </is>
       </c>
       <c r="C36" s="16" t="inlineStr">
         <is>
-          <t>Abatacept — B-lymphocyte depletion</t>
+          <t>Checking for all hidden acetaminophen sources</t>
         </is>
       </c>
       <c r="D36" s="16" t="inlineStr">
         <is>
-          <t>Tocilizumab — IL-6 receptor signaling</t>
+          <t>Starting folate to prevent bone marrow toxicity</t>
         </is>
       </c>
       <c r="E36" s="16" t="inlineStr">
         <is>
-          <t>Etanercept — IL-6 receptor signaling</t>
+          <t>Screening for tuberculosis and hepatitis B/C</t>
         </is>
       </c>
       <c r="F36" s="16" t="inlineStr">
         <is>
-          <t>Rituximab — TNF-α signaling</t>
+          <t>Adding an ACE inhibitor to protect the kidney</t>
         </is>
       </c>
       <c r="G36" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H36" s="17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I36" s="1" t="n"/>
@@ -3466,35 +3466,35 @@
       </c>
       <c r="B37" s="16" t="inlineStr">
         <is>
-          <t>Which conventional DMARD requires a baseline eye exam and annual screening after 5 years because of retinopathy?</t>
+          <t>Match the drug to its target: which pairing is correct?</t>
         </is>
       </c>
       <c r="C37" s="16" t="inlineStr">
         <is>
-          <t>Methotrexate</t>
+          <t>Abatacept — B-lymphocyte depletion</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>Mycophenolate mofetil</t>
+          <t>Tocilizumab — IL-6 receptor signaling</t>
         </is>
       </c>
       <c r="E37" s="16" t="inlineStr">
         <is>
-          <t>Leflunomide</t>
+          <t>Etanercept — IL-6 receptor signaling</t>
         </is>
       </c>
       <c r="F37" s="16" t="inlineStr">
         <is>
-          <t>Hydroxychloroquine</t>
+          <t>Rituximab — TNF-α signaling</t>
         </is>
       </c>
       <c r="G37" s="14" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="H37" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I37" s="1" t="n"/>
@@ -3523,31 +3523,31 @@
       </c>
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t>Pain by mechanism: which is right?</t>
+          <t>Which conventional DMARD requires a baseline eye exam and annual screening after 5 years because of retinopathy?</t>
         </is>
       </c>
       <c r="C38" s="16" t="inlineStr">
         <is>
-          <t>CBC, liver, kidney labs every 1–3 months</t>
+          <t>Methotrexate</t>
         </is>
       </c>
       <c r="D38" s="16" t="inlineStr">
         <is>
-          <t>N-acetylcysteine — glutathione precursor</t>
+          <t>Mycophenolate mofetil</t>
         </is>
       </c>
       <c r="E38" s="16" t="inlineStr">
         <is>
-          <t>Common first-line for mild-moderate pain</t>
+          <t>Leflunomide</t>
         </is>
       </c>
       <c r="F38" s="16" t="inlineStr">
         <is>
-          <t>Nociceptive · inflammatory · neuropathic</t>
+          <t>Hydroxychloroquine</t>
         </is>
       </c>
       <c r="G38" s="14" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="H38" s="18" t="inlineStr">
         <is>
@@ -3580,27 +3580,27 @@
       </c>
       <c r="B39" s="16" t="inlineStr">
         <is>
-          <t>Chronic pain: which is right?</t>
+          <t>Pain by mechanism: which is right?</t>
         </is>
       </c>
       <c r="C39" s="16" t="inlineStr">
         <is>
-          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
+          <t>CBC, liver, kidney labs every 1–3 months</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
         <is>
-          <t>Persists beyond expected healing, often &gt; 3 months</t>
+          <t>N-acetylcysteine — glutathione precursor</t>
         </is>
       </c>
       <c r="E39" s="16" t="inlineStr">
         <is>
-          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
+          <t>Common first-line for mild-moderate pain</t>
         </is>
       </c>
       <c r="F39" s="16" t="inlineStr">
         <is>
-          <t>Housekeeping: gastric protection, renal blood flow</t>
+          <t>Nociceptive · inflammatory · neuropathic</t>
         </is>
       </c>
       <c r="G39" s="14" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="H39" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I39" s="1" t="n"/>
@@ -3637,27 +3637,27 @@
       </c>
       <c r="B40" s="16" t="inlineStr">
         <is>
-          <t>4 pain mediators: which is right?</t>
+          <t>Chronic pain: which is right?</t>
         </is>
       </c>
       <c r="C40" s="16" t="inlineStr">
         <is>
-          <t>Prostaglandins, bradykinin, histamine, cytokines (TNF-α, IL-1, IL-6)</t>
+          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
         </is>
       </c>
       <c r="D40" s="16" t="inlineStr">
         <is>
-          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
+          <t>Persists beyond expected healing, often &gt; 3 months</t>
         </is>
       </c>
       <c r="E40" s="16" t="inlineStr">
         <is>
-          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
+          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
         </is>
       </c>
       <c r="F40" s="16" t="inlineStr">
         <is>
-          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
+          <t>Housekeeping: gastric protection, renal blood flow</t>
         </is>
       </c>
       <c r="G40" s="14" t="n">
@@ -3665,7 +3665,7 @@
       </c>
       <c r="H40" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I40" s="1" t="n"/>
@@ -3694,27 +3694,27 @@
       </c>
       <c r="B41" s="16" t="inlineStr">
         <is>
-          <t>Corticosteroid site: which is right?</t>
+          <t>4 pain mediators: which is right?</t>
         </is>
       </c>
       <c r="C41" s="16" t="inlineStr">
         <is>
-          <t>TB + hepatitis B/C screen; update vaccines (live) first</t>
+          <t>Prostaglandins, bradykinin, histamine, cytokines (TNF-α, IL-1, IL-6)</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
+          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
         </is>
       </c>
       <c r="E41" s="16" t="inlineStr">
         <is>
-          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
+          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
         </is>
       </c>
       <c r="F41" s="16" t="inlineStr">
         <is>
-          <t>Anti-CD20; after TNF-inhibitor failure; check hepatitis B</t>
+          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
         </is>
       </c>
       <c r="G41" s="14" t="n">
@@ -3722,7 +3722,7 @@
       </c>
       <c r="H41" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I41" s="1" t="n"/>
@@ -3751,35 +3751,35 @@
       </c>
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>NSAID site: which is right?</t>
+          <t>Corticosteroid site: which is right?</t>
         </is>
       </c>
       <c r="C42" s="16" t="inlineStr">
         <is>
-          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
+          <t>TB + hepatitis B/C screen; update vaccines (live) first</t>
         </is>
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>COX → prostaglandins specifically</t>
+          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
         </is>
       </c>
       <c r="E42" s="16" t="inlineStr">
         <is>
-          <t>More potent; more GI/CNS effects</t>
+          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
         </is>
       </c>
       <c r="F42" s="16" t="inlineStr">
         <is>
-          <t>Alters lysosomal and TLR signaling</t>
+          <t>Anti-CD20; after TNF-inhibitor failure; check hepatitis B</t>
         </is>
       </c>
       <c r="G42" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H42" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I42" s="1" t="n"/>
@@ -3808,31 +3808,31 @@
       </c>
       <c r="B43" s="16" t="inlineStr">
         <is>
-          <t>Acetaminophen effects: which is right?</t>
+          <t>NSAID site: which is right?</t>
         </is>
       </c>
       <c r="C43" s="16" t="inlineStr">
         <is>
-          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
+          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
+          <t>COX → prostaglandins specifically</t>
         </is>
       </c>
       <c r="E43" s="16" t="inlineStr">
         <is>
-          <t>Persists beyond expected healing, often &gt; 3 months</t>
+          <t>More potent; more GI/CNS effects</t>
         </is>
       </c>
       <c r="F43" s="16" t="inlineStr">
         <is>
-          <t>Housekeeping: gastric protection, renal blood flow</t>
+          <t>Alters lysosomal and TLR signaling</t>
         </is>
       </c>
       <c r="G43" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H43" s="18" t="inlineStr">
         <is>
@@ -3865,31 +3865,31 @@
       </c>
       <c r="B44" s="16" t="inlineStr">
         <is>
-          <t>Acetaminophen toxic metabolite: which is right?</t>
+          <t>Acetaminophen effects: which is right?</t>
         </is>
       </c>
       <c r="C44" s="16" t="inlineStr">
         <is>
-          <t>Alters RA’s course, not just symptoms</t>
+          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
         </is>
       </c>
       <c r="D44" s="16" t="inlineStr">
         <is>
-          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
+          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
         </is>
       </c>
       <c r="E44" s="16" t="inlineStr">
         <is>
-          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
+          <t>Persists beyond expected healing, often &gt; 3 months</t>
         </is>
       </c>
       <c r="F44" s="16" t="inlineStr">
         <is>
-          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
+          <t>Housekeeping: gastric protection, renal blood flow</t>
         </is>
       </c>
       <c r="G44" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H44" s="18" t="inlineStr">
         <is>
@@ -3922,35 +3922,35 @@
       </c>
       <c r="B45" s="16" t="inlineStr">
         <is>
-          <t>Acetaminophen antidote: which is right?</t>
+          <t>Acetaminophen toxic metabolite: which is right?</t>
         </is>
       </c>
       <c r="C45" s="16" t="inlineStr">
         <is>
-          <t>Common first-line for mild-moderate pain</t>
+          <t>Alters RA’s course, not just symptoms</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
-          <t>CBC, liver, kidney labs every 1–3 months</t>
+          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
         </is>
       </c>
       <c r="E45" s="16" t="inlineStr">
         <is>
-          <t>Nociceptive · inflammatory · neuropathic</t>
+          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
         </is>
       </c>
       <c r="F45" s="16" t="inlineStr">
         <is>
-          <t>N-acetylcysteine — glutathione precursor</t>
+          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
         </is>
       </c>
       <c r="G45" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H45" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I45" s="1" t="n"/>
@@ -3979,27 +3979,27 @@
       </c>
       <c r="B46" s="16" t="inlineStr">
         <is>
-          <t>Hidden acetaminophen: which is right?</t>
+          <t>Acetaminophen antidote: which is right?</t>
         </is>
       </c>
       <c r="C46" s="16" t="inlineStr">
         <is>
-          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
+          <t>Common first-line for mild-moderate pain</t>
         </is>
       </c>
       <c r="D46" s="16" t="inlineStr">
         <is>
-          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
+          <t>CBC, liver, kidney labs every 1–3 months</t>
         </is>
       </c>
       <c r="E46" s="16" t="inlineStr">
         <is>
-          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
+          <t>Nociceptive · inflammatory · neuropathic</t>
         </is>
       </c>
       <c r="F46" s="16" t="inlineStr">
         <is>
-          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
+          <t>N-acetylcysteine — glutathione precursor</t>
         </is>
       </c>
       <c r="G46" s="14" t="n">
@@ -4007,7 +4007,7 @@
       </c>
       <c r="H46" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I46" s="1" t="n"/>
@@ -4036,27 +4036,27 @@
       </c>
       <c r="B47" s="16" t="inlineStr">
         <is>
-          <t>COX-1: which is right?</t>
+          <t>Hidden acetaminophen: which is right?</t>
         </is>
       </c>
       <c r="C47" s="16" t="inlineStr">
         <is>
-          <t>Persists beyond expected healing, often &gt; 3 months</t>
+          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>Housekeeping: gastric protection, renal blood flow</t>
+          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
         </is>
       </c>
       <c r="E47" s="16" t="inlineStr">
         <is>
-          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
+          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
         </is>
       </c>
       <c r="F47" s="16" t="inlineStr">
         <is>
-          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
+          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
         </is>
       </c>
       <c r="G47" s="14" t="n">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="H47" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I47" s="1" t="n"/>
@@ -4093,27 +4093,27 @@
       </c>
       <c r="B48" s="16" t="inlineStr">
         <is>
-          <t>COX-2: which is right?</t>
+          <t>COX-1: which is right?</t>
         </is>
       </c>
       <c r="C48" s="16" t="inlineStr">
         <is>
-          <t>~90% glucuronidation/sulfation (safe) · ~5–10% CYP2E1 → NAPQI</t>
+          <t>Persists beyond expected healing, often &gt; 3 months</t>
         </is>
       </c>
       <c r="D48" s="16" t="inlineStr">
         <is>
-          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
+          <t>Housekeeping: gastric protection, renal blood flow</t>
         </is>
       </c>
       <c r="E48" s="16" t="inlineStr">
         <is>
-          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
+          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
         </is>
       </c>
       <c r="F48" s="16" t="inlineStr">
         <is>
-          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
+          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
         </is>
       </c>
       <c r="G48" s="14" t="n">
@@ -4150,27 +4150,27 @@
       </c>
       <c r="B49" s="16" t="inlineStr">
         <is>
-          <t>Ibuprofen: which is right?</t>
+          <t>COX-2: which is right?</t>
         </is>
       </c>
       <c r="C49" s="16" t="inlineStr">
         <is>
-          <t>Nociceptive · inflammatory · neuropathic</t>
+          <t>~90% glucuronidation/sulfation (safe) · ~5–10% CYP2E1 → NAPQI</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
         <is>
-          <t>N-acetylcysteine — glutathione precursor</t>
+          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
         </is>
       </c>
       <c r="E49" s="16" t="inlineStr">
         <is>
-          <t>Common first-line for mild-moderate pain</t>
+          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
         </is>
       </c>
       <c r="F49" s="16" t="inlineStr">
         <is>
-          <t>CBC, liver, kidney labs every 1–3 months</t>
+          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
         </is>
       </c>
       <c r="G49" s="14" t="n">
@@ -4178,7 +4178,7 @@
       </c>
       <c r="H49" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I49" s="1" t="n"/>
@@ -4207,35 +4207,35 @@
       </c>
       <c r="B50" s="16" t="inlineStr">
         <is>
-          <t>Naproxen: which is right?</t>
+          <t>Ibuprofen: which is right?</t>
         </is>
       </c>
       <c r="C50" s="16" t="inlineStr">
         <is>
-          <t>≤ 7.5 mg daily long term, taper</t>
+          <t>Nociceptive · inflammatory · neuropathic</t>
         </is>
       </c>
       <c r="D50" s="16" t="inlineStr">
         <is>
-          <t>Immunosuppression → infection</t>
+          <t>N-acetylcysteine — glutathione precursor</t>
         </is>
       </c>
       <c r="E50" s="16" t="inlineStr">
         <is>
-          <t>DHODH (pyrimidine synthesis)</t>
+          <t>Common first-line for mild-moderate pain</t>
         </is>
       </c>
       <c r="F50" s="16" t="inlineStr">
         <is>
-          <t>Longer half-life, twice-daily</t>
+          <t>CBC, liver, kidney labs every 1–3 months</t>
         </is>
       </c>
       <c r="G50" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H50" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I50" s="1" t="n"/>
@@ -4264,27 +4264,27 @@
       </c>
       <c r="B51" s="16" t="inlineStr">
         <is>
-          <t>Diclofenac: which is right?</t>
+          <t>Naproxen: which is right?</t>
         </is>
       </c>
       <c r="C51" s="16" t="inlineStr">
         <is>
-          <t>Centrilobular necrosis</t>
+          <t>≤ 7.5 mg daily long term, taper</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>Tocilizumab</t>
+          <t>Immunosuppression → infection</t>
         </is>
       </c>
       <c r="E51" s="16" t="inlineStr">
         <is>
-          <t>↑ GI ulcer risk</t>
+          <t>DHODH (pyrimidine synthesis)</t>
         </is>
       </c>
       <c r="F51" s="16" t="inlineStr">
         <is>
-          <t>Oral and topical</t>
+          <t>Longer half-life, twice-daily</t>
         </is>
       </c>
       <c r="G51" s="14" t="n">
@@ -4321,27 +4321,27 @@
       </c>
       <c r="B52" s="16" t="inlineStr">
         <is>
-          <t>Indomethacin: which is right?</t>
+          <t>Diclofenac: which is right?</t>
         </is>
       </c>
       <c r="C52" s="16" t="inlineStr">
         <is>
-          <t>More potent; more GI/CNS effects</t>
+          <t>Centrilobular necrosis</t>
         </is>
       </c>
       <c r="D52" s="16" t="inlineStr">
         <is>
-          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
+          <t>Tocilizumab</t>
         </is>
       </c>
       <c r="E52" s="16" t="inlineStr">
         <is>
-          <t>10–20× more selective for COX-2</t>
+          <t>↑ GI ulcer risk</t>
         </is>
       </c>
       <c r="F52" s="16" t="inlineStr">
         <is>
-          <t>COX → prostaglandins specifically</t>
+          <t>Oral and topical</t>
         </is>
       </c>
       <c r="G52" s="14" t="n">
@@ -4349,7 +4349,7 @@
       </c>
       <c r="H52" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I52" s="1" t="n"/>
@@ -4378,35 +4378,35 @@
       </c>
       <c r="B53" s="16" t="inlineStr">
         <is>
-          <t>Ketorolac: which is right?</t>
+          <t>Indomethacin: which is right?</t>
         </is>
       </c>
       <c r="C53" s="16" t="inlineStr">
         <is>
-          <t>Nociceptive · inflammatory · neuropathic</t>
+          <t>More potent; more GI/CNS effects</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>CBC, liver, kidney labs every 1–3 months</t>
+          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
         </is>
       </c>
       <c r="E53" s="16" t="inlineStr">
         <is>
-          <t>8 h, 120 mcg/mL → above the line → start NAC</t>
+          <t>10–20× more selective for COX-2</t>
         </is>
       </c>
       <c r="F53" s="16" t="inlineStr">
         <is>
-          <t>Short-term only; significant GI/renal risk</t>
+          <t>COX → prostaglandins specifically</t>
         </is>
       </c>
       <c r="G53" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H53" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I53" s="1" t="n"/>
@@ -4435,35 +4435,35 @@
       </c>
       <c r="B54" s="16" t="inlineStr">
         <is>
-          <t>Celecoxib trade-off: which is right?</t>
+          <t>Ketorolac: which is right?</t>
         </is>
       </c>
       <c r="C54" s="16" t="inlineStr">
         <is>
-          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
+          <t>Nociceptive · inflammatory · neuropathic</t>
         </is>
       </c>
       <c r="D54" s="16" t="inlineStr">
         <is>
-          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
+          <t>CBC, liver, kidney labs every 1–3 months</t>
         </is>
       </c>
       <c r="E54" s="16" t="inlineStr">
         <is>
-          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
+          <t>8 h, 120 mcg/mL → above the line → start NAC</t>
         </is>
       </c>
       <c r="F54" s="16" t="inlineStr">
         <is>
-          <t>Alters RA’s course, not just symptoms</t>
+          <t>Short-term only; significant GI/renal risk</t>
         </is>
       </c>
       <c r="G54" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H54" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I54" s="1" t="n"/>
@@ -4492,35 +4492,35 @@
       </c>
       <c r="B55" s="16" t="inlineStr">
         <is>
-          <t>NSAID adverse effects: which is right?</t>
+          <t>Celecoxib trade-off: which is right?</t>
         </is>
       </c>
       <c r="C55" s="16" t="inlineStr">
         <is>
-          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
+          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>Anti-CD20; after TNF-inhibitor failure; check hepatitis B</t>
+          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
         </is>
       </c>
       <c r="E55" s="16" t="inlineStr">
         <is>
-          <t>NSAID relief in days · DMARD protection over weeks–months</t>
+          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
         </is>
       </c>
       <c r="F55" s="16" t="inlineStr">
         <is>
-          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
+          <t>Alters RA’s course, not just symptoms</t>
         </is>
       </c>
       <c r="G55" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H55" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I55" s="1" t="n"/>
@@ -4549,27 +4549,27 @@
       </c>
       <c r="B56" s="16" t="inlineStr">
         <is>
-          <t>NSAID cautions: which is right?</t>
+          <t>NSAID adverse effects: which is right?</t>
         </is>
       </c>
       <c r="C56" s="16" t="inlineStr">
         <is>
-          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
+          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
         </is>
       </c>
       <c r="D56" s="16" t="inlineStr">
         <is>
-          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
+          <t>Anti-CD20; after TNF-inhibitor failure; check hepatitis B</t>
         </is>
       </c>
       <c r="E56" s="16" t="inlineStr">
         <is>
-          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
+          <t>NSAID relief in days · DMARD protection over weeks–months</t>
         </is>
       </c>
       <c r="F56" s="16" t="inlineStr">
         <is>
-          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
+          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
         </is>
       </c>
       <c r="G56" s="14" t="n">
@@ -4577,7 +4577,7 @@
       </c>
       <c r="H56" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I56" s="1" t="n"/>
@@ -4606,31 +4606,31 @@
       </c>
       <c r="B57" s="16" t="inlineStr">
         <is>
-          <t>Triple whammy: which is right?</t>
+          <t>NSAID cautions: which is right?</t>
         </is>
       </c>
       <c r="C57" s="16" t="inlineStr">
         <is>
-          <t>Alters lysosomal and TLR signaling</t>
+          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
+          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
         </is>
       </c>
       <c r="E57" s="16" t="inlineStr">
         <is>
-          <t>COX → prostaglandins specifically</t>
+          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
         </is>
       </c>
       <c r="F57" s="16" t="inlineStr">
         <is>
-          <t>More potent; more GI/CNS effects</t>
+          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
         </is>
       </c>
       <c r="G57" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H57" s="18" t="inlineStr">
         <is>
@@ -4663,27 +4663,27 @@
       </c>
       <c r="B58" s="16" t="inlineStr">
         <is>
-          <t>NSAID + corticosteroid: which is right?</t>
+          <t>Triple whammy: which is right?</t>
         </is>
       </c>
       <c r="C58" s="16" t="inlineStr">
         <is>
-          <t>Tocilizumab</t>
+          <t>Alters lysosomal and TLR signaling</t>
         </is>
       </c>
       <c r="D58" s="16" t="inlineStr">
         <is>
-          <t>↑ GI ulcer risk</t>
+          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
         </is>
       </c>
       <c r="E58" s="16" t="inlineStr">
         <is>
-          <t>Rituximab</t>
+          <t>COX → prostaglandins specifically</t>
         </is>
       </c>
       <c r="F58" s="16" t="inlineStr">
         <is>
-          <t>Oral and topical</t>
+          <t>More potent; more GI/CNS effects</t>
         </is>
       </c>
       <c r="G58" s="14" t="n">
@@ -4720,35 +4720,35 @@
       </c>
       <c r="B59" s="16" t="inlineStr">
         <is>
-          <t>OA vs. RA: which is right?</t>
+          <t>NSAID + corticosteroid: which is right?</t>
         </is>
       </c>
       <c r="C59" s="16" t="inlineStr">
         <is>
-          <t>Baricitinib, tofacitinib, upadacitinib — oral; zoster, ↑ LDL</t>
+          <t>Tocilizumab</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
         <is>
-          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
+          <t>↑ GI ulcer risk</t>
         </is>
       </c>
       <c r="E59" s="16" t="inlineStr">
         <is>
-          <t>~90% glucuronidation/sulfation (safe) · ~5–10% CYP2E1 → NAPQI</t>
+          <t>Rituximab</t>
         </is>
       </c>
       <c r="F59" s="16" t="inlineStr">
         <is>
-          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
+          <t>Oral and topical</t>
         </is>
       </c>
       <c r="G59" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H59" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I59" s="1" t="n"/>
@@ -4777,35 +4777,35 @@
       </c>
       <c r="B60" s="16" t="inlineStr">
         <is>
-          <t>DMARD: which is right?</t>
+          <t>OA vs. RA: which is right?</t>
         </is>
       </c>
       <c r="C60" s="16" t="inlineStr">
         <is>
-          <t>Alters RA’s course, not just symptoms</t>
+          <t>Baricitinib, tofacitinib, upadacitinib — oral; zoster, ↑ LDL</t>
         </is>
       </c>
       <c r="D60" s="16" t="inlineStr">
         <is>
-          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
+          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
         </is>
       </c>
       <c r="E60" s="16" t="inlineStr">
         <is>
-          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
+          <t>~90% glucuronidation/sulfation (safe) · ~5–10% CYP2E1 → NAPQI</t>
         </is>
       </c>
       <c r="F60" s="16" t="inlineStr">
         <is>
-          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
+          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
         </is>
       </c>
       <c r="G60" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H60" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I60" s="1" t="n"/>
@@ -4834,35 +4834,35 @@
       </c>
       <c r="B61" s="16" t="inlineStr">
         <is>
-          <t>Methotrexate: which is right?</t>
+          <t>DMARD: which is right?</t>
         </is>
       </c>
       <c r="C61" s="16" t="inlineStr">
         <is>
-          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
+          <t>Alters RA’s course, not just symptoms</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
+          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
         </is>
       </c>
       <c r="E61" s="16" t="inlineStr">
         <is>
-          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
+          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
         </is>
       </c>
       <c r="F61" s="16" t="inlineStr">
         <is>
-          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
+          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
         </is>
       </c>
       <c r="G61" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H61" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I61" s="1" t="n"/>
@@ -4891,35 +4891,35 @@
       </c>
       <c r="B62" s="16" t="inlineStr">
         <is>
-          <t>TNF inhibitors: which is right?</t>
+          <t>Methotrexate: which is right?</t>
         </is>
       </c>
       <c r="C62" s="16" t="inlineStr">
         <is>
-          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
+          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
         </is>
       </c>
       <c r="D62" s="16" t="inlineStr">
         <is>
-          <t>COX → prostaglandins specifically</t>
+          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
         </is>
       </c>
       <c r="E62" s="16" t="inlineStr">
         <is>
-          <t>Alters lysosomal and TLR signaling</t>
+          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
         </is>
       </c>
       <c r="F62" s="16" t="inlineStr">
         <is>
-          <t>Adalimumab, etanercept, infliximab</t>
+          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
         </is>
       </c>
       <c r="G62" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H62" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I62" s="1" t="n"/>
@@ -4948,27 +4948,27 @@
       </c>
       <c r="B63" s="16" t="inlineStr">
         <is>
-          <t>IL-6 inhibitor: which is right?</t>
+          <t>TNF inhibitors: which is right?</t>
         </is>
       </c>
       <c r="C63" s="16" t="inlineStr">
         <is>
-          <t>Tocilizumab</t>
+          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
         <is>
-          <t>Rituximab</t>
+          <t>COX → prostaglandins specifically</t>
         </is>
       </c>
       <c r="E63" s="16" t="inlineStr">
         <is>
-          <t>Abatacept</t>
+          <t>Alters lysosomal and TLR signaling</t>
         </is>
       </c>
       <c r="F63" s="16" t="inlineStr">
         <is>
-          <t>↑ GI ulcer risk</t>
+          <t>Adalimumab, etanercept, infliximab</t>
         </is>
       </c>
       <c r="G63" s="14" t="n">
@@ -4976,7 +4976,7 @@
       </c>
       <c r="H63" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I63" s="1" t="n"/>
@@ -5005,22 +5005,22 @@
       </c>
       <c r="B64" s="16" t="inlineStr">
         <is>
-          <t>B-cell therapy: which is right?</t>
+          <t>IL-6 inhibitor: which is right?</t>
         </is>
       </c>
       <c r="C64" s="16" t="inlineStr">
         <is>
+          <t>Tocilizumab</t>
+        </is>
+      </c>
+      <c r="D64" s="16" t="inlineStr">
+        <is>
+          <t>Rituximab</t>
+        </is>
+      </c>
+      <c r="E64" s="16" t="inlineStr">
+        <is>
           <t>Abatacept</t>
-        </is>
-      </c>
-      <c r="D64" s="16" t="inlineStr">
-        <is>
-          <t>Tocilizumab</t>
-        </is>
-      </c>
-      <c r="E64" s="16" t="inlineStr">
-        <is>
-          <t>Rituximab</t>
         </is>
       </c>
       <c r="F64" s="16" t="inlineStr">
@@ -5033,7 +5033,7 @@
       </c>
       <c r="H64" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I64" s="1" t="n"/>
@@ -5062,22 +5062,22 @@
       </c>
       <c r="B65" s="16" t="inlineStr">
         <is>
-          <t>T-cell costimulation: which is right?</t>
+          <t>B-cell therapy: which is right?</t>
         </is>
       </c>
       <c r="C65" s="16" t="inlineStr">
         <is>
+          <t>Abatacept</t>
+        </is>
+      </c>
+      <c r="D65" s="16" t="inlineStr">
+        <is>
+          <t>Tocilizumab</t>
+        </is>
+      </c>
+      <c r="E65" s="16" t="inlineStr">
+        <is>
           <t>Rituximab</t>
-        </is>
-      </c>
-      <c r="D65" s="16" t="inlineStr">
-        <is>
-          <t>Abatacept</t>
-        </is>
-      </c>
-      <c r="E65" s="16" t="inlineStr">
-        <is>
-          <t>Tocilizumab</t>
         </is>
       </c>
       <c r="F65" s="16" t="inlineStr">
@@ -5090,7 +5090,7 @@
       </c>
       <c r="H65" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I65" s="1" t="n"/>
@@ -5119,27 +5119,27 @@
       </c>
       <c r="B66" s="16" t="inlineStr">
         <is>
-          <t>DMARD shared risk: which is right?</t>
+          <t>T-cell costimulation: which is right?</t>
         </is>
       </c>
       <c r="C66" s="16" t="inlineStr">
         <is>
-          <t>DHODH (pyrimidine synthesis)</t>
+          <t>Rituximab</t>
         </is>
       </c>
       <c r="D66" s="16" t="inlineStr">
         <is>
-          <t>Immunosuppression → infection</t>
+          <t>Abatacept</t>
         </is>
       </c>
       <c r="E66" s="16" t="inlineStr">
         <is>
-          <t>≤ 7.5 mg daily long term, taper</t>
+          <t>Tocilizumab</t>
         </is>
       </c>
       <c r="F66" s="16" t="inlineStr">
         <is>
-          <t>Longer half-life, twice-daily</t>
+          <t>↑ GI ulcer risk</t>
         </is>
       </c>
       <c r="G66" s="14" t="n">
@@ -5176,31 +5176,31 @@
       </c>
       <c r="B67" s="16" t="inlineStr">
         <is>
-          <t>Before biologics: which is right?</t>
+          <t>DMARD shared risk: which is right?</t>
         </is>
       </c>
       <c r="C67" s="16" t="inlineStr">
         <is>
-          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
+          <t>DHODH (pyrimidine synthesis)</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
         <is>
-          <t>TB + hepatitis B/C screen; update vaccines (live) first</t>
+          <t>Immunosuppression → infection</t>
         </is>
       </c>
       <c r="E67" s="16" t="inlineStr">
         <is>
-          <t>NSAID relief in days · DMARD protection over weeks–months</t>
+          <t>≤ 7.5 mg daily long term, taper</t>
         </is>
       </c>
       <c r="F67" s="16" t="inlineStr">
         <is>
-          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
+          <t>Longer half-life, twice-daily</t>
         </is>
       </c>
       <c r="G67" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H67" s="18" t="inlineStr">
         <is>
@@ -5233,27 +5233,27 @@
       </c>
       <c r="B68" s="16" t="inlineStr">
         <is>
-          <t>Acetaminophen routes: which is right?</t>
+          <t>Before biologics: which is right?</t>
         </is>
       </c>
       <c r="C68" s="16" t="inlineStr">
         <is>
-          <t>~90% glucuronidation/sulfation (safe) · ~5–10% CYP2E1 → NAPQI</t>
+          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
         </is>
       </c>
       <c r="D68" s="16" t="inlineStr">
         <is>
-          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
+          <t>TB + hepatitis B/C screen; update vaccines (live) first</t>
         </is>
       </c>
       <c r="E68" s="16" t="inlineStr">
         <is>
-          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
+          <t>NSAID relief in days · DMARD protection over weeks–months</t>
         </is>
       </c>
       <c r="F68" s="16" t="inlineStr">
         <is>
-          <t>Baricitinib, tofacitinib, upadacitinib — oral; zoster, ↑ LDL</t>
+          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
         </is>
       </c>
       <c r="G68" s="14" t="n">
@@ -5261,7 +5261,7 @@
       </c>
       <c r="H68" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I68" s="1" t="n"/>
@@ -5290,27 +5290,27 @@
       </c>
       <c r="B69" s="16" t="inlineStr">
         <is>
-          <t>Who's at higher acetaminophen risk: which is right?</t>
+          <t>Acetaminophen routes: which is right?</t>
         </is>
       </c>
       <c r="C69" s="16" t="inlineStr">
         <is>
-          <t>Synovitis → pannus; TNF-α and IL-6 drive erosion</t>
+          <t>~90% glucuronidation/sulfation (safe) · ~5–10% CYP2E1 → NAPQI</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
         <is>
-          <t>Chronic alcohol use, fasting (↓ GSH, ↑ CYP2E1)</t>
+          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
         </is>
       </c>
       <c r="E69" s="16" t="inlineStr">
         <is>
-          <t>Likely anti-inflammatory via adenosine release</t>
+          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
         </is>
       </c>
       <c r="F69" s="16" t="inlineStr">
         <is>
-          <t>8 h, 120 mcg/mL → above the line → start NAC</t>
+          <t>Baricitinib, tofacitinib, upadacitinib — oral; zoster, ↑ LDL</t>
         </is>
       </c>
       <c r="G69" s="14" t="n">
@@ -5318,7 +5318,7 @@
       </c>
       <c r="H69" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I69" s="1" t="n"/>
@@ -5347,31 +5347,31 @@
       </c>
       <c r="B70" s="16" t="inlineStr">
         <is>
-          <t>Liver lesion in overdose: which is right?</t>
+          <t>Who's at higher acetaminophen risk: which is right?</t>
         </is>
       </c>
       <c r="C70" s="16" t="inlineStr">
         <is>
-          <t>PGI2 falls, TXA2 preserved</t>
+          <t>Synovitis → pannus; TNF-α and IL-6 drive erosion</t>
         </is>
       </c>
       <c r="D70" s="16" t="inlineStr">
         <is>
-          <t>Centrilobular necrosis</t>
+          <t>Chronic alcohol use, fasting (↓ GSH, ↑ CYP2E1)</t>
         </is>
       </c>
       <c r="E70" s="16" t="inlineStr">
         <is>
-          <t>VTE (DVT/PE), MACE, cancer</t>
+          <t>Likely anti-inflammatory via adenosine release</t>
         </is>
       </c>
       <c r="F70" s="16" t="inlineStr">
         <is>
-          <t>DHODH (pyrimidine synthesis)</t>
+          <t>8 h, 120 mcg/mL → above the line → start NAC</t>
         </is>
       </c>
       <c r="G70" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H70" s="18" t="inlineStr">
         <is>
@@ -5404,31 +5404,31 @@
       </c>
       <c r="B71" s="16" t="inlineStr">
         <is>
-          <t>Rumack-Matthew nomogram: which is right?</t>
+          <t>Liver lesion in overdose: which is right?</t>
         </is>
       </c>
       <c r="C71" s="16" t="inlineStr">
         <is>
-          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
+          <t>PGI2 falls, TXA2 preserved</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
         <is>
-          <t>Single acute ingestion; level ≥ 4 h; above the line → NAC; not used &gt; 24 h</t>
+          <t>Centrilobular necrosis</t>
         </is>
       </c>
       <c r="E71" s="16" t="inlineStr">
         <is>
-          <t>Prostaglandins, bradykinin, histamine, cytokines (TNF-α, IL-1, IL-6)</t>
+          <t>VTE (DVT/PE), MACE, cancer</t>
         </is>
       </c>
       <c r="F71" s="16" t="inlineStr">
         <is>
-          <t>GI: ↓ mucus/bicarbonate · kidney: ↓ afferent dilation · platelets: ↓ TXA2</t>
+          <t>DHODH (pyrimidine synthesis)</t>
         </is>
       </c>
       <c r="G71" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H71" s="18" t="inlineStr">
         <is>
@@ -5461,27 +5461,27 @@
       </c>
       <c r="B72" s="16" t="inlineStr">
         <is>
-          <t>Nomogram example: which is right?</t>
+          <t>Rumack-Matthew nomogram: which is right?</t>
         </is>
       </c>
       <c r="C72" s="16" t="inlineStr">
         <is>
-          <t>Chronic alcohol use, fasting (↓ GSH, ↑ CYP2E1)</t>
+          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
         </is>
       </c>
       <c r="D72" s="16" t="inlineStr">
         <is>
-          <t>8 h, 120 mcg/mL → above the line → start NAC</t>
+          <t>Single acute ingestion; level ≥ 4 h; above the line → NAC; not used &gt; 24 h</t>
         </is>
       </c>
       <c r="E72" s="16" t="inlineStr">
         <is>
-          <t>Likely anti-inflammatory via adenosine release</t>
+          <t>Prostaglandins, bradykinin, histamine, cytokines (TNF-α, IL-1, IL-6)</t>
         </is>
       </c>
       <c r="F72" s="16" t="inlineStr">
         <is>
-          <t>Short-term only; significant GI/renal risk</t>
+          <t>GI: ↓ mucus/bicarbonate · kidney: ↓ afferent dilation · platelets: ↓ TXA2</t>
         </is>
       </c>
       <c r="G72" s="14" t="n">
@@ -5518,27 +5518,27 @@
       </c>
       <c r="B73" s="16" t="inlineStr">
         <is>
-          <t>Nomogram line (illustrative): which is right?</t>
+          <t>Nomogram example: which is right?</t>
         </is>
       </c>
       <c r="C73" s="16" t="inlineStr">
         <is>
-          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
+          <t>Chronic alcohol use, fasting (↓ GSH, ↑ CYP2E1)</t>
         </is>
       </c>
       <c r="D73" s="16" t="inlineStr">
         <is>
-          <t>Persists beyond expected healing, often &gt; 3 months</t>
+          <t>8 h, 120 mcg/mL → above the line → start NAC</t>
         </is>
       </c>
       <c r="E73" s="16" t="inlineStr">
         <is>
-          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
+          <t>Likely anti-inflammatory via adenosine release</t>
         </is>
       </c>
       <c r="F73" s="16" t="inlineStr">
         <is>
-          <t>Housekeeping: gastric protection, renal blood flow</t>
+          <t>Short-term only; significant GI/renal risk</t>
         </is>
       </c>
       <c r="G73" s="14" t="n">
@@ -5546,7 +5546,7 @@
       </c>
       <c r="H73" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I73" s="1" t="n"/>
@@ -5575,31 +5575,31 @@
       </c>
       <c r="B74" s="16" t="inlineStr">
         <is>
-          <t>Celecoxib CV mechanism: which is right?</t>
+          <t>Nomogram line (illustrative): which is right?</t>
         </is>
       </c>
       <c r="C74" s="16" t="inlineStr">
         <is>
-          <t>Longer half-life, twice-daily</t>
+          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
         </is>
       </c>
       <c r="D74" s="16" t="inlineStr">
         <is>
-          <t>VTE (DVT/PE), MACE, cancer</t>
+          <t>Persists beyond expected healing, often &gt; 3 months</t>
         </is>
       </c>
       <c r="E74" s="16" t="inlineStr">
         <is>
-          <t>PGI2 falls, TXA2 preserved</t>
+          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
         </is>
       </c>
       <c r="F74" s="16" t="inlineStr">
         <is>
-          <t>DHODH (pyrimidine synthesis)</t>
+          <t>Housekeeping: gastric protection, renal blood flow</t>
         </is>
       </c>
       <c r="G74" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H74" s="18" t="inlineStr">
         <is>
@@ -5632,35 +5632,35 @@
       </c>
       <c r="B75" s="16" t="inlineStr">
         <is>
-          <t>NSAID organ effects: which is right?</t>
+          <t>Celecoxib CV mechanism: which is right?</t>
         </is>
       </c>
       <c r="C75" s="16" t="inlineStr">
         <is>
-          <t>GI: ↓ mucus/bicarbonate · kidney: ↓ afferent dilation · platelets: ↓ TXA2</t>
+          <t>Longer half-life, twice-daily</t>
         </is>
       </c>
       <c r="D75" s="16" t="inlineStr">
         <is>
-          <t>Prostaglandins, bradykinin, histamine, cytokines (TNF-α, IL-1, IL-6)</t>
+          <t>VTE (DVT/PE), MACE, cancer</t>
         </is>
       </c>
       <c r="E75" s="16" t="inlineStr">
         <is>
-          <t>Single acute ingestion; level ≥ 4 h; above the line → NAC; not used &gt; 24 h</t>
+          <t>PGI2 falls, TXA2 preserved</t>
         </is>
       </c>
       <c r="F75" s="16" t="inlineStr">
         <is>
-          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
+          <t>DHODH (pyrimidine synthesis)</t>
         </is>
       </c>
       <c r="G75" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H75" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I75" s="1" t="n"/>
@@ -5689,27 +5689,27 @@
       </c>
       <c r="B76" s="16" t="inlineStr">
         <is>
-          <t>RA joint destruction: which is right?</t>
+          <t>NSAID organ effects: which is right?</t>
         </is>
       </c>
       <c r="C76" s="16" t="inlineStr">
         <is>
-          <t>Synovitis → pannus; TNF-α and IL-6 drive erosion</t>
+          <t>GI: ↓ mucus/bicarbonate · kidney: ↓ afferent dilation · platelets: ↓ TXA2</t>
         </is>
       </c>
       <c r="D76" s="16" t="inlineStr">
         <is>
-          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
+          <t>Prostaglandins, bradykinin, histamine, cytokines (TNF-α, IL-1, IL-6)</t>
         </is>
       </c>
       <c r="E76" s="16" t="inlineStr">
         <is>
-          <t>Housekeeping: gastric protection, renal blood flow</t>
+          <t>Single acute ingestion; level ≥ 4 h; above the line → NAC; not used &gt; 24 h</t>
         </is>
       </c>
       <c r="F76" s="16" t="inlineStr">
         <is>
-          <t>Chronic alcohol use, fasting (↓ GSH, ↑ CYP2E1)</t>
+          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
         </is>
       </c>
       <c r="G76" s="14" t="n">
@@ -5746,27 +5746,27 @@
       </c>
       <c r="B77" s="16" t="inlineStr">
         <is>
-          <t>NSAID vs. DMARD onset: which is right?</t>
+          <t>RA joint destruction: which is right?</t>
         </is>
       </c>
       <c r="C77" s="16" t="inlineStr">
         <is>
-          <t>Anti-CD20; after TNF-inhibitor failure; check hepatitis B</t>
+          <t>Synovitis → pannus; TNF-α and IL-6 drive erosion</t>
         </is>
       </c>
       <c r="D77" s="16" t="inlineStr">
         <is>
-          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
+          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
         </is>
       </c>
       <c r="E77" s="16" t="inlineStr">
         <is>
-          <t>NSAID relief in days · DMARD protection over weeks–months</t>
+          <t>Housekeeping: gastric protection, renal blood flow</t>
         </is>
       </c>
       <c r="F77" s="16" t="inlineStr">
         <is>
-          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
+          <t>Chronic alcohol use, fasting (↓ GSH, ↑ CYP2E1)</t>
         </is>
       </c>
       <c r="G77" s="14" t="n">
@@ -5774,7 +5774,7 @@
       </c>
       <c r="H77" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I77" s="1" t="n"/>
@@ -5803,31 +5803,31 @@
       </c>
       <c r="B78" s="16" t="inlineStr">
         <is>
-          <t>Leflunomide target: which is right?</t>
+          <t>NSAID vs. DMARD onset: which is right?</t>
         </is>
       </c>
       <c r="C78" s="16" t="inlineStr">
         <is>
-          <t>PGI2 falls, TXA2 preserved</t>
+          <t>Anti-CD20; after TNF-inhibitor failure; check hepatitis B</t>
         </is>
       </c>
       <c r="D78" s="16" t="inlineStr">
         <is>
-          <t>Immunosuppression → infection</t>
+          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
         </is>
       </c>
       <c r="E78" s="16" t="inlineStr">
         <is>
-          <t>DHODH (pyrimidine synthesis)</t>
+          <t>NSAID relief in days · DMARD protection over weeks–months</t>
         </is>
       </c>
       <c r="F78" s="16" t="inlineStr">
         <is>
-          <t>Longer half-life, twice-daily</t>
+          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
         </is>
       </c>
       <c r="G78" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H78" s="18" t="inlineStr">
         <is>
@@ -5860,27 +5860,27 @@
       </c>
       <c r="B79" s="16" t="inlineStr">
         <is>
-          <t>Hydroxychloroquine action: which is right?</t>
+          <t>Leflunomide target: which is right?</t>
         </is>
       </c>
       <c r="C79" s="16" t="inlineStr">
         <is>
-          <t>Alters lysosomal and TLR signaling</t>
+          <t>PGI2 falls, TXA2 preserved</t>
         </is>
       </c>
       <c r="D79" s="16" t="inlineStr">
         <is>
-          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
+          <t>Immunosuppression → infection</t>
         </is>
       </c>
       <c r="E79" s="16" t="inlineStr">
         <is>
-          <t>COX → prostaglandins specifically</t>
+          <t>DHODH (pyrimidine synthesis)</t>
         </is>
       </c>
       <c r="F79" s="16" t="inlineStr">
         <is>
-          <t>Adalimumab, etanercept, infliximab</t>
+          <t>Longer half-life, twice-daily</t>
         </is>
       </c>
       <c r="G79" s="14" t="n">
@@ -5888,7 +5888,7 @@
       </c>
       <c r="H79" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I79" s="1" t="n"/>
@@ -5917,35 +5917,35 @@
       </c>
       <c r="B80" s="16" t="inlineStr">
         <is>
-          <t>Methotrexate at low dose: which is right?</t>
+          <t>Hydroxychloroquine action: which is right?</t>
         </is>
       </c>
       <c r="C80" s="16" t="inlineStr">
         <is>
-          <t>Synovitis → pannus; TNF-α and IL-6 drive erosion</t>
+          <t>Alters lysosomal and TLR signaling</t>
         </is>
       </c>
       <c r="D80" s="16" t="inlineStr">
         <is>
-          <t>Chronic alcohol use, fasting (↓ GSH, ↑ CYP2E1)</t>
+          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
         </is>
       </c>
       <c r="E80" s="16" t="inlineStr">
         <is>
-          <t>Likely anti-inflammatory via adenosine release</t>
+          <t>COX → prostaglandins specifically</t>
         </is>
       </c>
       <c r="F80" s="16" t="inlineStr">
         <is>
-          <t>8 h, 120 mcg/mL → above the line → start NAC</t>
+          <t>Adalimumab, etanercept, infliximab</t>
         </is>
       </c>
       <c r="G80" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H80" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I80" s="1" t="n"/>
@@ -5974,27 +5974,27 @@
       </c>
       <c r="B81" s="16" t="inlineStr">
         <is>
-          <t>Abatacept: which is right?</t>
+          <t>Methotrexate at low dose: which is right?</t>
         </is>
       </c>
       <c r="C81" s="16" t="inlineStr">
         <is>
-          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
+          <t>Synovitis → pannus; TNF-α and IL-6 drive erosion</t>
         </is>
       </c>
       <c r="D81" s="16" t="inlineStr">
         <is>
-          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
+          <t>Chronic alcohol use, fasting (↓ GSH, ↑ CYP2E1)</t>
         </is>
       </c>
       <c r="E81" s="16" t="inlineStr">
         <is>
-          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
+          <t>Likely anti-inflammatory via adenosine release</t>
         </is>
       </c>
       <c r="F81" s="16" t="inlineStr">
         <is>
-          <t>Prostaglandins, bradykinin, histamine, cytokines (TNF-α, IL-1, IL-6)</t>
+          <t>8 h, 120 mcg/mL → above the line → start NAC</t>
         </is>
       </c>
       <c r="G81" s="14" t="n">
@@ -6031,27 +6031,27 @@
       </c>
       <c r="B82" s="16" t="inlineStr">
         <is>
-          <t>Rituximab: which is right?</t>
+          <t>Abatacept: which is right?</t>
         </is>
       </c>
       <c r="C82" s="16" t="inlineStr">
         <is>
-          <t>Anti-CD20; after TNF-inhibitor failure; check hepatitis B</t>
+          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
         </is>
       </c>
       <c r="D82" s="16" t="inlineStr">
         <is>
-          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
+          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
         </is>
       </c>
       <c r="E82" s="16" t="inlineStr">
         <is>
-          <t>NSAID relief in days · DMARD protection over weeks–months</t>
+          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
         </is>
       </c>
       <c r="F82" s="16" t="inlineStr">
         <is>
-          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
+          <t>Prostaglandins, bradykinin, histamine, cytokines (TNF-α, IL-1, IL-6)</t>
         </is>
       </c>
       <c r="G82" s="14" t="n">
@@ -6059,7 +6059,7 @@
       </c>
       <c r="H82" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I82" s="1" t="n"/>
@@ -6088,27 +6088,27 @@
       </c>
       <c r="B83" s="16" t="inlineStr">
         <is>
-          <t>Infection monitoring on DMARDs: which is right?</t>
+          <t>Rituximab: which is right?</t>
         </is>
       </c>
       <c r="C83" s="16" t="inlineStr">
         <is>
-          <t>CBC, liver, kidney labs every 1–3 months</t>
+          <t>Anti-CD20; after TNF-inhibitor failure; check hepatitis B</t>
         </is>
       </c>
       <c r="D83" s="16" t="inlineStr">
         <is>
-          <t>Nociceptive · inflammatory · neuropathic</t>
+          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
         </is>
       </c>
       <c r="E83" s="16" t="inlineStr">
         <is>
-          <t>Common first-line for mild-moderate pain</t>
+          <t>NSAID relief in days · DMARD protection over weeks–months</t>
         </is>
       </c>
       <c r="F83" s="16" t="inlineStr">
         <is>
-          <t>N-acetylcysteine — glutathione precursor</t>
+          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
         </is>
       </c>
       <c r="G83" s="14" t="n">
@@ -6145,31 +6145,31 @@
       </c>
       <c r="B84" s="16" t="inlineStr">
         <is>
-          <t>Acetaminophen max (adults): which is right?</t>
+          <t>Infection monitoring on DMARDs: which is right?</t>
         </is>
       </c>
       <c r="C84" s="16" t="inlineStr">
         <is>
-          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
+          <t>CBC, liver, kidney labs every 1–3 months</t>
         </is>
       </c>
       <c r="D84" s="16" t="inlineStr">
         <is>
-          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
+          <t>Nociceptive · inflammatory · neuropathic</t>
         </is>
       </c>
       <c r="E84" s="16" t="inlineStr">
         <is>
-          <t>Alters RA’s course, not just symptoms</t>
+          <t>Common first-line for mild-moderate pain</t>
         </is>
       </c>
       <c r="F84" s="16" t="inlineStr">
         <is>
-          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
+          <t>N-acetylcysteine — glutathione precursor</t>
         </is>
       </c>
       <c r="G84" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H84" s="18" t="inlineStr">
         <is>
@@ -6202,35 +6202,35 @@
       </c>
       <c r="B85" s="16" t="inlineStr">
         <is>
-          <t>Aspirin vs. other NSAIDs: which is right?</t>
+          <t>Acetaminophen max (adults): which is right?</t>
         </is>
       </c>
       <c r="C85" s="16" t="inlineStr">
         <is>
-          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
+          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
         </is>
       </c>
       <c r="D85" s="16" t="inlineStr">
         <is>
-          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
+          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
         </is>
       </c>
       <c r="E85" s="16" t="inlineStr">
         <is>
-          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
+          <t>Alters RA’s course, not just symptoms</t>
         </is>
       </c>
       <c r="F85" s="16" t="inlineStr">
         <is>
-          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
+          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
         </is>
       </c>
       <c r="G85" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H85" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I85" s="1" t="n"/>
@@ -6259,31 +6259,31 @@
       </c>
       <c r="B86" s="16" t="inlineStr">
         <is>
-          <t>Celecoxib selectivity: which is right?</t>
+          <t>Aspirin vs. other NSAIDs: which is right?</t>
         </is>
       </c>
       <c r="C86" s="16" t="inlineStr">
         <is>
-          <t>Malignancy, especially lymphoma</t>
+          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
         </is>
       </c>
       <c r="D86" s="16" t="inlineStr">
         <is>
-          <t>10–20× more selective for COX-2</t>
+          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
         </is>
       </c>
       <c r="E86" s="16" t="inlineStr">
         <is>
-          <t>≤ 7.5 mg daily long term, taper</t>
+          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
         </is>
       </c>
       <c r="F86" s="16" t="inlineStr">
         <is>
-          <t>7.5 mg weekly → 15–25 mg weekly</t>
+          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
         </is>
       </c>
       <c r="G86" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H86" s="18" t="inlineStr">
         <is>
@@ -6316,17 +6316,17 @@
       </c>
       <c r="B87" s="16" t="inlineStr">
         <is>
-          <t>Methotrexate dose: which is right?</t>
+          <t>Celecoxib selectivity: which is right?</t>
         </is>
       </c>
       <c r="C87" s="16" t="inlineStr">
         <is>
+          <t>Malignancy, especially lymphoma</t>
+        </is>
+      </c>
+      <c r="D87" s="16" t="inlineStr">
+        <is>
           <t>10–20× more selective for COX-2</t>
-        </is>
-      </c>
-      <c r="D87" s="16" t="inlineStr">
-        <is>
-          <t>Malignancy, especially lymphoma</t>
         </is>
       </c>
       <c r="E87" s="16" t="inlineStr">
@@ -6344,7 +6344,7 @@
       </c>
       <c r="H87" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I87" s="1" t="n"/>
@@ -6373,27 +6373,27 @@
       </c>
       <c r="B88" s="16" t="inlineStr">
         <is>
-          <t>Hydroxychloroquine monitoring: which is right?</t>
+          <t>Methotrexate dose: which is right?</t>
         </is>
       </c>
       <c r="C88" s="16" t="inlineStr">
         <is>
-          <t>Baseline eye exam; annual after 5 years</t>
+          <t>10–20× more selective for COX-2</t>
         </is>
       </c>
       <c r="D88" s="16" t="inlineStr">
         <is>
-          <t>CBC, liver, kidney labs every 1–3 months</t>
+          <t>Malignancy, especially lymphoma</t>
         </is>
       </c>
       <c r="E88" s="16" t="inlineStr">
         <is>
-          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
+          <t>≤ 7.5 mg daily long term, taper</t>
         </is>
       </c>
       <c r="F88" s="16" t="inlineStr">
         <is>
-          <t>Common first-line for mild-moderate pain</t>
+          <t>7.5 mg weekly → 15–25 mg weekly</t>
         </is>
       </c>
       <c r="G88" s="14" t="n">
@@ -6401,7 +6401,7 @@
       </c>
       <c r="H88" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I88" s="1" t="n"/>
@@ -6430,27 +6430,27 @@
       </c>
       <c r="B89" s="16" t="inlineStr">
         <is>
-          <t>TNF inhibitor boxed warning: which is right?</t>
+          <t>Hydroxychloroquine monitoring: which is right?</t>
         </is>
       </c>
       <c r="C89" s="16" t="inlineStr">
         <is>
-          <t>10–20× more selective for COX-2</t>
+          <t>Baseline eye exam; annual after 5 years</t>
         </is>
       </c>
       <c r="D89" s="16" t="inlineStr">
         <is>
-          <t>7.5 mg weekly → 15–25 mg weekly</t>
+          <t>CBC, liver, kidney labs every 1–3 months</t>
         </is>
       </c>
       <c r="E89" s="16" t="inlineStr">
         <is>
-          <t>Malignancy, especially lymphoma</t>
+          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
         </is>
       </c>
       <c r="F89" s="16" t="inlineStr">
         <is>
-          <t>≤ 7.5 mg daily long term, taper</t>
+          <t>Common first-line for mild-moderate pain</t>
         </is>
       </c>
       <c r="G89" s="14" t="n">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="H89" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I89" s="1" t="n"/>
@@ -6487,27 +6487,27 @@
       </c>
       <c r="B90" s="16" t="inlineStr">
         <is>
-          <t>JAK inhibitor boxed warning: which is right?</t>
+          <t>TNF inhibitor boxed warning: which is right?</t>
         </is>
       </c>
       <c r="C90" s="16" t="inlineStr">
         <is>
-          <t>VTE (DVT/PE), MACE, cancer</t>
+          <t>10–20× more selective for COX-2</t>
         </is>
       </c>
       <c r="D90" s="16" t="inlineStr">
         <is>
-          <t>Longer half-life, twice-daily</t>
+          <t>7.5 mg weekly → 15–25 mg weekly</t>
         </is>
       </c>
       <c r="E90" s="16" t="inlineStr">
         <is>
-          <t>PGI2 falls, TXA2 preserved</t>
+          <t>Malignancy, especially lymphoma</t>
         </is>
       </c>
       <c r="F90" s="16" t="inlineStr">
         <is>
-          <t>DHODH (pyrimidine synthesis)</t>
+          <t>≤ 7.5 mg daily long term, taper</t>
         </is>
       </c>
       <c r="G90" s="14" t="n">
@@ -6515,7 +6515,7 @@
       </c>
       <c r="H90" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I90" s="1" t="n"/>
@@ -6544,35 +6544,35 @@
       </c>
       <c r="B91" s="16" t="inlineStr">
         <is>
-          <t>JAK inhibitors: which is right?</t>
+          <t>JAK inhibitor boxed warning: which is right?</t>
         </is>
       </c>
       <c r="C91" s="16" t="inlineStr">
         <is>
-          <t>~90% glucuronidation/sulfation (safe) · ~5–10% CYP2E1 → NAPQI</t>
+          <t>VTE (DVT/PE), MACE, cancer</t>
         </is>
       </c>
       <c r="D91" s="16" t="inlineStr">
         <is>
-          <t>Baricitinib, tofacitinib, upadacitinib — oral; zoster, ↑ LDL</t>
+          <t>Longer half-life, twice-daily</t>
         </is>
       </c>
       <c r="E91" s="16" t="inlineStr">
         <is>
-          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
+          <t>PGI2 falls, TXA2 preserved</t>
         </is>
       </c>
       <c r="F91" s="16" t="inlineStr">
         <is>
-          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
+          <t>DHODH (pyrimidine synthesis)</t>
         </is>
       </c>
       <c r="G91" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H91" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I91" s="1" t="n"/>
@@ -6601,31 +6601,31 @@
       </c>
       <c r="B92" s="16" t="inlineStr">
         <is>
-          <t>RA prednisone ceiling: which is right?</t>
+          <t>JAK inhibitors: which is right?</t>
         </is>
       </c>
       <c r="C92" s="16" t="inlineStr">
         <is>
-          <t>7.5 mg weekly → 15–25 mg weekly</t>
+          <t>~90% glucuronidation/sulfation (safe) · ~5–10% CYP2E1 → NAPQI</t>
         </is>
       </c>
       <c r="D92" s="16" t="inlineStr">
         <is>
-          <t>≤ 7.5 mg daily long term, taper</t>
+          <t>Baricitinib, tofacitinib, upadacitinib — oral; zoster, ↑ LDL</t>
         </is>
       </c>
       <c r="E92" s="16" t="inlineStr">
         <is>
-          <t>Malignancy, especially lymphoma</t>
+          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
         </is>
       </c>
       <c r="F92" s="16" t="inlineStr">
         <is>
-          <t>10–20× more selective for COX-2</t>
+          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
         </is>
       </c>
       <c r="G92" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H92" s="18" t="inlineStr">
         <is>
@@ -6653,14 +6653,42 @@
       <c r="AA92" s="1" t="n"/>
     </row>
     <row r="93" ht="25.5" customHeight="1">
-      <c r="A93" s="11" t="n"/>
-      <c r="B93" s="16" t="n"/>
-      <c r="C93" s="16" t="n"/>
-      <c r="D93" s="16" t="n"/>
-      <c r="E93" s="16" t="n"/>
-      <c r="F93" s="16" t="n"/>
-      <c r="G93" s="14" t="n"/>
-      <c r="H93" s="18" t="n"/>
+      <c r="A93" s="11" t="n">
+        <v>85</v>
+      </c>
+      <c r="B93" s="16" t="inlineStr">
+        <is>
+          <t>RA prednisone ceiling: which is right?</t>
+        </is>
+      </c>
+      <c r="C93" s="16" t="inlineStr">
+        <is>
+          <t>7.5 mg weekly → 15–25 mg weekly</t>
+        </is>
+      </c>
+      <c r="D93" s="16" t="inlineStr">
+        <is>
+          <t>≤ 7.5 mg daily long term, taper</t>
+        </is>
+      </c>
+      <c r="E93" s="16" t="inlineStr">
+        <is>
+          <t>Malignancy, especially lymphoma</t>
+        </is>
+      </c>
+      <c r="F93" s="16" t="inlineStr">
+        <is>
+          <t>10–20× more selective for COX-2</t>
+        </is>
+      </c>
+      <c r="G93" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="H93" s="18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="I93" s="1" t="n"/>
       <c r="J93" s="1" t="n"/>
       <c r="K93" s="1" t="n"/>

</xml_diff>

<commit_message>
Unit 2 practice exam: 20 applied decision-style questions across both sessions (70 total)
</commit_message>
<xml_diff>
--- a/docs/sketch/kahoot/unit2_L03.xlsx
+++ b/docs/sketch/kahoot/unit2_L03.xlsx
@@ -1875,22 +1875,22 @@
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
+          <t>It raises renal blood flow excessively</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>It depletes glutathione in the heart</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
+        <is>
           <t>TXA2 falls while PGI2 is preserved</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>It raises renal blood flow excessively</t>
-        </is>
-      </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="F9" s="14" t="inlineStr">
         <is>
           <t>PGI2 falls while platelet TXA2 is preserved</t>
-        </is>
-      </c>
-      <c r="F9" s="14" t="inlineStr">
-        <is>
-          <t>It depletes glutathione in the heart</t>
         </is>
       </c>
       <c r="G9" s="14" t="n">
@@ -1898,7 +1898,7 @@
       </c>
       <c r="H9" s="15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I9" s="1" t="n"/>
@@ -1927,27 +1927,27 @@
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>Which set lists methotrexate's key adverse effects from the lecture?</t>
+          <t>A patient stable on warfarin is started on celecoxib for osteoarthritis. What should the clinician anticipate?</t>
         </is>
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>Hypersensitivity, lymphoma, heart failure</t>
+          <t>Hemolysis requiring G6PD testing</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>Retinopathy, cardiomyopathy, myopathy</t>
+          <t>Faster renal clearance of warfarin</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>Hepatotoxicity, marrow suppression, pulmonary toxicity</t>
+          <t>Higher bleeding risk — monitor INR closely</t>
         </is>
       </c>
       <c r="F10" s="14" t="inlineStr">
         <is>
-          <t>Tinnitus, aseptic meningitis, rash</t>
+          <t>Lower INR and clot formation</t>
         </is>
       </c>
       <c r="G10" s="14" t="n">
@@ -1984,27 +1984,27 @@
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>Which sequence describes joint destruction in rheumatoid arthritis, as opposed to osteoarthritis?</t>
+          <t>Which set lists methotrexate's key adverse effects from the lecture?</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>Uric acid crystals deposit and trigger a flare</t>
+          <t>GI bleeding, AKI, cardiovascular events</t>
         </is>
       </c>
       <c r="D11" s="21" t="inlineStr">
         <is>
-          <t>Synovitis forms a pannus; TNF-α and IL-6 drive erosion</t>
+          <t>Hepatotoxicity, marrow suppression, pulmonary toxicity</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>Mechanical wear degrades cartilage; osteophytes form</t>
+          <t>Hypersensitivity, lymphoma, heart failure</t>
         </is>
       </c>
       <c r="F11" s="14" t="inlineStr">
         <is>
-          <t>NAPQI binds proteins in the synovial lining</t>
+          <t>Tinnitus, aseptic meningitis, rash</t>
         </is>
       </c>
       <c r="G11" s="14" t="n">
@@ -2041,27 +2041,27 @@
       </c>
       <c r="B12" s="14" t="inlineStr">
         <is>
-          <t>A patient with RA cannot tolerate methotrexate. Which conventional DMARD does the lecture name as the alternative?</t>
+          <t>Which sequence describes joint destruction in rheumatoid arthritis, as opposed to osteoarthritis?</t>
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>Hydroxychloroquine</t>
+          <t>Synovitis forms a pannus; TNF-α and IL-6 drive erosion</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>Rituximab</t>
+          <t>NAPQI binds proteins in the synovial lining</t>
         </is>
       </c>
       <c r="E12" s="14" t="inlineStr">
         <is>
-          <t>Sulfasalazine</t>
+          <t>Prostaglandin loss thins the gastric mucosa</t>
         </is>
       </c>
       <c r="F12" s="14" t="inlineStr">
         <is>
-          <t>Leflunomide</t>
+          <t>Uric acid crystals deposit and trigger a flare</t>
         </is>
       </c>
       <c r="G12" s="14" t="n">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="H12" s="15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I12" s="1" t="n"/>
@@ -2098,35 +2098,35 @@
       </c>
       <c r="B13" s="14" t="inlineStr">
         <is>
-          <t>Rituximab treats rheumatoid arthritis by which mechanism?</t>
+          <t>A patient with RA cannot tolerate methotrexate. Which conventional DMARD does the lecture name as the alternative?</t>
         </is>
       </c>
       <c r="C13" s="14" t="inlineStr">
         <is>
-          <t>Depleting or modulating B lymphocytes</t>
+          <t>Celecoxib</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
         <is>
-          <t>Blocking IL-6 receptor signaling</t>
+          <t>Hydroxychloroquine</t>
         </is>
       </c>
       <c r="E13" s="14" t="inlineStr">
         <is>
-          <t>Inhibiting dihydrofolate reductase</t>
+          <t>Leflunomide</t>
         </is>
       </c>
       <c r="F13" s="14" t="inlineStr">
         <is>
-          <t>Blocking TNF-α signaling</t>
+          <t>Rituximab</t>
         </is>
       </c>
       <c r="G13" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H13" s="15" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I13" s="1" t="n"/>
@@ -2155,31 +2155,31 @@
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>A patient will start infliximab next month and is due for a live vaccine. When should the vaccine be given?</t>
+          <t>Rituximab treats rheumatoid arthritis by which mechanism?</t>
         </is>
       </c>
       <c r="C14" s="14" t="inlineStr">
         <is>
-          <t>Before infliximab is started</t>
+          <t>Depleting or modulating B lymphocytes</t>
         </is>
       </c>
       <c r="D14" s="14" t="inlineStr">
         <is>
-          <t>One week after the first infusion</t>
+          <t>Blocking T-cell costimulation</t>
         </is>
       </c>
       <c r="E14" s="14" t="inlineStr">
         <is>
-          <t>Only if a fever develops on therapy</t>
+          <t>Blocking TNF-α signaling</t>
         </is>
       </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
-          <t>Any time, since biologics don't affect immunity</t>
+          <t>Blocking IL-6 receptor signaling</t>
         </is>
       </c>
       <c r="G14" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H14" s="15" t="inlineStr">
         <is>
@@ -2212,35 +2212,35 @@
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>Which NSAID is noted for oral and topical formulations?</t>
+          <t>A patient will start infliximab next month and is due for a live vaccine. When should the vaccine be given?</t>
         </is>
       </c>
       <c r="C15" s="14" t="inlineStr">
         <is>
-          <t>Naproxen</t>
+          <t>Never — vaccines are banned for life</t>
         </is>
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>Ketorolac</t>
+          <t>Before infliximab is started</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
         <is>
-          <t>Diclofenac</t>
+          <t>Only if a fever develops on therapy</t>
         </is>
       </c>
       <c r="F15" s="14" t="inlineStr">
         <is>
-          <t>Indomethacin</t>
+          <t>Any time, since biologics don't affect immunity</t>
         </is>
       </c>
       <c r="G15" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H15" s="15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I15" s="1" t="n"/>
@@ -2269,35 +2269,35 @@
       </c>
       <c r="B16" s="14" t="inlineStr">
         <is>
-          <t>Why do corticosteroids suppress a broader range of inflammatory mediators than NSAIDs?</t>
+          <t>Which NSAID is noted for oral and topical formulations?</t>
         </is>
       </c>
       <c r="C16" s="14" t="inlineStr">
         <is>
-          <t>They deplete B cells that release prostaglandins</t>
+          <t>Indomethacin</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr">
         <is>
-          <t>They block phospholipase A₂, upstream of COX</t>
+          <t>Celecoxib</t>
         </is>
       </c>
       <c r="E16" s="14" t="inlineStr">
         <is>
-          <t>They act centrally on the hypothalamus</t>
+          <t>Naproxen</t>
         </is>
       </c>
       <c r="F16" s="14" t="inlineStr">
         <is>
-          <t>They block COX-2 more strongly than any NSAID</t>
+          <t>Diclofenac</t>
         </is>
       </c>
       <c r="G16" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H16" s="15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I16" s="1" t="n"/>
@@ -2326,35 +2326,35 @@
       </c>
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>A 72-year-old with CKD, hypertension, and anticoagulation has an acute gout flare. Which option is often preferred?</t>
+          <t>Why do corticosteroids suppress a broader range of inflammatory mediators than NSAIDs?</t>
         </is>
       </c>
       <c r="C17" s="14" t="inlineStr">
         <is>
-          <t>Full-dose oral naproxen</t>
+          <t>They deplete B cells that release prostaglandins</t>
         </is>
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>Starting allopurinol today</t>
+          <t>They block phospholipase A₂, upstream of COX</t>
         </is>
       </c>
       <c r="E17" s="14" t="inlineStr">
         <is>
-          <t>A short corticosteroid course</t>
+          <t>They block COX-2 more strongly than any NSAID</t>
         </is>
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>Probenecid to clear uric acid</t>
+          <t>They neutralize TNF-α outside the cell</t>
         </is>
       </c>
       <c r="G17" s="14" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="H17" s="15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I17" s="1" t="n"/>
@@ -2383,35 +2383,35 @@
       </c>
       <c r="B18" s="14" t="inlineStr">
         <is>
-          <t>Which drug pairing does the lecture flag for a higher GI ulcer risk?</t>
+          <t>A 72-year-old with CKD, hypertension, and anticoagulation has an acute gout flare. Which option is often preferred?</t>
         </is>
       </c>
       <c r="C18" s="14" t="inlineStr">
         <is>
-          <t>NSAID plus an ACE inhibitor</t>
+          <t>A short corticosteroid course</t>
         </is>
       </c>
       <c r="D18" s="14" t="inlineStr">
         <is>
-          <t>NSAID plus a diuretic</t>
+          <t>Full-dose oral naproxen</t>
         </is>
       </c>
       <c r="E18" s="14" t="inlineStr">
         <is>
-          <t>NSAID plus a corticosteroid</t>
+          <t>Full-dose colchicine, unadjusted</t>
         </is>
       </c>
       <c r="F18" s="14" t="inlineStr">
         <is>
-          <t>Acetaminophen plus N-acetylcysteine</t>
+          <t>Probenecid to clear uric acid</t>
         </is>
       </c>
       <c r="G18" s="14" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="H18" s="15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I18" s="1" t="n"/>
@@ -2440,35 +2440,35 @@
       </c>
       <c r="B19" s="14" t="inlineStr">
         <is>
-          <t>Which statement correctly describes COX-1?</t>
+          <t>Which drug pairing does the lecture flag for a higher GI ulcer risk?</t>
         </is>
       </c>
       <c r="C19" s="14" t="inlineStr">
         <is>
-          <t>Inducible enzyme found mainly at inflamed sites</t>
+          <t>Acetaminophen plus N-acetylcysteine</t>
         </is>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>Main source of inflammatory prostaglandins</t>
+          <t>NSAID plus a corticosteroid</t>
         </is>
       </c>
       <c r="E19" s="14" t="inlineStr">
         <is>
-          <t>Target of celecoxib's selective inhibition</t>
+          <t>NSAID plus a diuretic</t>
         </is>
       </c>
       <c r="F19" s="14" t="inlineStr">
         <is>
-          <t>Housekeeping enzyme protecting stomach and renal flow</t>
+          <t>NSAID plus an ACE inhibitor</t>
         </is>
       </c>
       <c r="G19" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H19" s="15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I19" s="1" t="n"/>
@@ -2497,35 +2497,35 @@
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>Per the textbook, which instruction about ketorolac is correct?</t>
+          <t>Which statement correctly describes COX-1?</t>
         </is>
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>Maximum daily dose is 240 mg</t>
+          <t>Housekeeping enzyme protecting stomach and renal flow</t>
         </is>
       </c>
       <c r="D20" s="14" t="inlineStr">
         <is>
-          <t>Safe long-term in renal impairment</t>
+          <t>Inducible enzyme found mainly at inflamed sites</t>
         </is>
       </c>
       <c r="E20" s="14" t="inlineStr">
         <is>
-          <t>Start therapy with an oral dose</t>
+          <t>Enzyme that converts acetaminophen to NAPQI</t>
         </is>
       </c>
       <c r="F20" s="14" t="inlineStr">
         <is>
-          <t>Use no longer than 5 days</t>
+          <t>Main source of inflammatory prostaglandins</t>
         </is>
       </c>
       <c r="G20" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H20" s="15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I20" s="1" t="n"/>
@@ -2554,27 +2554,27 @@
       </c>
       <c r="B21" s="14" t="inlineStr">
         <is>
-          <t>Which effect is acetaminophen least reliable for?</t>
+          <t>Per the textbook, which instruction about ketorolac is correct?</t>
         </is>
       </c>
       <c r="C21" s="14" t="inlineStr">
         <is>
-          <t>Pain in a patient with CKD</t>
+          <t>Start therapy with an oral dose</t>
         </is>
       </c>
       <c r="D21" s="14" t="inlineStr">
         <is>
-          <t>Reducing peripheral inflammation</t>
+          <t>Maximum daily dose is 240 mg</t>
         </is>
       </c>
       <c r="E21" s="14" t="inlineStr">
         <is>
-          <t>Relieving mild-to-moderate pain</t>
+          <t>Double the dose in patients over 65</t>
         </is>
       </c>
       <c r="F21" s="14" t="inlineStr">
         <is>
-          <t>Lowering fever</t>
+          <t>Use no longer than 5 days</t>
         </is>
       </c>
       <c r="G21" s="14" t="n">
@@ -2582,7 +2582,7 @@
       </c>
       <c r="H21" s="15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I21" s="1" t="n"/>
@@ -2611,27 +2611,27 @@
       </c>
       <c r="B22" s="14" t="inlineStr">
         <is>
-          <t>What defines a drug as “disease-modifying” in rheumatoid arthritis?</t>
+          <t>A patient develops a GI bleed while taking a standard dose of naproxen. How is this adverse effect best classified?</t>
         </is>
       </c>
       <c r="C22" s="14" t="inlineStr">
         <is>
-          <t>It lowers fever through the hypothalamus</t>
+          <t>Type B — idiosyncratic and unpredictable</t>
         </is>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>It relieves pain faster than NSAIDs</t>
+          <t>Pharmacogenomic reaction from HLA-B*58:01</t>
         </is>
       </c>
       <c r="E22" s="14" t="inlineStr">
         <is>
-          <t>It slows or halts joint destruction</t>
+          <t>Type A — predictable from COX-1 inhibition</t>
         </is>
       </c>
       <c r="F22" s="14" t="inlineStr">
         <is>
-          <t>It selectively blocks the COX-2 isoform</t>
+          <t>Therapeutic effect of reduced inflammation</t>
         </is>
       </c>
       <c r="G22" s="14" t="n">
@@ -2668,31 +2668,31 @@
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>Which non-drug approaches does the lecture include in osteoarthritis management?</t>
+          <t>Which effect is acetaminophen least reliable for?</t>
         </is>
       </c>
       <c r="C23" s="14" t="inlineStr">
         <is>
-          <t>Glutathione replenishment, label review</t>
+          <t>Pain in a patient with CKD</t>
         </is>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
-          <t>Activity modification, physical therapy, weight management</t>
+          <t>Reducing peripheral inflammation</t>
         </is>
       </c>
       <c r="E23" s="14" t="inlineStr">
         <is>
-          <t>Live vaccines, TB screening, folate</t>
+          <t>First-line mild osteoarthritis pain</t>
         </is>
       </c>
       <c r="F23" s="14" t="inlineStr">
         <is>
-          <t>Nerve ablation, spinal cord stimulation</t>
+          <t>Lowering fever</t>
         </is>
       </c>
       <c r="G23" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H23" s="15" t="inlineStr">
         <is>
@@ -2725,35 +2725,35 @@
       </c>
       <c r="B24" s="14" t="inlineStr">
         <is>
-          <t>A prescription reads infliximab. What does the stem “-ximab” tell you?</t>
+          <t>What defines a drug as “disease-modifying” in rheumatoid arthritis?</t>
         </is>
       </c>
       <c r="C24" s="14" t="inlineStr">
         <is>
-          <t>A receptor fusion protein</t>
+          <t>It slows or halts joint destruction</t>
         </is>
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
-          <t>A fully human monoclonal antibody</t>
+          <t>It relieves pain faster than NSAIDs</t>
         </is>
       </c>
       <c r="E24" s="14" t="inlineStr">
         <is>
-          <t>A chimeric monoclonal antibody</t>
+          <t>It lowers fever through the hypothalamus</t>
         </is>
       </c>
       <c r="F24" s="14" t="inlineStr">
         <is>
-          <t>A kinase inhibitor</t>
+          <t>It selectively blocks the COX-2 isoform</t>
         </is>
       </c>
       <c r="G24" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H24" s="15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I24" s="1" t="n"/>
@@ -2782,27 +2782,27 @@
       </c>
       <c r="B25" s="14" t="inlineStr">
         <is>
-          <t>A pharmacist calls: a new prescription reads “methotrexate 15 mg by mouth daily” for RA. What is the safety problem?</t>
+          <t>A pharmacy label reads ‘methotrexate 15 mg by mouth daily’ for a new RA patient. What is the most appropriate action?</t>
         </is>
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
-          <t>It should be IV only in RA</t>
+          <t>Dispense it — daily dosing gives faster control</t>
         </is>
       </c>
       <c r="D25" s="14" t="inlineStr">
         <is>
-          <t>It needs N-acetylcysteine with each dose</t>
+          <t>Switch to IV methotrexate to bypass first-pass</t>
         </is>
       </c>
       <c r="E25" s="14" t="inlineStr">
         <is>
-          <t>It should be weekly; daily dosing can be fatal</t>
+          <t>Add an NSAID to protect the liver from toxicity</t>
         </is>
       </c>
       <c r="F25" s="14" t="inlineStr">
         <is>
-          <t>It should be twice daily for steady levels</t>
+          <t>Hold it; correct to once weekly with folate</t>
         </is>
       </c>
       <c r="G25" s="14" t="n">
@@ -2810,7 +2810,7 @@
       </c>
       <c r="H25" s="15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I25" s="1" t="n"/>
@@ -2839,27 +2839,27 @@
       </c>
       <c r="B26" s="14" t="inlineStr">
         <is>
-          <t>Which sequence describes how tissue injury produces musculoskeletal pain?</t>
+          <t>Which non-drug approaches does the lecture include in osteoarthritis management?</t>
         </is>
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>Injury → COX-1 induction → gastric protection → pain</t>
+          <t>Nerve ablation, spinal cord stimulation</t>
         </is>
       </c>
       <c r="D26" s="14" t="inlineStr">
         <is>
-          <t>Injury → nerve transection → cortical atrophy → pain</t>
+          <t>Activity modification, physical therapy, weight management</t>
         </is>
       </c>
       <c r="E26" s="14" t="inlineStr">
         <is>
-          <t>Injury → T-cell depletion → B-cell surge → pain</t>
+          <t>Glutathione replenishment, label review</t>
         </is>
       </c>
       <c r="F26" s="14" t="inlineStr">
         <is>
-          <t>Injury → mediator release → nociceptor sensitization → pain</t>
+          <t>Fasting, high-protein diet, bed rest</t>
         </is>
       </c>
       <c r="G26" s="14" t="n">
@@ -2867,7 +2867,7 @@
       </c>
       <c r="H26" s="15" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I26" s="1" t="n"/>
@@ -2896,27 +2896,27 @@
       </c>
       <c r="B27" s="14" t="inlineStr">
         <is>
-          <t>Which drug is a TNF inhibitor?</t>
+          <t>A prescription reads infliximab. What does the stem “-ximab” tell you?</t>
         </is>
       </c>
       <c r="C27" s="14" t="inlineStr">
         <is>
-          <t>Rituximab</t>
+          <t>A kinase inhibitor</t>
         </is>
       </c>
       <c r="D27" s="14" t="inlineStr">
         <is>
-          <t>Abatacept</t>
+          <t>A humanized monoclonal antibody</t>
         </is>
       </c>
       <c r="E27" s="14" t="inlineStr">
         <is>
-          <t>Tocilizumab</t>
+          <t>A receptor fusion protein</t>
         </is>
       </c>
       <c r="F27" s="14" t="inlineStr">
         <is>
-          <t>Etanercept</t>
+          <t>A chimeric monoclonal antibody</t>
         </is>
       </c>
       <c r="G27" s="14" t="n">
@@ -2953,31 +2953,31 @@
       </c>
       <c r="B28" s="14" t="inlineStr">
         <is>
-          <t>Which mediator is the primary target of NSAID therapy within the inflammatory pain pathway?</t>
+          <t>A pharmacist calls: a new prescription reads “methotrexate 15 mg by mouth daily” for RA. What is the safety problem?</t>
         </is>
       </c>
       <c r="C28" s="14" t="inlineStr">
         <is>
-          <t>Bradykinin</t>
+          <t>It needs N-acetylcysteine with each dose</t>
         </is>
       </c>
       <c r="D28" s="14" t="inlineStr">
         <is>
-          <t>Histamine</t>
+          <t>It should be IV only in RA</t>
         </is>
       </c>
       <c r="E28" s="14" t="inlineStr">
         <is>
-          <t>Cytokines broadly (e.g., all of TNF-α, IL-1, IL-6)</t>
+          <t>Nothing — daily dosing is standard for RA</t>
         </is>
       </c>
       <c r="F28" s="14" t="inlineStr">
         <is>
-          <t>Prostaglandins</t>
+          <t>It should be weekly; daily dosing can be fatal</t>
         </is>
       </c>
       <c r="G28" s="14" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="H28" s="15" t="inlineStr">
         <is>
@@ -3010,27 +3010,27 @@
       </c>
       <c r="B29" s="16" t="inlineStr">
         <is>
-          <t>In acetaminophen overdose, hepatotoxicity results primarily from which mechanism?</t>
+          <t>Which sequence describes how tissue injury produces musculoskeletal pain?</t>
         </is>
       </c>
       <c r="C29" s="16" t="inlineStr">
         <is>
-          <t>Excess Phase II glucuronidation</t>
+          <t>Injury → nerve transection → cortical atrophy → pain</t>
         </is>
       </c>
       <c r="D29" s="16" t="inlineStr">
         <is>
-          <t>Accumulation of NAPQI after glutathione stores are depleted</t>
+          <t>Injury → mediator release → nociceptor sensitization → pain</t>
         </is>
       </c>
       <c r="E29" s="16" t="inlineStr">
         <is>
-          <t>Direct COX inhibition in the liver</t>
+          <t>Injury → COX-1 induction → gastric protection → pain</t>
         </is>
       </c>
       <c r="F29" s="16" t="inlineStr">
         <is>
-          <t>Renal crystal formation</t>
+          <t>Injury → glutathione loss → NAPQI build-up → pain</t>
         </is>
       </c>
       <c r="G29" s="14" t="n">
@@ -3067,31 +3067,31 @@
       </c>
       <c r="B30" s="16" t="inlineStr">
         <is>
-          <t>In acetaminophen overdose, why is N-acetylcysteine effective?</t>
+          <t>Which drug is a TNF inhibitor?</t>
         </is>
       </c>
       <c r="C30" s="16" t="inlineStr">
         <is>
-          <t>It blocks COX in the liver and lowers prostaglandin levels</t>
+          <t>Abatacept</t>
         </is>
       </c>
       <c r="D30" s="16" t="inlineStr">
         <is>
-          <t>It is a glutathione precursor that restores NAPQI detoxification</t>
+          <t>Etanercept</t>
         </is>
       </c>
       <c r="E30" s="16" t="inlineStr">
         <is>
-          <t>It inhibits the enzyme that forms NAPQI from the drug</t>
+          <t>Rituximab</t>
         </is>
       </c>
       <c r="F30" s="16" t="inlineStr">
         <is>
-          <t>It binds acetaminophen in the gut and prevents absorption</t>
+          <t>Tocilizumab</t>
         </is>
       </c>
       <c r="G30" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H30" s="17" t="inlineStr">
         <is>
@@ -3124,27 +3124,27 @@
       </c>
       <c r="B31" s="16" t="inlineStr">
         <is>
-          <t>Which statement best explains why nonselective NSAIDs cause GI and renal adverse effects?</t>
+          <t>Which mediator is the primary target of NSAID therapy within the inflammatory pain pathway?</t>
         </is>
       </c>
       <c r="C31" s="16" t="inlineStr">
         <is>
-          <t>They deplete glutathione, which injures the gut and kidney</t>
+          <t>Bradykinin</t>
         </is>
       </c>
       <c r="D31" s="16" t="inlineStr">
         <is>
-          <t>They block TNF-α, which normally protects the stomach lining</t>
+          <t>Histamine</t>
         </is>
       </c>
       <c r="E31" s="16" t="inlineStr">
         <is>
-          <t>They inhibit COX-1, which protects gastric mucosa and renal blood flow</t>
+          <t>Cytokines broadly (e.g., all of TNF-α, IL-1, IL-6)</t>
         </is>
       </c>
       <c r="F31" s="16" t="inlineStr">
         <is>
-          <t>They block phospholipase A₂ and stop all mediator release</t>
+          <t>Prostaglandins</t>
         </is>
       </c>
       <c r="G31" s="14" t="n">
@@ -3152,7 +3152,7 @@
       </c>
       <c r="H31" s="17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I31" s="1" t="n"/>
@@ -3181,27 +3181,27 @@
       </c>
       <c r="B32" s="16" t="inlineStr">
         <is>
-          <t>Which nonselective NSAID does the lecture restrict to short-term use because of significant GI and renal risk?</t>
+          <t>In acetaminophen overdose, hepatotoxicity results primarily from which mechanism?</t>
         </is>
       </c>
       <c r="C32" s="16" t="inlineStr">
         <is>
-          <t>Celecoxib</t>
+          <t>Excess Phase II glucuronidation</t>
         </is>
       </c>
       <c r="D32" s="16" t="inlineStr">
         <is>
-          <t>Ketorolac</t>
+          <t>Accumulation of NAPQI after glutathione stores are depleted</t>
         </is>
       </c>
       <c r="E32" s="16" t="inlineStr">
         <is>
-          <t>Naproxen</t>
+          <t>Direct COX inhibition in the liver</t>
         </is>
       </c>
       <c r="F32" s="16" t="inlineStr">
         <is>
-          <t>Diclofenac</t>
+          <t>Renal crystal formation</t>
         </is>
       </c>
       <c r="G32" s="14" t="n">
@@ -3238,27 +3238,27 @@
       </c>
       <c r="B33" s="16" t="inlineStr">
         <is>
-          <t>What is the key difference in treatment goals between osteoarthritis and rheumatoid arthritis?</t>
+          <t>In acetaminophen overdose, why is N-acetylcysteine effective?</t>
         </is>
       </c>
       <c r="C33" s="16" t="inlineStr">
         <is>
-          <t>OA aims at pain and function; RA aims to suppress disease activity</t>
+          <t>It blocks COX in the liver and lowers prostaglandin levels</t>
         </is>
       </c>
       <c r="D33" s="16" t="inlineStr">
         <is>
-          <t>OA aims at cartilage regrowth with DMARDs</t>
+          <t>It is a glutathione precursor that restores NAPQI detoxification</t>
         </is>
       </c>
       <c r="E33" s="16" t="inlineStr">
         <is>
-          <t>OA aims to suppress immunity; RA aims at pain relief only</t>
+          <t>It inhibits the enzyme that forms NAPQI from the drug</t>
         </is>
       </c>
       <c r="F33" s="16" t="inlineStr">
         <is>
-          <t>RA aims at weight loss; OA aims at infection control</t>
+          <t>It binds acetaminophen in the gut and prevents absorption</t>
         </is>
       </c>
       <c r="G33" s="14" t="n">
@@ -3266,7 +3266,7 @@
       </c>
       <c r="H33" s="17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I33" s="1" t="n"/>
@@ -3295,27 +3295,27 @@
       </c>
       <c r="B34" s="16" t="inlineStr">
         <is>
-          <t>What is methotrexate’s mechanism as taught in the lecture, and what is co-prescribed to reduce its toxicity?</t>
+          <t>Which statement best explains why nonselective NSAIDs cause GI and renal adverse effects?</t>
         </is>
       </c>
       <c r="C34" s="16" t="inlineStr">
         <is>
-          <t>COX-2 inhibition; a proton pump inhibitor</t>
+          <t>They deplete glutathione, which injures the gut and kidney</t>
         </is>
       </c>
       <c r="D34" s="16" t="inlineStr">
         <is>
-          <t>Phospholipase A₂ blockade; calcium supplementation</t>
+          <t>They block TNF-α, which normally protects the stomach lining</t>
         </is>
       </c>
       <c r="E34" s="16" t="inlineStr">
         <is>
-          <t>TNF-α blockade; tuberculosis screening</t>
+          <t>They inhibit COX-1, which protects gastric mucosa and renal blood flow</t>
         </is>
       </c>
       <c r="F34" s="16" t="inlineStr">
         <is>
-          <t>Dihydrofolate reductase inhibition; folate supplementation</t>
+          <t>They block phospholipase A₂ and stop all mediator release</t>
         </is>
       </c>
       <c r="G34" s="14" t="n">
@@ -3323,7 +3323,7 @@
       </c>
       <c r="H34" s="17" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I34" s="1" t="n"/>
@@ -3352,35 +3352,35 @@
       </c>
       <c r="B35" s="16" t="inlineStr">
         <is>
-          <t>A 29-year-old with active RA who is planning a pregnancy needs a DMARD. Which drug from the lecture is contraindicated?</t>
+          <t>Which nonselective NSAID does the lecture restrict to short-term use because of significant GI and renal risk?</t>
         </is>
       </c>
       <c r="C35" s="16" t="inlineStr">
         <is>
-          <t>Celecoxib, because it is a disease-modifying drug</t>
+          <t>Celecoxib</t>
         </is>
       </c>
       <c r="D35" s="16" t="inlineStr">
         <is>
-          <t>Acetaminophen, because it is a DMARD</t>
+          <t>Ketorolac</t>
         </is>
       </c>
       <c r="E35" s="16" t="inlineStr">
         <is>
-          <t>Hydroxychloroquine, because of its poor safety profile</t>
+          <t>Naproxen</t>
         </is>
       </c>
       <c r="F35" s="16" t="inlineStr">
         <is>
-          <t>Methotrexate, because it is teratogenic</t>
+          <t>Diclofenac</t>
         </is>
       </c>
       <c r="G35" s="14" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="H35" s="17" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I35" s="1" t="n"/>
@@ -3409,27 +3409,27 @@
       </c>
       <c r="B36" s="16" t="inlineStr">
         <is>
-          <t>Before starting adalimumab for rheumatoid arthritis, which baseline step does the lecture specifically call for?</t>
+          <t>What is the key difference in treatment goals between osteoarthritis and rheumatoid arthritis?</t>
         </is>
       </c>
       <c r="C36" s="16" t="inlineStr">
         <is>
-          <t>Checking for all hidden acetaminophen sources</t>
+          <t>OA aims at pain and function; RA aims to suppress disease activity</t>
         </is>
       </c>
       <c r="D36" s="16" t="inlineStr">
         <is>
-          <t>Starting folate to prevent bone marrow toxicity</t>
+          <t>OA aims at cartilage regrowth with DMARDs</t>
         </is>
       </c>
       <c r="E36" s="16" t="inlineStr">
         <is>
-          <t>Screening for tuberculosis and hepatitis B/C</t>
+          <t>OA aims to suppress immunity; RA aims at pain relief only</t>
         </is>
       </c>
       <c r="F36" s="16" t="inlineStr">
         <is>
-          <t>Adding an ACE inhibitor to protect the kidney</t>
+          <t>RA aims at weight loss; OA aims at infection control</t>
         </is>
       </c>
       <c r="G36" s="14" t="n">
@@ -3437,7 +3437,7 @@
       </c>
       <c r="H36" s="17" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I36" s="1" t="n"/>
@@ -3466,35 +3466,35 @@
       </c>
       <c r="B37" s="16" t="inlineStr">
         <is>
-          <t>Match the drug to its target: which pairing is correct?</t>
+          <t>What is methotrexate’s mechanism as taught in the lecture, and what is co-prescribed to reduce its toxicity?</t>
         </is>
       </c>
       <c r="C37" s="16" t="inlineStr">
         <is>
-          <t>Abatacept — B-lymphocyte depletion</t>
+          <t>COX-2 inhibition; a proton pump inhibitor</t>
         </is>
       </c>
       <c r="D37" s="16" t="inlineStr">
         <is>
-          <t>Tocilizumab — IL-6 receptor signaling</t>
+          <t>Phospholipase A₂ blockade; calcium supplementation</t>
         </is>
       </c>
       <c r="E37" s="16" t="inlineStr">
         <is>
-          <t>Etanercept — IL-6 receptor signaling</t>
+          <t>TNF-α blockade; tuberculosis screening</t>
         </is>
       </c>
       <c r="F37" s="16" t="inlineStr">
         <is>
-          <t>Rituximab — TNF-α signaling</t>
+          <t>Dihydrofolate reductase inhibition; folate supplementation</t>
         </is>
       </c>
       <c r="G37" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H37" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I37" s="1" t="n"/>
@@ -3523,27 +3523,27 @@
       </c>
       <c r="B38" s="16" t="inlineStr">
         <is>
-          <t>Which conventional DMARD requires a baseline eye exam and annual screening after 5 years because of retinopathy?</t>
+          <t>A 29-year-old with active RA who is planning a pregnancy needs a DMARD. Which drug from the lecture is contraindicated?</t>
         </is>
       </c>
       <c r="C38" s="16" t="inlineStr">
         <is>
-          <t>Methotrexate</t>
+          <t>Celecoxib, because it is a disease-modifying drug</t>
         </is>
       </c>
       <c r="D38" s="16" t="inlineStr">
         <is>
-          <t>Mycophenolate mofetil</t>
+          <t>Acetaminophen, because it is a DMARD</t>
         </is>
       </c>
       <c r="E38" s="16" t="inlineStr">
         <is>
-          <t>Leflunomide</t>
+          <t>Hydroxychloroquine, because of its poor safety profile</t>
         </is>
       </c>
       <c r="F38" s="16" t="inlineStr">
         <is>
-          <t>Hydroxychloroquine</t>
+          <t>Methotrexate, because it is teratogenic</t>
         </is>
       </c>
       <c r="G38" s="14" t="n">
@@ -3580,27 +3580,27 @@
       </c>
       <c r="B39" s="16" t="inlineStr">
         <is>
-          <t>Pain by mechanism: which is right?</t>
+          <t>Before starting adalimumab for rheumatoid arthritis, which baseline step does the lecture specifically call for?</t>
         </is>
       </c>
       <c r="C39" s="16" t="inlineStr">
         <is>
-          <t>CBC, liver, kidney labs every 1–3 months</t>
+          <t>Checking for all hidden acetaminophen sources</t>
         </is>
       </c>
       <c r="D39" s="16" t="inlineStr">
         <is>
-          <t>N-acetylcysteine — glutathione precursor</t>
+          <t>Starting folate to prevent bone marrow toxicity</t>
         </is>
       </c>
       <c r="E39" s="16" t="inlineStr">
         <is>
-          <t>Common first-line for mild-moderate pain</t>
+          <t>Screening for tuberculosis and hepatitis B/C</t>
         </is>
       </c>
       <c r="F39" s="16" t="inlineStr">
         <is>
-          <t>Nociceptive · inflammatory · neuropathic</t>
+          <t>Adding an ACE inhibitor to protect the kidney</t>
         </is>
       </c>
       <c r="G39" s="14" t="n">
@@ -3608,7 +3608,7 @@
       </c>
       <c r="H39" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I39" s="1" t="n"/>
@@ -3637,31 +3637,31 @@
       </c>
       <c r="B40" s="16" t="inlineStr">
         <is>
-          <t>Chronic pain: which is right?</t>
+          <t>Match the drug to its target: which pairing is correct?</t>
         </is>
       </c>
       <c r="C40" s="16" t="inlineStr">
         <is>
-          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
+          <t>Abatacept — B-lymphocyte depletion</t>
         </is>
       </c>
       <c r="D40" s="16" t="inlineStr">
         <is>
-          <t>Persists beyond expected healing, often &gt; 3 months</t>
+          <t>Tocilizumab — IL-6 receptor signaling</t>
         </is>
       </c>
       <c r="E40" s="16" t="inlineStr">
         <is>
-          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
+          <t>Etanercept — IL-6 receptor signaling</t>
         </is>
       </c>
       <c r="F40" s="16" t="inlineStr">
         <is>
-          <t>Housekeeping: gastric protection, renal blood flow</t>
+          <t>Rituximab — TNF-α signaling</t>
         </is>
       </c>
       <c r="G40" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H40" s="18" t="inlineStr">
         <is>
@@ -3694,35 +3694,35 @@
       </c>
       <c r="B41" s="16" t="inlineStr">
         <is>
-          <t>4 pain mediators: which is right?</t>
+          <t>Which conventional DMARD requires a baseline eye exam and annual screening after 5 years because of retinopathy?</t>
         </is>
       </c>
       <c r="C41" s="16" t="inlineStr">
         <is>
-          <t>Prostaglandins, bradykinin, histamine, cytokines (TNF-α, IL-1, IL-6)</t>
+          <t>Methotrexate</t>
         </is>
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
+          <t>Mycophenolate mofetil</t>
         </is>
       </c>
       <c r="E41" s="16" t="inlineStr">
         <is>
-          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
+          <t>Leflunomide</t>
         </is>
       </c>
       <c r="F41" s="16" t="inlineStr">
         <is>
-          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
+          <t>Hydroxychloroquine</t>
         </is>
       </c>
       <c r="G41" s="14" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="H41" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I41" s="1" t="n"/>
@@ -3751,27 +3751,27 @@
       </c>
       <c r="B42" s="16" t="inlineStr">
         <is>
-          <t>Corticosteroid site: which is right?</t>
+          <t>Pain by mechanism: which is right?</t>
         </is>
       </c>
       <c r="C42" s="16" t="inlineStr">
         <is>
-          <t>TB + hepatitis B/C screen; update vaccines (live) first</t>
+          <t>CBC, liver, kidney labs every 1–3 months</t>
         </is>
       </c>
       <c r="D42" s="16" t="inlineStr">
         <is>
-          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
+          <t>N-acetylcysteine — glutathione precursor</t>
         </is>
       </c>
       <c r="E42" s="16" t="inlineStr">
         <is>
-          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
+          <t>Common first-line for mild-moderate pain</t>
         </is>
       </c>
       <c r="F42" s="16" t="inlineStr">
         <is>
-          <t>Anti-CD20; after TNF-inhibitor failure; check hepatitis B</t>
+          <t>Nociceptive · inflammatory · neuropathic</t>
         </is>
       </c>
       <c r="G42" s="14" t="n">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="H42" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I42" s="1" t="n"/>
@@ -3808,31 +3808,31 @@
       </c>
       <c r="B43" s="16" t="inlineStr">
         <is>
-          <t>NSAID site: which is right?</t>
+          <t>Chronic pain: which is right?</t>
         </is>
       </c>
       <c r="C43" s="16" t="inlineStr">
         <is>
-          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
+          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
         </is>
       </c>
       <c r="D43" s="16" t="inlineStr">
         <is>
-          <t>COX → prostaglandins specifically</t>
+          <t>Persists beyond expected healing, often &gt; 3 months</t>
         </is>
       </c>
       <c r="E43" s="16" t="inlineStr">
         <is>
-          <t>More potent; more GI/CNS effects</t>
+          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
         </is>
       </c>
       <c r="F43" s="16" t="inlineStr">
         <is>
-          <t>Alters lysosomal and TLR signaling</t>
+          <t>Housekeeping: gastric protection, renal blood flow</t>
         </is>
       </c>
       <c r="G43" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H43" s="18" t="inlineStr">
         <is>
@@ -3865,27 +3865,27 @@
       </c>
       <c r="B44" s="16" t="inlineStr">
         <is>
-          <t>Acetaminophen effects: which is right?</t>
+          <t>4 pain mediators: which is right?</t>
         </is>
       </c>
       <c r="C44" s="16" t="inlineStr">
         <is>
-          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
+          <t>Prostaglandins, bradykinin, histamine, cytokines (TNF-α, IL-1, IL-6)</t>
         </is>
       </c>
       <c r="D44" s="16" t="inlineStr">
         <is>
-          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
+          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
         </is>
       </c>
       <c r="E44" s="16" t="inlineStr">
         <is>
-          <t>Persists beyond expected healing, often &gt; 3 months</t>
+          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
         </is>
       </c>
       <c r="F44" s="16" t="inlineStr">
         <is>
-          <t>Housekeeping: gastric protection, renal blood flow</t>
+          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
         </is>
       </c>
       <c r="G44" s="14" t="n">
@@ -3893,7 +3893,7 @@
       </c>
       <c r="H44" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I44" s="1" t="n"/>
@@ -3922,35 +3922,35 @@
       </c>
       <c r="B45" s="16" t="inlineStr">
         <is>
-          <t>Acetaminophen toxic metabolite: which is right?</t>
+          <t>Corticosteroid site: which is right?</t>
         </is>
       </c>
       <c r="C45" s="16" t="inlineStr">
         <is>
-          <t>Alters RA’s course, not just symptoms</t>
+          <t>TB + hepatitis B/C screen; update vaccines (live) first</t>
         </is>
       </c>
       <c r="D45" s="16" t="inlineStr">
         <is>
-          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
+          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
         </is>
       </c>
       <c r="E45" s="16" t="inlineStr">
         <is>
-          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
+          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
         </is>
       </c>
       <c r="F45" s="16" t="inlineStr">
         <is>
-          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
+          <t>Anti-CD20; after TNF-inhibitor failure; check hepatitis B</t>
         </is>
       </c>
       <c r="G45" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H45" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I45" s="1" t="n"/>
@@ -3979,35 +3979,35 @@
       </c>
       <c r="B46" s="16" t="inlineStr">
         <is>
-          <t>Acetaminophen antidote: which is right?</t>
+          <t>NSAID site: which is right?</t>
         </is>
       </c>
       <c r="C46" s="16" t="inlineStr">
         <is>
-          <t>Common first-line for mild-moderate pain</t>
+          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
         </is>
       </c>
       <c r="D46" s="16" t="inlineStr">
         <is>
-          <t>CBC, liver, kidney labs every 1–3 months</t>
+          <t>COX → prostaglandins specifically</t>
         </is>
       </c>
       <c r="E46" s="16" t="inlineStr">
         <is>
-          <t>Nociceptive · inflammatory · neuropathic</t>
+          <t>More potent; more GI/CNS effects</t>
         </is>
       </c>
       <c r="F46" s="16" t="inlineStr">
         <is>
-          <t>N-acetylcysteine — glutathione precursor</t>
+          <t>Alters lysosomal and TLR signaling</t>
         </is>
       </c>
       <c r="G46" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H46" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I46" s="1" t="n"/>
@@ -4036,27 +4036,27 @@
       </c>
       <c r="B47" s="16" t="inlineStr">
         <is>
-          <t>Hidden acetaminophen: which is right?</t>
+          <t>Acetaminophen effects: which is right?</t>
         </is>
       </c>
       <c r="C47" s="16" t="inlineStr">
         <is>
-          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
+          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
         </is>
       </c>
       <c r="D47" s="16" t="inlineStr">
         <is>
-          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
+          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
         </is>
       </c>
       <c r="E47" s="16" t="inlineStr">
         <is>
-          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
+          <t>Persists beyond expected healing, often &gt; 3 months</t>
         </is>
       </c>
       <c r="F47" s="16" t="inlineStr">
         <is>
-          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
+          <t>Housekeeping: gastric protection, renal blood flow</t>
         </is>
       </c>
       <c r="G47" s="14" t="n">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="H47" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I47" s="1" t="n"/>
@@ -4093,31 +4093,31 @@
       </c>
       <c r="B48" s="16" t="inlineStr">
         <is>
-          <t>COX-1: which is right?</t>
+          <t>Acetaminophen toxic metabolite: which is right?</t>
         </is>
       </c>
       <c r="C48" s="16" t="inlineStr">
         <is>
-          <t>Persists beyond expected healing, often &gt; 3 months</t>
+          <t>Alters RA’s course, not just symptoms</t>
         </is>
       </c>
       <c r="D48" s="16" t="inlineStr">
         <is>
-          <t>Housekeeping: gastric protection, renal blood flow</t>
+          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
         </is>
       </c>
       <c r="E48" s="16" t="inlineStr">
         <is>
-          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
+          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
         </is>
       </c>
       <c r="F48" s="16" t="inlineStr">
         <is>
-          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
+          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
         </is>
       </c>
       <c r="G48" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H48" s="18" t="inlineStr">
         <is>
@@ -4150,27 +4150,27 @@
       </c>
       <c r="B49" s="16" t="inlineStr">
         <is>
-          <t>COX-2: which is right?</t>
+          <t>Acetaminophen antidote: which is right?</t>
         </is>
       </c>
       <c r="C49" s="16" t="inlineStr">
         <is>
-          <t>~90% glucuronidation/sulfation (safe) · ~5–10% CYP2E1 → NAPQI</t>
+          <t>Common first-line for mild-moderate pain</t>
         </is>
       </c>
       <c r="D49" s="16" t="inlineStr">
         <is>
-          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
+          <t>CBC, liver, kidney labs every 1–3 months</t>
         </is>
       </c>
       <c r="E49" s="16" t="inlineStr">
         <is>
-          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
+          <t>Nociceptive · inflammatory · neuropathic</t>
         </is>
       </c>
       <c r="F49" s="16" t="inlineStr">
         <is>
-          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
+          <t>N-acetylcysteine — glutathione precursor</t>
         </is>
       </c>
       <c r="G49" s="14" t="n">
@@ -4178,7 +4178,7 @@
       </c>
       <c r="H49" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I49" s="1" t="n"/>
@@ -4207,27 +4207,27 @@
       </c>
       <c r="B50" s="16" t="inlineStr">
         <is>
-          <t>Ibuprofen: which is right?</t>
+          <t>Hidden acetaminophen: which is right?</t>
         </is>
       </c>
       <c r="C50" s="16" t="inlineStr">
         <is>
-          <t>Nociceptive · inflammatory · neuropathic</t>
+          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
         </is>
       </c>
       <c r="D50" s="16" t="inlineStr">
         <is>
-          <t>N-acetylcysteine — glutathione precursor</t>
+          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
         </is>
       </c>
       <c r="E50" s="16" t="inlineStr">
         <is>
-          <t>Common first-line for mild-moderate pain</t>
+          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
         </is>
       </c>
       <c r="F50" s="16" t="inlineStr">
         <is>
-          <t>CBC, liver, kidney labs every 1–3 months</t>
+          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
         </is>
       </c>
       <c r="G50" s="14" t="n">
@@ -4264,35 +4264,35 @@
       </c>
       <c r="B51" s="16" t="inlineStr">
         <is>
-          <t>Naproxen: which is right?</t>
+          <t>COX-1: which is right?</t>
         </is>
       </c>
       <c r="C51" s="16" t="inlineStr">
         <is>
-          <t>≤ 7.5 mg daily long term, taper</t>
+          <t>Persists beyond expected healing, often &gt; 3 months</t>
         </is>
       </c>
       <c r="D51" s="16" t="inlineStr">
         <is>
-          <t>Immunosuppression → infection</t>
+          <t>Housekeeping: gastric protection, renal blood flow</t>
         </is>
       </c>
       <c r="E51" s="16" t="inlineStr">
         <is>
-          <t>DHODH (pyrimidine synthesis)</t>
+          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
         </is>
       </c>
       <c r="F51" s="16" t="inlineStr">
         <is>
-          <t>Longer half-life, twice-daily</t>
+          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
         </is>
       </c>
       <c r="G51" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H51" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I51" s="1" t="n"/>
@@ -4321,35 +4321,35 @@
       </c>
       <c r="B52" s="16" t="inlineStr">
         <is>
-          <t>Diclofenac: which is right?</t>
+          <t>COX-2: which is right?</t>
         </is>
       </c>
       <c r="C52" s="16" t="inlineStr">
         <is>
-          <t>Centrilobular necrosis</t>
+          <t>~90% glucuronidation/sulfation (safe) · ~5–10% CYP2E1 → NAPQI</t>
         </is>
       </c>
       <c r="D52" s="16" t="inlineStr">
         <is>
-          <t>Tocilizumab</t>
+          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
         </is>
       </c>
       <c r="E52" s="16" t="inlineStr">
         <is>
-          <t>↑ GI ulcer risk</t>
+          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
         </is>
       </c>
       <c r="F52" s="16" t="inlineStr">
         <is>
-          <t>Oral and topical</t>
+          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
         </is>
       </c>
       <c r="G52" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H52" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I52" s="1" t="n"/>
@@ -4378,35 +4378,35 @@
       </c>
       <c r="B53" s="16" t="inlineStr">
         <is>
-          <t>Indomethacin: which is right?</t>
+          <t>Ibuprofen: which is right?</t>
         </is>
       </c>
       <c r="C53" s="16" t="inlineStr">
         <is>
-          <t>More potent; more GI/CNS effects</t>
+          <t>Nociceptive · inflammatory · neuropathic</t>
         </is>
       </c>
       <c r="D53" s="16" t="inlineStr">
         <is>
-          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
+          <t>N-acetylcysteine — glutathione precursor</t>
         </is>
       </c>
       <c r="E53" s="16" t="inlineStr">
         <is>
-          <t>10–20× more selective for COX-2</t>
+          <t>Common first-line for mild-moderate pain</t>
         </is>
       </c>
       <c r="F53" s="16" t="inlineStr">
         <is>
-          <t>COX → prostaglandins specifically</t>
+          <t>CBC, liver, kidney labs every 1–3 months</t>
         </is>
       </c>
       <c r="G53" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H53" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I53" s="1" t="n"/>
@@ -4435,31 +4435,31 @@
       </c>
       <c r="B54" s="16" t="inlineStr">
         <is>
-          <t>Ketorolac: which is right?</t>
+          <t>Naproxen: which is right?</t>
         </is>
       </c>
       <c r="C54" s="16" t="inlineStr">
         <is>
-          <t>Nociceptive · inflammatory · neuropathic</t>
+          <t>≤ 7.5 mg daily long term, taper</t>
         </is>
       </c>
       <c r="D54" s="16" t="inlineStr">
         <is>
-          <t>CBC, liver, kidney labs every 1–3 months</t>
+          <t>Immunosuppression → infection</t>
         </is>
       </c>
       <c r="E54" s="16" t="inlineStr">
         <is>
-          <t>8 h, 120 mcg/mL → above the line → start NAC</t>
+          <t>DHODH (pyrimidine synthesis)</t>
         </is>
       </c>
       <c r="F54" s="16" t="inlineStr">
         <is>
-          <t>Short-term only; significant GI/renal risk</t>
+          <t>Longer half-life, twice-daily</t>
         </is>
       </c>
       <c r="G54" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H54" s="18" t="inlineStr">
         <is>
@@ -4492,27 +4492,27 @@
       </c>
       <c r="B55" s="16" t="inlineStr">
         <is>
-          <t>Celecoxib trade-off: which is right?</t>
+          <t>Diclofenac: which is right?</t>
         </is>
       </c>
       <c r="C55" s="16" t="inlineStr">
         <is>
-          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
+          <t>Centrilobular necrosis</t>
         </is>
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
+          <t>Tocilizumab</t>
         </is>
       </c>
       <c r="E55" s="16" t="inlineStr">
         <is>
-          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
+          <t>↑ GI ulcer risk</t>
         </is>
       </c>
       <c r="F55" s="16" t="inlineStr">
         <is>
-          <t>Alters RA’s course, not just symptoms</t>
+          <t>Oral and topical</t>
         </is>
       </c>
       <c r="G55" s="14" t="n">
@@ -4520,7 +4520,7 @@
       </c>
       <c r="H55" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I55" s="1" t="n"/>
@@ -4549,35 +4549,35 @@
       </c>
       <c r="B56" s="16" t="inlineStr">
         <is>
-          <t>NSAID adverse effects: which is right?</t>
+          <t>Indomethacin: which is right?</t>
         </is>
       </c>
       <c r="C56" s="16" t="inlineStr">
         <is>
-          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
+          <t>More potent; more GI/CNS effects</t>
         </is>
       </c>
       <c r="D56" s="16" t="inlineStr">
         <is>
-          <t>Anti-CD20; after TNF-inhibitor failure; check hepatitis B</t>
+          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
         </is>
       </c>
       <c r="E56" s="16" t="inlineStr">
         <is>
-          <t>NSAID relief in days · DMARD protection over weeks–months</t>
+          <t>10–20× more selective for COX-2</t>
         </is>
       </c>
       <c r="F56" s="16" t="inlineStr">
         <is>
-          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
+          <t>COX → prostaglandins specifically</t>
         </is>
       </c>
       <c r="G56" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H56" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I56" s="1" t="n"/>
@@ -4606,27 +4606,27 @@
       </c>
       <c r="B57" s="16" t="inlineStr">
         <is>
-          <t>NSAID cautions: which is right?</t>
+          <t>Ketorolac: which is right?</t>
         </is>
       </c>
       <c r="C57" s="16" t="inlineStr">
         <is>
-          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
+          <t>Nociceptive · inflammatory · neuropathic</t>
         </is>
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
+          <t>CBC, liver, kidney labs every 1–3 months</t>
         </is>
       </c>
       <c r="E57" s="16" t="inlineStr">
         <is>
-          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
+          <t>8 h, 120 mcg/mL → above the line → start NAC</t>
         </is>
       </c>
       <c r="F57" s="16" t="inlineStr">
         <is>
-          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
+          <t>Short-term only; significant GI/renal risk</t>
         </is>
       </c>
       <c r="G57" s="14" t="n">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="H57" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I57" s="1" t="n"/>
@@ -4663,27 +4663,27 @@
       </c>
       <c r="B58" s="16" t="inlineStr">
         <is>
-          <t>Triple whammy: which is right?</t>
+          <t>Celecoxib trade-off: which is right?</t>
         </is>
       </c>
       <c r="C58" s="16" t="inlineStr">
         <is>
-          <t>Alters lysosomal and TLR signaling</t>
+          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
         </is>
       </c>
       <c r="D58" s="16" t="inlineStr">
         <is>
-          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
+          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
         </is>
       </c>
       <c r="E58" s="16" t="inlineStr">
         <is>
-          <t>COX → prostaglandins specifically</t>
+          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
         </is>
       </c>
       <c r="F58" s="16" t="inlineStr">
         <is>
-          <t>More potent; more GI/CNS effects</t>
+          <t>Alters RA’s course, not just symptoms</t>
         </is>
       </c>
       <c r="G58" s="14" t="n">
@@ -4720,35 +4720,35 @@
       </c>
       <c r="B59" s="16" t="inlineStr">
         <is>
-          <t>NSAID + corticosteroid: which is right?</t>
+          <t>NSAID adverse effects: which is right?</t>
         </is>
       </c>
       <c r="C59" s="16" t="inlineStr">
         <is>
-          <t>Tocilizumab</t>
+          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
         <is>
-          <t>↑ GI ulcer risk</t>
+          <t>Anti-CD20; after TNF-inhibitor failure; check hepatitis B</t>
         </is>
       </c>
       <c r="E59" s="16" t="inlineStr">
         <is>
-          <t>Rituximab</t>
+          <t>NSAID relief in days · DMARD protection over weeks–months</t>
         </is>
       </c>
       <c r="F59" s="16" t="inlineStr">
         <is>
-          <t>Oral and topical</t>
+          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
         </is>
       </c>
       <c r="G59" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H59" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I59" s="1" t="n"/>
@@ -4777,27 +4777,27 @@
       </c>
       <c r="B60" s="16" t="inlineStr">
         <is>
-          <t>OA vs. RA: which is right?</t>
+          <t>NSAID cautions: which is right?</t>
         </is>
       </c>
       <c r="C60" s="16" t="inlineStr">
         <is>
-          <t>Baricitinib, tofacitinib, upadacitinib — oral; zoster, ↑ LDL</t>
+          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
         </is>
       </c>
       <c r="D60" s="16" t="inlineStr">
         <is>
-          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
+          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
         </is>
       </c>
       <c r="E60" s="16" t="inlineStr">
         <is>
-          <t>~90% glucuronidation/sulfation (safe) · ~5–10% CYP2E1 → NAPQI</t>
+          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
         </is>
       </c>
       <c r="F60" s="16" t="inlineStr">
         <is>
-          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
+          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
         </is>
       </c>
       <c r="G60" s="14" t="n">
@@ -4805,7 +4805,7 @@
       </c>
       <c r="H60" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I60" s="1" t="n"/>
@@ -4834,27 +4834,27 @@
       </c>
       <c r="B61" s="16" t="inlineStr">
         <is>
-          <t>DMARD: which is right?</t>
+          <t>Triple whammy: which is right?</t>
         </is>
       </c>
       <c r="C61" s="16" t="inlineStr">
         <is>
-          <t>Alters RA’s course, not just symptoms</t>
+          <t>Alters lysosomal and TLR signaling</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
+          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
         </is>
       </c>
       <c r="E61" s="16" t="inlineStr">
         <is>
-          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
+          <t>COX → prostaglandins specifically</t>
         </is>
       </c>
       <c r="F61" s="16" t="inlineStr">
         <is>
-          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
+          <t>More potent; more GI/CNS effects</t>
         </is>
       </c>
       <c r="G61" s="14" t="n">
@@ -4862,7 +4862,7 @@
       </c>
       <c r="H61" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I61" s="1" t="n"/>
@@ -4891,35 +4891,35 @@
       </c>
       <c r="B62" s="16" t="inlineStr">
         <is>
-          <t>Methotrexate: which is right?</t>
+          <t>NSAID + corticosteroid: which is right?</t>
         </is>
       </c>
       <c r="C62" s="16" t="inlineStr">
         <is>
-          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
+          <t>Tocilizumab</t>
         </is>
       </c>
       <c r="D62" s="16" t="inlineStr">
         <is>
-          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
+          <t>↑ GI ulcer risk</t>
         </is>
       </c>
       <c r="E62" s="16" t="inlineStr">
         <is>
-          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
+          <t>Rituximab</t>
         </is>
       </c>
       <c r="F62" s="16" t="inlineStr">
         <is>
-          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
+          <t>Oral and topical</t>
         </is>
       </c>
       <c r="G62" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H62" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I62" s="1" t="n"/>
@@ -4948,31 +4948,31 @@
       </c>
       <c r="B63" s="16" t="inlineStr">
         <is>
-          <t>TNF inhibitors: which is right?</t>
+          <t>OA vs. RA: which is right?</t>
         </is>
       </c>
       <c r="C63" s="16" t="inlineStr">
         <is>
-          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
+          <t>Baricitinib, tofacitinib, upadacitinib — oral; zoster, ↑ LDL</t>
         </is>
       </c>
       <c r="D63" s="16" t="inlineStr">
         <is>
-          <t>COX → prostaglandins specifically</t>
+          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
         </is>
       </c>
       <c r="E63" s="16" t="inlineStr">
         <is>
-          <t>Alters lysosomal and TLR signaling</t>
+          <t>~90% glucuronidation/sulfation (safe) · ~5–10% CYP2E1 → NAPQI</t>
         </is>
       </c>
       <c r="F63" s="16" t="inlineStr">
         <is>
-          <t>Adalimumab, etanercept, infliximab</t>
+          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
         </is>
       </c>
       <c r="G63" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H63" s="18" t="inlineStr">
         <is>
@@ -5005,27 +5005,27 @@
       </c>
       <c r="B64" s="16" t="inlineStr">
         <is>
-          <t>IL-6 inhibitor: which is right?</t>
+          <t>DMARD: which is right?</t>
         </is>
       </c>
       <c r="C64" s="16" t="inlineStr">
         <is>
-          <t>Tocilizumab</t>
+          <t>Alters RA’s course, not just symptoms</t>
         </is>
       </c>
       <c r="D64" s="16" t="inlineStr">
         <is>
-          <t>Rituximab</t>
+          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
         </is>
       </c>
       <c r="E64" s="16" t="inlineStr">
         <is>
-          <t>Abatacept</t>
+          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
         </is>
       </c>
       <c r="F64" s="16" t="inlineStr">
         <is>
-          <t>↑ GI ulcer risk</t>
+          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
         </is>
       </c>
       <c r="G64" s="14" t="n">
@@ -5062,31 +5062,31 @@
       </c>
       <c r="B65" s="16" t="inlineStr">
         <is>
-          <t>B-cell therapy: which is right?</t>
+          <t>Methotrexate: which is right?</t>
         </is>
       </c>
       <c r="C65" s="16" t="inlineStr">
         <is>
-          <t>Abatacept</t>
+          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
         <is>
-          <t>Tocilizumab</t>
+          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
         </is>
       </c>
       <c r="E65" s="16" t="inlineStr">
         <is>
-          <t>Rituximab</t>
+          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
         </is>
       </c>
       <c r="F65" s="16" t="inlineStr">
         <is>
-          <t>↑ GI ulcer risk</t>
+          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
         </is>
       </c>
       <c r="G65" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H65" s="18" t="inlineStr">
         <is>
@@ -5119,27 +5119,27 @@
       </c>
       <c r="B66" s="16" t="inlineStr">
         <is>
-          <t>T-cell costimulation: which is right?</t>
+          <t>TNF inhibitors: which is right?</t>
         </is>
       </c>
       <c r="C66" s="16" t="inlineStr">
         <is>
-          <t>Rituximab</t>
+          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
         </is>
       </c>
       <c r="D66" s="16" t="inlineStr">
         <is>
-          <t>Abatacept</t>
+          <t>COX → prostaglandins specifically</t>
         </is>
       </c>
       <c r="E66" s="16" t="inlineStr">
         <is>
-          <t>Tocilizumab</t>
+          <t>Alters lysosomal and TLR signaling</t>
         </is>
       </c>
       <c r="F66" s="16" t="inlineStr">
         <is>
-          <t>↑ GI ulcer risk</t>
+          <t>Adalimumab, etanercept, infliximab</t>
         </is>
       </c>
       <c r="G66" s="14" t="n">
@@ -5147,7 +5147,7 @@
       </c>
       <c r="H66" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I66" s="1" t="n"/>
@@ -5176,27 +5176,27 @@
       </c>
       <c r="B67" s="16" t="inlineStr">
         <is>
-          <t>DMARD shared risk: which is right?</t>
+          <t>IL-6 inhibitor: which is right?</t>
         </is>
       </c>
       <c r="C67" s="16" t="inlineStr">
         <is>
-          <t>DHODH (pyrimidine synthesis)</t>
+          <t>Tocilizumab</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
         <is>
-          <t>Immunosuppression → infection</t>
+          <t>Rituximab</t>
         </is>
       </c>
       <c r="E67" s="16" t="inlineStr">
         <is>
-          <t>≤ 7.5 mg daily long term, taper</t>
+          <t>Abatacept</t>
         </is>
       </c>
       <c r="F67" s="16" t="inlineStr">
         <is>
-          <t>Longer half-life, twice-daily</t>
+          <t>↑ GI ulcer risk</t>
         </is>
       </c>
       <c r="G67" s="14" t="n">
@@ -5204,7 +5204,7 @@
       </c>
       <c r="H67" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I67" s="1" t="n"/>
@@ -5233,35 +5233,35 @@
       </c>
       <c r="B68" s="16" t="inlineStr">
         <is>
-          <t>Before biologics: which is right?</t>
+          <t>B-cell therapy: which is right?</t>
         </is>
       </c>
       <c r="C68" s="16" t="inlineStr">
         <is>
-          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
+          <t>Abatacept</t>
         </is>
       </c>
       <c r="D68" s="16" t="inlineStr">
         <is>
-          <t>TB + hepatitis B/C screen; update vaccines (live) first</t>
+          <t>Tocilizumab</t>
         </is>
       </c>
       <c r="E68" s="16" t="inlineStr">
         <is>
-          <t>NSAID relief in days · DMARD protection over weeks–months</t>
+          <t>Rituximab</t>
         </is>
       </c>
       <c r="F68" s="16" t="inlineStr">
         <is>
-          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
+          <t>↑ GI ulcer risk</t>
         </is>
       </c>
       <c r="G68" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H68" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I68" s="1" t="n"/>
@@ -5290,35 +5290,35 @@
       </c>
       <c r="B69" s="16" t="inlineStr">
         <is>
-          <t>Acetaminophen routes: which is right?</t>
+          <t>T-cell costimulation: which is right?</t>
         </is>
       </c>
       <c r="C69" s="16" t="inlineStr">
         <is>
-          <t>~90% glucuronidation/sulfation (safe) · ~5–10% CYP2E1 → NAPQI</t>
+          <t>Rituximab</t>
         </is>
       </c>
       <c r="D69" s="16" t="inlineStr">
         <is>
-          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
+          <t>Abatacept</t>
         </is>
       </c>
       <c r="E69" s="16" t="inlineStr">
         <is>
-          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
+          <t>Tocilizumab</t>
         </is>
       </c>
       <c r="F69" s="16" t="inlineStr">
         <is>
-          <t>Baricitinib, tofacitinib, upadacitinib — oral; zoster, ↑ LDL</t>
+          <t>↑ GI ulcer risk</t>
         </is>
       </c>
       <c r="G69" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H69" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I69" s="1" t="n"/>
@@ -5347,31 +5347,31 @@
       </c>
       <c r="B70" s="16" t="inlineStr">
         <is>
-          <t>Who's at higher acetaminophen risk: which is right?</t>
+          <t>DMARD shared risk: which is right?</t>
         </is>
       </c>
       <c r="C70" s="16" t="inlineStr">
         <is>
-          <t>Synovitis → pannus; TNF-α and IL-6 drive erosion</t>
+          <t>DHODH (pyrimidine synthesis)</t>
         </is>
       </c>
       <c r="D70" s="16" t="inlineStr">
         <is>
-          <t>Chronic alcohol use, fasting (↓ GSH, ↑ CYP2E1)</t>
+          <t>Immunosuppression → infection</t>
         </is>
       </c>
       <c r="E70" s="16" t="inlineStr">
         <is>
-          <t>Likely anti-inflammatory via adenosine release</t>
+          <t>≤ 7.5 mg daily long term, taper</t>
         </is>
       </c>
       <c r="F70" s="16" t="inlineStr">
         <is>
-          <t>8 h, 120 mcg/mL → above the line → start NAC</t>
+          <t>Longer half-life, twice-daily</t>
         </is>
       </c>
       <c r="G70" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H70" s="18" t="inlineStr">
         <is>
@@ -5404,31 +5404,31 @@
       </c>
       <c r="B71" s="16" t="inlineStr">
         <is>
-          <t>Liver lesion in overdose: which is right?</t>
+          <t>Before biologics: which is right?</t>
         </is>
       </c>
       <c r="C71" s="16" t="inlineStr">
         <is>
-          <t>PGI2 falls, TXA2 preserved</t>
+          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
         </is>
       </c>
       <c r="D71" s="16" t="inlineStr">
         <is>
-          <t>Centrilobular necrosis</t>
+          <t>TB + hepatitis B/C screen; update vaccines (live) first</t>
         </is>
       </c>
       <c r="E71" s="16" t="inlineStr">
         <is>
-          <t>VTE (DVT/PE), MACE, cancer</t>
+          <t>NSAID relief in days · DMARD protection over weeks–months</t>
         </is>
       </c>
       <c r="F71" s="16" t="inlineStr">
         <is>
-          <t>DHODH (pyrimidine synthesis)</t>
+          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
         </is>
       </c>
       <c r="G71" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H71" s="18" t="inlineStr">
         <is>
@@ -5461,27 +5461,27 @@
       </c>
       <c r="B72" s="16" t="inlineStr">
         <is>
-          <t>Rumack-Matthew nomogram: which is right?</t>
+          <t>Acetaminophen routes: which is right?</t>
         </is>
       </c>
       <c r="C72" s="16" t="inlineStr">
         <is>
-          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
+          <t>~90% glucuronidation/sulfation (safe) · ~5–10% CYP2E1 → NAPQI</t>
         </is>
       </c>
       <c r="D72" s="16" t="inlineStr">
         <is>
-          <t>Single acute ingestion; level ≥ 4 h; above the line → NAC; not used &gt; 24 h</t>
+          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
         </is>
       </c>
       <c r="E72" s="16" t="inlineStr">
         <is>
-          <t>Prostaglandins, bradykinin, histamine, cytokines (TNF-α, IL-1, IL-6)</t>
+          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
         </is>
       </c>
       <c r="F72" s="16" t="inlineStr">
         <is>
-          <t>GI: ↓ mucus/bicarbonate · kidney: ↓ afferent dilation · platelets: ↓ TXA2</t>
+          <t>Baricitinib, tofacitinib, upadacitinib — oral; zoster, ↑ LDL</t>
         </is>
       </c>
       <c r="G72" s="14" t="n">
@@ -5489,7 +5489,7 @@
       </c>
       <c r="H72" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I72" s="1" t="n"/>
@@ -5518,27 +5518,27 @@
       </c>
       <c r="B73" s="16" t="inlineStr">
         <is>
-          <t>Nomogram example: which is right?</t>
+          <t>Who's at higher acetaminophen risk: which is right?</t>
         </is>
       </c>
       <c r="C73" s="16" t="inlineStr">
         <is>
+          <t>Synovitis → pannus; TNF-α and IL-6 drive erosion</t>
+        </is>
+      </c>
+      <c r="D73" s="16" t="inlineStr">
+        <is>
           <t>Chronic alcohol use, fasting (↓ GSH, ↑ CYP2E1)</t>
         </is>
       </c>
-      <c r="D73" s="16" t="inlineStr">
+      <c r="E73" s="16" t="inlineStr">
+        <is>
+          <t>Likely anti-inflammatory via adenosine release</t>
+        </is>
+      </c>
+      <c r="F73" s="16" t="inlineStr">
         <is>
           <t>8 h, 120 mcg/mL → above the line → start NAC</t>
-        </is>
-      </c>
-      <c r="E73" s="16" t="inlineStr">
-        <is>
-          <t>Likely anti-inflammatory via adenosine release</t>
-        </is>
-      </c>
-      <c r="F73" s="16" t="inlineStr">
-        <is>
-          <t>Short-term only; significant GI/renal risk</t>
         </is>
       </c>
       <c r="G73" s="14" t="n">
@@ -5575,35 +5575,35 @@
       </c>
       <c r="B74" s="16" t="inlineStr">
         <is>
-          <t>Nomogram line (illustrative): which is right?</t>
+          <t>Liver lesion in overdose: which is right?</t>
         </is>
       </c>
       <c r="C74" s="16" t="inlineStr">
         <is>
-          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
+          <t>PGI2 falls, TXA2 preserved</t>
         </is>
       </c>
       <c r="D74" s="16" t="inlineStr">
         <is>
-          <t>Persists beyond expected healing, often &gt; 3 months</t>
+          <t>Centrilobular necrosis</t>
         </is>
       </c>
       <c r="E74" s="16" t="inlineStr">
         <is>
-          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
+          <t>VTE (DVT/PE), MACE, cancer</t>
         </is>
       </c>
       <c r="F74" s="16" t="inlineStr">
         <is>
-          <t>Housekeeping: gastric protection, renal blood flow</t>
+          <t>DHODH (pyrimidine synthesis)</t>
         </is>
       </c>
       <c r="G74" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H74" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I74" s="1" t="n"/>
@@ -5632,35 +5632,35 @@
       </c>
       <c r="B75" s="16" t="inlineStr">
         <is>
-          <t>Celecoxib CV mechanism: which is right?</t>
+          <t>Rumack-Matthew nomogram: which is right?</t>
         </is>
       </c>
       <c r="C75" s="16" t="inlineStr">
         <is>
-          <t>Longer half-life, twice-daily</t>
+          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
         </is>
       </c>
       <c r="D75" s="16" t="inlineStr">
         <is>
-          <t>VTE (DVT/PE), MACE, cancer</t>
+          <t>Single acute ingestion; level ≥ 4 h; above the line → NAC; not used &gt; 24 h</t>
         </is>
       </c>
       <c r="E75" s="16" t="inlineStr">
         <is>
-          <t>PGI2 falls, TXA2 preserved</t>
+          <t>Prostaglandins, bradykinin, histamine, cytokines (TNF-α, IL-1, IL-6)</t>
         </is>
       </c>
       <c r="F75" s="16" t="inlineStr">
         <is>
-          <t>DHODH (pyrimidine synthesis)</t>
+          <t>GI: ↓ mucus/bicarbonate · kidney: ↓ afferent dilation · platelets: ↓ TXA2</t>
         </is>
       </c>
       <c r="G75" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H75" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I75" s="1" t="n"/>
@@ -5689,27 +5689,27 @@
       </c>
       <c r="B76" s="16" t="inlineStr">
         <is>
-          <t>NSAID organ effects: which is right?</t>
+          <t>Nomogram example: which is right?</t>
         </is>
       </c>
       <c r="C76" s="16" t="inlineStr">
         <is>
-          <t>GI: ↓ mucus/bicarbonate · kidney: ↓ afferent dilation · platelets: ↓ TXA2</t>
+          <t>Chronic alcohol use, fasting (↓ GSH, ↑ CYP2E1)</t>
         </is>
       </c>
       <c r="D76" s="16" t="inlineStr">
         <is>
-          <t>Prostaglandins, bradykinin, histamine, cytokines (TNF-α, IL-1, IL-6)</t>
+          <t>8 h, 120 mcg/mL → above the line → start NAC</t>
         </is>
       </c>
       <c r="E76" s="16" t="inlineStr">
         <is>
-          <t>Single acute ingestion; level ≥ 4 h; above the line → NAC; not used &gt; 24 h</t>
+          <t>Likely anti-inflammatory via adenosine release</t>
         </is>
       </c>
       <c r="F76" s="16" t="inlineStr">
         <is>
-          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
+          <t>Short-term only; significant GI/renal risk</t>
         </is>
       </c>
       <c r="G76" s="14" t="n">
@@ -5717,7 +5717,7 @@
       </c>
       <c r="H76" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I76" s="1" t="n"/>
@@ -5746,27 +5746,27 @@
       </c>
       <c r="B77" s="16" t="inlineStr">
         <is>
-          <t>RA joint destruction: which is right?</t>
+          <t>Nomogram line (illustrative): which is right?</t>
         </is>
       </c>
       <c r="C77" s="16" t="inlineStr">
         <is>
-          <t>Synovitis → pannus; TNF-α and IL-6 drive erosion</t>
+          <t>Analgesic + antipyretic; minimal anti-inflammatory</t>
         </is>
       </c>
       <c r="D77" s="16" t="inlineStr">
         <is>
+          <t>Persists beyond expected healing, often &gt; 3 months</t>
+        </is>
+      </c>
+      <c r="E77" s="16" t="inlineStr">
+        <is>
           <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
         </is>
       </c>
-      <c r="E77" s="16" t="inlineStr">
+      <c r="F77" s="16" t="inlineStr">
         <is>
           <t>Housekeeping: gastric protection, renal blood flow</t>
-        </is>
-      </c>
-      <c r="F77" s="16" t="inlineStr">
-        <is>
-          <t>Chronic alcohol use, fasting (↓ GSH, ↑ CYP2E1)</t>
         </is>
       </c>
       <c r="G77" s="14" t="n">
@@ -5774,7 +5774,7 @@
       </c>
       <c r="H77" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I77" s="1" t="n"/>
@@ -5803,31 +5803,31 @@
       </c>
       <c r="B78" s="16" t="inlineStr">
         <is>
-          <t>NSAID vs. DMARD onset: which is right?</t>
+          <t>Celecoxib CV mechanism: which is right?</t>
         </is>
       </c>
       <c r="C78" s="16" t="inlineStr">
         <is>
-          <t>Anti-CD20; after TNF-inhibitor failure; check hepatitis B</t>
+          <t>Longer half-life, twice-daily</t>
         </is>
       </c>
       <c r="D78" s="16" t="inlineStr">
         <is>
-          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
+          <t>VTE (DVT/PE), MACE, cancer</t>
         </is>
       </c>
       <c r="E78" s="16" t="inlineStr">
         <is>
-          <t>NSAID relief in days · DMARD protection over weeks–months</t>
+          <t>PGI2 falls, TXA2 preserved</t>
         </is>
       </c>
       <c r="F78" s="16" t="inlineStr">
         <is>
-          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
+          <t>DHODH (pyrimidine synthesis)</t>
         </is>
       </c>
       <c r="G78" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H78" s="18" t="inlineStr">
         <is>
@@ -5860,35 +5860,35 @@
       </c>
       <c r="B79" s="16" t="inlineStr">
         <is>
-          <t>Leflunomide target: which is right?</t>
+          <t>NSAID organ effects: which is right?</t>
         </is>
       </c>
       <c r="C79" s="16" t="inlineStr">
         <is>
-          <t>PGI2 falls, TXA2 preserved</t>
+          <t>GI: ↓ mucus/bicarbonate · kidney: ↓ afferent dilation · platelets: ↓ TXA2</t>
         </is>
       </c>
       <c r="D79" s="16" t="inlineStr">
         <is>
-          <t>Immunosuppression → infection</t>
+          <t>Prostaglandins, bradykinin, histamine, cytokines (TNF-α, IL-1, IL-6)</t>
         </is>
       </c>
       <c r="E79" s="16" t="inlineStr">
         <is>
-          <t>DHODH (pyrimidine synthesis)</t>
+          <t>Single acute ingestion; level ≥ 4 h; above the line → NAC; not used &gt; 24 h</t>
         </is>
       </c>
       <c r="F79" s="16" t="inlineStr">
         <is>
-          <t>Longer half-life, twice-daily</t>
+          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
         </is>
       </c>
       <c r="G79" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H79" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I79" s="1" t="n"/>
@@ -5917,31 +5917,31 @@
       </c>
       <c r="B80" s="16" t="inlineStr">
         <is>
-          <t>Hydroxychloroquine action: which is right?</t>
+          <t>RA joint destruction: which is right?</t>
         </is>
       </c>
       <c r="C80" s="16" t="inlineStr">
         <is>
-          <t>Alters lysosomal and TLR signaling</t>
+          <t>Synovitis → pannus; TNF-α and IL-6 drive erosion</t>
         </is>
       </c>
       <c r="D80" s="16" t="inlineStr">
         <is>
-          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
+          <t>150 mcg/mL at 4 h, halving every 4 h, 4.7 at 24 h</t>
         </is>
       </c>
       <c r="E80" s="16" t="inlineStr">
         <is>
-          <t>COX → prostaglandins specifically</t>
+          <t>Housekeeping: gastric protection, renal blood flow</t>
         </is>
       </c>
       <c r="F80" s="16" t="inlineStr">
         <is>
-          <t>Adalimumab, etanercept, infliximab</t>
+          <t>Chronic alcohol use, fasting (↓ GSH, ↑ CYP2E1)</t>
         </is>
       </c>
       <c r="G80" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H80" s="18" t="inlineStr">
         <is>
@@ -5974,27 +5974,27 @@
       </c>
       <c r="B81" s="16" t="inlineStr">
         <is>
-          <t>Methotrexate at low dose: which is right?</t>
+          <t>NSAID vs. DMARD onset: which is right?</t>
         </is>
       </c>
       <c r="C81" s="16" t="inlineStr">
         <is>
-          <t>Synovitis → pannus; TNF-α and IL-6 drive erosion</t>
+          <t>Anti-CD20; after TNF-inhibitor failure; check hepatitis B</t>
         </is>
       </c>
       <c r="D81" s="16" t="inlineStr">
         <is>
-          <t>Chronic alcohol use, fasting (↓ GSH, ↑ CYP2E1)</t>
+          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
         </is>
       </c>
       <c r="E81" s="16" t="inlineStr">
         <is>
-          <t>Likely anti-inflammatory via adenosine release</t>
+          <t>NSAID relief in days · DMARD protection over weeks–months</t>
         </is>
       </c>
       <c r="F81" s="16" t="inlineStr">
         <is>
-          <t>8 h, 120 mcg/mL → above the line → start NAC</t>
+          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
         </is>
       </c>
       <c r="G81" s="14" t="n">
@@ -6031,31 +6031,31 @@
       </c>
       <c r="B82" s="16" t="inlineStr">
         <is>
-          <t>Abatacept: which is right?</t>
+          <t>Leflunomide target: which is right?</t>
         </is>
       </c>
       <c r="C82" s="16" t="inlineStr">
         <is>
-          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
+          <t>PGI2 falls, TXA2 preserved</t>
         </is>
       </c>
       <c r="D82" s="16" t="inlineStr">
         <is>
-          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
+          <t>Immunosuppression → infection</t>
         </is>
       </c>
       <c r="E82" s="16" t="inlineStr">
         <is>
-          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
+          <t>DHODH (pyrimidine synthesis)</t>
         </is>
       </c>
       <c r="F82" s="16" t="inlineStr">
         <is>
-          <t>Prostaglandins, bradykinin, histamine, cytokines (TNF-α, IL-1, IL-6)</t>
+          <t>Longer half-life, twice-daily</t>
         </is>
       </c>
       <c r="G82" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H82" s="18" t="inlineStr">
         <is>
@@ -6088,31 +6088,31 @@
       </c>
       <c r="B83" s="16" t="inlineStr">
         <is>
-          <t>Rituximab: which is right?</t>
+          <t>Hydroxychloroquine action: which is right?</t>
         </is>
       </c>
       <c r="C83" s="16" t="inlineStr">
         <is>
-          <t>Anti-CD20; after TNF-inhibitor failure; check hepatitis B</t>
+          <t>Alters lysosomal and TLR signaling</t>
         </is>
       </c>
       <c r="D83" s="16" t="inlineStr">
         <is>
-          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
+          <t>NSAID + ACEi/ARB + diuretic → AKI</t>
         </is>
       </c>
       <c r="E83" s="16" t="inlineStr">
         <is>
-          <t>NSAID relief in days · DMARD protection over weeks–months</t>
+          <t>COX → prostaglandins specifically</t>
         </is>
       </c>
       <c r="F83" s="16" t="inlineStr">
         <is>
-          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
+          <t>Adalimumab, etanercept, infliximab</t>
         </is>
       </c>
       <c r="G83" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H83" s="18" t="inlineStr">
         <is>
@@ -6145,27 +6145,27 @@
       </c>
       <c r="B84" s="16" t="inlineStr">
         <is>
-          <t>Infection monitoring on DMARDs: which is right?</t>
+          <t>Methotrexate at low dose: which is right?</t>
         </is>
       </c>
       <c r="C84" s="16" t="inlineStr">
         <is>
-          <t>CBC, liver, kidney labs every 1–3 months</t>
+          <t>Synovitis → pannus; TNF-α and IL-6 drive erosion</t>
         </is>
       </c>
       <c r="D84" s="16" t="inlineStr">
         <is>
-          <t>Nociceptive · inflammatory · neuropathic</t>
+          <t>Chronic alcohol use, fasting (↓ GSH, ↑ CYP2E1)</t>
         </is>
       </c>
       <c r="E84" s="16" t="inlineStr">
         <is>
-          <t>Common first-line for mild-moderate pain</t>
+          <t>Likely anti-inflammatory via adenosine release</t>
         </is>
       </c>
       <c r="F84" s="16" t="inlineStr">
         <is>
-          <t>N-acetylcysteine — glutathione precursor</t>
+          <t>8 h, 120 mcg/mL → above the line → start NAC</t>
         </is>
       </c>
       <c r="G84" s="14" t="n">
@@ -6173,7 +6173,7 @@
       </c>
       <c r="H84" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I84" s="1" t="n"/>
@@ -6202,35 +6202,35 @@
       </c>
       <c r="B85" s="16" t="inlineStr">
         <is>
-          <t>Acetaminophen max (adults): which is right?</t>
+          <t>Abatacept: which is right?</t>
         </is>
       </c>
       <c r="C85" s="16" t="inlineStr">
         <is>
-          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
+          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
         </is>
       </c>
       <c r="D85" s="16" t="inlineStr">
         <is>
-          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
+          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
         </is>
       </c>
       <c r="E85" s="16" t="inlineStr">
         <is>
-          <t>Alters RA’s course, not just symptoms</t>
+          <t>CTLA-4-Ig: binds CD80/86, blocks CD28 costimulation — acts earliest</t>
         </is>
       </c>
       <c r="F85" s="16" t="inlineStr">
         <is>
-          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
+          <t>Prostaglandins, bradykinin, histamine, cytokines (TNF-α, IL-1, IL-6)</t>
         </is>
       </c>
       <c r="G85" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H85" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I85" s="1" t="n"/>
@@ -6259,27 +6259,27 @@
       </c>
       <c r="B86" s="16" t="inlineStr">
         <is>
-          <t>Aspirin vs. other NSAIDs: which is right?</t>
+          <t>Rituximab: which is right?</t>
         </is>
       </c>
       <c r="C86" s="16" t="inlineStr">
         <is>
-          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
+          <t>Anti-CD20; after TNF-inhibitor failure; check hepatitis B</t>
         </is>
       </c>
       <c r="D86" s="16" t="inlineStr">
         <is>
-          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
+          <t>GI (ulcer, bleed) · renal (AKI, fluid) · CV (HTN, events)</t>
         </is>
       </c>
       <c r="E86" s="16" t="inlineStr">
         <is>
-          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
+          <t>NSAID relief in days · DMARD protection over weeks–months</t>
         </is>
       </c>
       <c r="F86" s="16" t="inlineStr">
         <is>
-          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
+          <t>Phospholipase A₂ (upstream) → broad mediator suppression</t>
         </is>
       </c>
       <c r="G86" s="14" t="n">
@@ -6287,7 +6287,7 @@
       </c>
       <c r="H86" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I86" s="1" t="n"/>
@@ -6316,35 +6316,35 @@
       </c>
       <c r="B87" s="16" t="inlineStr">
         <is>
-          <t>Celecoxib selectivity: which is right?</t>
+          <t>Infection monitoring on DMARDs: which is right?</t>
         </is>
       </c>
       <c r="C87" s="16" t="inlineStr">
         <is>
-          <t>Malignancy, especially lymphoma</t>
+          <t>CBC, liver, kidney labs every 1–3 months</t>
         </is>
       </c>
       <c r="D87" s="16" t="inlineStr">
         <is>
-          <t>10–20× more selective for COX-2</t>
+          <t>Nociceptive · inflammatory · neuropathic</t>
         </is>
       </c>
       <c r="E87" s="16" t="inlineStr">
         <is>
-          <t>≤ 7.5 mg daily long term, taper</t>
+          <t>Common first-line for mild-moderate pain</t>
         </is>
       </c>
       <c r="F87" s="16" t="inlineStr">
         <is>
-          <t>7.5 mg weekly → 15–25 mg weekly</t>
+          <t>N-acetylcysteine — glutathione precursor</t>
         </is>
       </c>
       <c r="G87" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H87" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I87" s="1" t="n"/>
@@ -6373,27 +6373,27 @@
       </c>
       <c r="B88" s="16" t="inlineStr">
         <is>
-          <t>Methotrexate dose: which is right?</t>
+          <t>Acetaminophen max (adults): which is right?</t>
         </is>
       </c>
       <c r="C88" s="16" t="inlineStr">
         <is>
-          <t>10–20× more selective for COX-2</t>
+          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
         </is>
       </c>
       <c r="D88" s="16" t="inlineStr">
         <is>
-          <t>Malignancy, especially lymphoma</t>
+          <t>↓ GI risk, ↑ CV risk, same renal risk</t>
         </is>
       </c>
       <c r="E88" s="16" t="inlineStr">
         <is>
-          <t>≤ 7.5 mg daily long term, taper</t>
+          <t>Alters RA’s course, not just symptoms</t>
         </is>
       </c>
       <c r="F88" s="16" t="inlineStr">
         <is>
-          <t>7.5 mg weekly → 15–25 mg weekly</t>
+          <t>NAPQI (N-acetyl-p-benzoquinone imine)</t>
         </is>
       </c>
       <c r="G88" s="14" t="n">
@@ -6401,7 +6401,7 @@
       </c>
       <c r="H88" s="18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I88" s="1" t="n"/>
@@ -6430,35 +6430,35 @@
       </c>
       <c r="B89" s="16" t="inlineStr">
         <is>
-          <t>Hydroxychloroquine monitoring: which is right?</t>
+          <t>Aspirin vs. other NSAIDs: which is right?</t>
         </is>
       </c>
       <c r="C89" s="16" t="inlineStr">
         <is>
-          <t>Baseline eye exam; annual after 5 years</t>
+          <t>GI bleed/ulcer, CKD, HF/CV disease, anticoagulant, late pregnancy</t>
         </is>
       </c>
       <c r="D89" s="16" t="inlineStr">
         <is>
-          <t>CBC, liver, kidney labs every 1–3 months</t>
+          <t>Aspirin: irreversible platelet COX (8–10 days); others reversible</t>
         </is>
       </c>
       <c r="E89" s="16" t="inlineStr">
         <is>
-          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
+          <t>Combination cold, flu, and sleep products — ask about ALL sources</t>
         </is>
       </c>
       <c r="F89" s="16" t="inlineStr">
         <is>
-          <t>Common first-line for mild-moderate pain</t>
+          <t>DHFR inhibitor · weekly · folate · liver/marrow/lung · teratogenic</t>
         </is>
       </c>
       <c r="G89" s="14" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="H89" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I89" s="1" t="n"/>
@@ -6487,27 +6487,27 @@
       </c>
       <c r="B90" s="16" t="inlineStr">
         <is>
-          <t>TNF inhibitor boxed warning: which is right?</t>
+          <t>Celecoxib selectivity: which is right?</t>
         </is>
       </c>
       <c r="C90" s="16" t="inlineStr">
         <is>
+          <t>Malignancy, especially lymphoma</t>
+        </is>
+      </c>
+      <c r="D90" s="16" t="inlineStr">
+        <is>
           <t>10–20× more selective for COX-2</t>
         </is>
       </c>
-      <c r="D90" s="16" t="inlineStr">
+      <c r="E90" s="16" t="inlineStr">
+        <is>
+          <t>≤ 7.5 mg daily long term, taper</t>
+        </is>
+      </c>
+      <c r="F90" s="16" t="inlineStr">
         <is>
           <t>7.5 mg weekly → 15–25 mg weekly</t>
-        </is>
-      </c>
-      <c r="E90" s="16" t="inlineStr">
-        <is>
-          <t>Malignancy, especially lymphoma</t>
-        </is>
-      </c>
-      <c r="F90" s="16" t="inlineStr">
-        <is>
-          <t>≤ 7.5 mg daily long term, taper</t>
         </is>
       </c>
       <c r="G90" s="14" t="n">
@@ -6515,7 +6515,7 @@
       </c>
       <c r="H90" s="18" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I90" s="1" t="n"/>
@@ -6544,27 +6544,27 @@
       </c>
       <c r="B91" s="16" t="inlineStr">
         <is>
-          <t>JAK inhibitor boxed warning: which is right?</t>
+          <t>Methotrexate dose: which is right?</t>
         </is>
       </c>
       <c r="C91" s="16" t="inlineStr">
         <is>
-          <t>VTE (DVT/PE), MACE, cancer</t>
+          <t>10–20× more selective for COX-2</t>
         </is>
       </c>
       <c r="D91" s="16" t="inlineStr">
         <is>
-          <t>Longer half-life, twice-daily</t>
+          <t>Malignancy, especially lymphoma</t>
         </is>
       </c>
       <c r="E91" s="16" t="inlineStr">
         <is>
-          <t>PGI2 falls, TXA2 preserved</t>
+          <t>≤ 7.5 mg daily long term, taper</t>
         </is>
       </c>
       <c r="F91" s="16" t="inlineStr">
         <is>
-          <t>DHODH (pyrimidine synthesis)</t>
+          <t>7.5 mg weekly → 15–25 mg weekly</t>
         </is>
       </c>
       <c r="G91" s="14" t="n">
@@ -6572,7 +6572,7 @@
       </c>
       <c r="H91" s="18" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I91" s="1" t="n"/>
@@ -6601,35 +6601,35 @@
       </c>
       <c r="B92" s="16" t="inlineStr">
         <is>
-          <t>JAK inhibitors: which is right?</t>
+          <t>Hydroxychloroquine monitoring: which is right?</t>
         </is>
       </c>
       <c r="C92" s="16" t="inlineStr">
         <is>
-          <t>~90% glucuronidation/sulfation (safe) · ~5–10% CYP2E1 → NAPQI</t>
+          <t>Baseline eye exam; annual after 5 years</t>
         </is>
       </c>
       <c r="D92" s="16" t="inlineStr">
         <is>
-          <t>Baricitinib, tofacitinib, upadacitinib — oral; zoster, ↑ LDL</t>
+          <t>CBC, liver, kidney labs every 1–3 months</t>
         </is>
       </c>
       <c r="E92" s="16" t="inlineStr">
         <is>
-          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
+          <t>Generally ≤ 4 g/day; 15 g may be fatal</t>
         </is>
       </c>
       <c r="F92" s="16" t="inlineStr">
         <is>
-          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
+          <t>Common first-line for mild-moderate pain</t>
         </is>
       </c>
       <c r="G92" s="14" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="H92" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I92" s="1" t="n"/>
@@ -6658,27 +6658,27 @@
       </c>
       <c r="B93" s="16" t="inlineStr">
         <is>
-          <t>RA prednisone ceiling: which is right?</t>
+          <t>TNF inhibitor boxed warning: which is right?</t>
         </is>
       </c>
       <c r="C93" s="16" t="inlineStr">
         <is>
+          <t>10–20× more selective for COX-2</t>
+        </is>
+      </c>
+      <c r="D93" s="16" t="inlineStr">
+        <is>
           <t>7.5 mg weekly → 15–25 mg weekly</t>
         </is>
       </c>
-      <c r="D93" s="16" t="inlineStr">
+      <c r="E93" s="16" t="inlineStr">
+        <is>
+          <t>Malignancy, especially lymphoma</t>
+        </is>
+      </c>
+      <c r="F93" s="16" t="inlineStr">
         <is>
           <t>≤ 7.5 mg daily long term, taper</t>
-        </is>
-      </c>
-      <c r="E93" s="16" t="inlineStr">
-        <is>
-          <t>Malignancy, especially lymphoma</t>
-        </is>
-      </c>
-      <c r="F93" s="16" t="inlineStr">
-        <is>
-          <t>10–20× more selective for COX-2</t>
         </is>
       </c>
       <c r="G93" s="14" t="n">
@@ -6686,7 +6686,7 @@
       </c>
       <c r="H93" s="18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I93" s="1" t="n"/>
@@ -6710,14 +6710,42 @@
       <c r="AA93" s="1" t="n"/>
     </row>
     <row r="94" ht="25.5" customHeight="1">
-      <c r="A94" s="11" t="n"/>
-      <c r="B94" s="16" t="n"/>
-      <c r="C94" s="16" t="n"/>
-      <c r="D94" s="16" t="n"/>
-      <c r="E94" s="16" t="n"/>
-      <c r="F94" s="16" t="n"/>
-      <c r="G94" s="14" t="n"/>
-      <c r="H94" s="18" t="n"/>
+      <c r="A94" s="11" t="n">
+        <v>86</v>
+      </c>
+      <c r="B94" s="16" t="inlineStr">
+        <is>
+          <t>JAK inhibitor boxed warning: which is right?</t>
+        </is>
+      </c>
+      <c r="C94" s="16" t="inlineStr">
+        <is>
+          <t>VTE (DVT/PE), MACE, cancer</t>
+        </is>
+      </c>
+      <c r="D94" s="16" t="inlineStr">
+        <is>
+          <t>Longer half-life, twice-daily</t>
+        </is>
+      </c>
+      <c r="E94" s="16" t="inlineStr">
+        <is>
+          <t>PGI2 falls, TXA2 preserved</t>
+        </is>
+      </c>
+      <c r="F94" s="16" t="inlineStr">
+        <is>
+          <t>DHODH (pyrimidine synthesis)</t>
+        </is>
+      </c>
+      <c r="G94" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="H94" s="18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="I94" s="1" t="n"/>
       <c r="J94" s="1" t="n"/>
       <c r="K94" s="1" t="n"/>
@@ -6739,14 +6767,42 @@
       <c r="AA94" s="1" t="n"/>
     </row>
     <row r="95" ht="25.5" customHeight="1">
-      <c r="A95" s="11" t="n"/>
-      <c r="B95" s="16" t="n"/>
-      <c r="C95" s="16" t="n"/>
-      <c r="D95" s="16" t="n"/>
-      <c r="E95" s="16" t="n"/>
-      <c r="F95" s="16" t="n"/>
-      <c r="G95" s="14" t="n"/>
-      <c r="H95" s="18" t="n"/>
+      <c r="A95" s="11" t="n">
+        <v>87</v>
+      </c>
+      <c r="B95" s="16" t="inlineStr">
+        <is>
+          <t>JAK inhibitors: which is right?</t>
+        </is>
+      </c>
+      <c r="C95" s="16" t="inlineStr">
+        <is>
+          <t>~90% glucuronidation/sulfation (safe) · ~5–10% CYP2E1 → NAPQI</t>
+        </is>
+      </c>
+      <c r="D95" s="16" t="inlineStr">
+        <is>
+          <t>Baricitinib, tofacitinib, upadacitinib — oral; zoster, ↑ LDL</t>
+        </is>
+      </c>
+      <c r="E95" s="16" t="inlineStr">
+        <is>
+          <t>Induced at inflammation; main inflammatory prostaglandin source</t>
+        </is>
+      </c>
+      <c r="F95" s="16" t="inlineStr">
+        <is>
+          <t>Degenerative → pain/function vs. autoimmune → suppress disease</t>
+        </is>
+      </c>
+      <c r="G95" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="H95" s="18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="I95" s="1" t="n"/>
       <c r="J95" s="1" t="n"/>
       <c r="K95" s="1" t="n"/>
@@ -6768,14 +6824,42 @@
       <c r="AA95" s="1" t="n"/>
     </row>
     <row r="96" ht="25.5" customHeight="1">
-      <c r="A96" s="11" t="n"/>
-      <c r="B96" s="16" t="n"/>
-      <c r="C96" s="16" t="n"/>
-      <c r="D96" s="16" t="n"/>
-      <c r="E96" s="16" t="n"/>
-      <c r="F96" s="16" t="n"/>
-      <c r="G96" s="14" t="n"/>
-      <c r="H96" s="18" t="n"/>
+      <c r="A96" s="11" t="n">
+        <v>88</v>
+      </c>
+      <c r="B96" s="16" t="inlineStr">
+        <is>
+          <t>RA prednisone ceiling: which is right?</t>
+        </is>
+      </c>
+      <c r="C96" s="16" t="inlineStr">
+        <is>
+          <t>7.5 mg weekly → 15–25 mg weekly</t>
+        </is>
+      </c>
+      <c r="D96" s="16" t="inlineStr">
+        <is>
+          <t>≤ 7.5 mg daily long term, taper</t>
+        </is>
+      </c>
+      <c r="E96" s="16" t="inlineStr">
+        <is>
+          <t>Malignancy, especially lymphoma</t>
+        </is>
+      </c>
+      <c r="F96" s="16" t="inlineStr">
+        <is>
+          <t>10–20× more selective for COX-2</t>
+        </is>
+      </c>
+      <c r="G96" s="14" t="n">
+        <v>20</v>
+      </c>
+      <c r="H96" s="18" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="I96" s="1" t="n"/>
       <c r="J96" s="1" t="n"/>
       <c r="K96" s="1" t="n"/>

</xml_diff>